<commit_message>
Add auto-renewal statuses, usage rule and forecast of the forecast
Statuses now come from what we know today. Auto-renewals get their own
statuses (no blockers, billing blocker, at risk before/after the notice
deadline, notice received). Over-usage adds an upsell line and task; under-usage
flags the CSM. Target statuses by 30 Oct give the forecast after actions.
Notice periods for auto-renewals are labelled as assumptions.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CVAHSCDuy4tEBaMUUSRsNB
</commit_message>
<xml_diff>
--- a/n8n-renewals-challenge/renewal_tracker.xlsx
+++ b/n8n-renewals-challenge/renewal_tracker.xlsx
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="329" uniqueCount="239">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="386" uniqueCount="270">
   <si>
     <t xml:space="preserve">Renewal tracker: a mock-up of the CRM renewal model</t>
   </si>
@@ -78,6 +78,24 @@
     <t xml:space="preserve">Renewal Status x days to renewal. Late statuses rise as the date gets closer; early statuses fall. Overdue has its own, lower column.</t>
   </si>
   <si>
+    <t xml:space="preserve">Auto-renewals</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Own statuses: Renewing: no blockers / Billing blocker / At risk (before or after the notice deadline) / Notice received / Renewed. A red status cell means the status does not match the renewal type.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Usage rule</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Usage +20%: renew as is plus an Upsell line and task (no automatic charge). Usage -20%: flag the CSM; auto-renewals move to At risk.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forecast of the forecast</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Weighted today vs weighted by 30 Oct if this week's actions move each status to its target.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Overdue rule</t>
   </si>
   <si>
@@ -168,7 +186,10 @@
     <t xml:space="preserve">Q4 2026 renewal pipeline: first slice (10 renewals, €375k ARR)</t>
   </si>
   <si>
-    <t xml:space="preserve">Blue on yellow = input. Everything else is a formula.</t>
+    <t xml:space="preserve">Target date</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Blue on yellow = input. Everything else is a formula. Columns AF-AH: the forecast after this week's actions.</t>
   </si>
   <si>
     <t xml:space="preserve">Base ARR (€)</t>
@@ -222,6 +243,24 @@
     <t xml:space="preserve">Forecast bucket</t>
   </si>
   <si>
+    <t xml:space="preserve">Notice period (days)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Notice deadline</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Usage signal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Target status by 30 Oct</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Target prob.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Weighted after actions (€)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Vantage Freight</t>
   </si>
   <si>
@@ -252,16 +291,19 @@
     <t xml:space="preserve">Yes: Manager, to agree the grace period before access is restricted</t>
   </si>
   <si>
+    <t xml:space="preserve">Waiting for PO</t>
+  </si>
+  <si>
     <t xml:space="preserve">Northwind Logistics</t>
   </si>
   <si>
     <t xml:space="preserve">Green</t>
   </si>
   <si>
-    <t xml:space="preserve">Waiting for PO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Signed 3 days late last year</t>
+    <t xml:space="preserve">Engaging customer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No quote sent; signatory unknown; signed 3 days late last year</t>
   </si>
   <si>
     <t xml:space="preserve">Quote and order form out today at €50.4k for e-signature; champion confirms signatory and PO need; signature booked for 27 Oct.</t>
@@ -273,12 +315,18 @@
     <t xml:space="preserve">CSM</t>
   </si>
   <si>
+    <t xml:space="preserve">PO received</t>
+  </si>
+  <si>
     <t xml:space="preserve">Pixelforge</t>
   </si>
   <si>
     <t xml:space="preserve">Auto</t>
   </si>
   <si>
+    <t xml:space="preserve">Billing blocker</t>
+  </si>
+  <si>
     <t xml:space="preserve">Card expired; billing contact unknown</t>
   </si>
   <si>
@@ -291,13 +339,16 @@
     <t xml:space="preserve">Me, Finance</t>
   </si>
   <si>
+    <t xml:space="preserve">Renewing: no blockers</t>
+  </si>
+  <si>
     <t xml:space="preserve">Halden Health</t>
   </si>
   <si>
     <t xml:space="preserve">Red</t>
   </si>
   <si>
-    <t xml:space="preserve">Engaging customer</t>
+    <t xml:space="preserve">Not started</t>
   </si>
   <si>
     <t xml:space="preserve">Champion left; new owner unknown</t>
@@ -363,7 +414,7 @@
     <t xml:space="preserve">Uplift notice by 22 Oct. New entity details; Legal: billing change or assignment; Finance updates billing before the invoice run.</t>
   </si>
   <si>
-    <t xml:space="preserve">Auto-renewal with the wrong billing entity; uplift notice due 22 Oct.</t>
+    <t xml:space="preserve">Auto-renewal with the wrong billing entity; uplift notice due 22 Oct (assumed 30-day notice).</t>
   </si>
   <si>
     <t xml:space="preserve">Finance, Legal</t>
@@ -399,13 +450,16 @@
     <t xml:space="preserve">Quanta Labs</t>
   </si>
   <si>
+    <t xml:space="preserve">At risk: before notice deadline</t>
+  </si>
+  <si>
     <t xml:space="preserve">Budget cuts in Q1; 2 check-ins unanswered</t>
   </si>
   <si>
     <t xml:space="preserve">CSM and exec sponsor via a new contact; I confirm the ~19 Nov notice date; offer right-sizing or a 2-year price lock before they cancel.</t>
   </si>
   <si>
-    <t xml:space="preserve">Auto-renewal, usage -20%, Q1 budget cuts, unresponsive. 60 days, but cancellation notice ~19 Nov.</t>
+    <t xml:space="preserve">Auto-renewal, usage -20%, Q1 budget cuts, unresponsive. 60 days, but the notice deadline is ~19 Nov (assumed 30-day notice).</t>
   </si>
   <si>
     <t xml:space="preserve">Total</t>
@@ -453,6 +507,15 @@
     <t xml:space="preserve">Net retention (new ARR / base, incl. 5% uplift)</t>
   </si>
   <si>
+    <t xml:space="preserve">Weighted today (statuses from what we know)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Weighted by 30 Oct, if this week's actions land</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Uplift from this week's actions</t>
+  </si>
+  <si>
     <t xml:space="preserve">Opportunity products: renewal / upsell / downgrade / cross-sell / churn per line</t>
   </si>
   <si>
@@ -630,7 +693,7 @@
     <t xml:space="preserve">Renewal probability: Renewal Status x days to renewal</t>
   </si>
   <si>
-    <t xml:space="preserve">Late statuses (Quoted and after) rise as the date gets closer. Early statuses (Not started, Engaging, Negotiation) fall as the date gets closer: no progress near the date is the risk. Blue = editable.</t>
+    <t xml:space="preserve">Manual: late statuses (Quoted and after) rise as the date gets closer; early statuses fall. Auto-renewal: a clean renewal rises; an open blocker or risk falls as the date gets closer. Blue = editable.</t>
   </si>
   <si>
     <t xml:space="preserve">Overdue</t>
@@ -651,15 +714,15 @@
     <t xml:space="preserve">Exit criteria (what must be true to be in this status)</t>
   </si>
   <si>
+    <t xml:space="preserve">Applies to</t>
+  </si>
+  <si>
     <t xml:space="preserve">--None--</t>
   </si>
   <si>
     <t xml:space="preserve">Not allowed. Every open renewal must have a status.</t>
   </si>
   <si>
-    <t xml:space="preserve">Not started</t>
-  </si>
-  <si>
     <t xml:space="preserve">Renewal opportunity exists; no customer contact about the renewal yet.</t>
   </si>
   <si>
@@ -675,9 +738,6 @@
     <t xml:space="preserve">Order form approved by the buyer; in their PO or signature workflow.</t>
   </si>
   <si>
-    <t xml:space="preserve">PO received</t>
-  </si>
-  <si>
     <t xml:space="preserve">PO or signature in hand; only booking and invoicing remain.</t>
   </si>
   <si>
@@ -693,7 +753,40 @@
     <t xml:space="preserve">Customer gave notice or will not renew.</t>
   </si>
   <si>
+    <t xml:space="preserve">Both</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Valid payment method, correct billing entity, uplift notice sent, usage stable or growing. (Overdue = payment failed: move to Billing blocker.)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Expired card, wrong legal entity, PO required. Admin fix, usually recoverable.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Usage down 20%+, silence or budget cuts, and the customer can still give notice.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">At risk: notice deadline passed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Same signals, but no notice was given: the contract has renewed. Risk shifts to payment.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Notice received</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Customer gave non-renewal or downgrade notice. Becomes a manual save negotiation.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Renewed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Invoiced and paid.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Overdue renewals use the Overdue column and are shown as Late. They still count in the quarter's forecast only if the expected close date is on or before quarter end. If they slip past quarter end they count 0% for that quarter and come back next quarter as a late renewal.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">n8n prices by workflow executions (users are unlimited). Usage +20% or more: renew as is, add an Upsell line and a CSM + Renewals task; never auto-charge unless the contract has an overage clause. Usage -20% or more: flag the CSM for an adoption plan; on an auto-renewal, set At risk.</t>
   </si>
   <si>
     <t xml:space="preserve">Commercial policy (section C) and the approval it triggers</t>
@@ -1403,7 +1496,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22"/>
@@ -1493,6 +1586,30 @@
       </c>
       <c r="B12" s="3" t="s">
         <v>20</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>26</v>
       </c>
     </row>
   </sheetData>
@@ -1530,50 +1647,50 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="I4" s="6" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="J4" s="6" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="K4" s="6" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="L4" s="6" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1598,7 +1715,7 @@
       </c>
       <c r="F5" s="8" t="str">
         <f aca="false">INDEX(Pipeline!$G$5:$G$14,MATCH($A5,Pipeline!$Y$5:$Y$14,0))</f>
-        <v>Waiting for PO</v>
+        <v>Engaging customer</v>
       </c>
       <c r="G5" s="8" t="str">
         <f aca="false">INDEX(Pipeline!$Z$5:$Z$14,MATCH($A5,Pipeline!$Y$5:$Y$14,0))&amp;""</f>
@@ -1696,7 +1813,7 @@
       </c>
       <c r="F7" s="8" t="str">
         <f aca="false">INDEX(Pipeline!$G$5:$G$14,MATCH($A7,Pipeline!$Y$5:$Y$14,0))</f>
-        <v>Waiting for PO</v>
+        <v>Billing blocker</v>
       </c>
       <c r="G7" s="8" t="str">
         <f aca="false">INDEX(Pipeline!$Z$5:$Z$14,MATCH($A7,Pipeline!$Y$5:$Y$14,0))&amp;""</f>
@@ -1745,7 +1862,7 @@
       </c>
       <c r="F8" s="8" t="str">
         <f aca="false">INDEX(Pipeline!$G$5:$G$14,MATCH($A8,Pipeline!$Y$5:$Y$14,0))</f>
-        <v>Engaging customer</v>
+        <v>Not started</v>
       </c>
       <c r="G8" s="8" t="str">
         <f aca="false">INDEX(Pipeline!$Z$5:$Z$14,MATCH($A8,Pipeline!$Y$5:$Y$14,0))&amp;""</f>
@@ -1892,7 +2009,7 @@
       </c>
       <c r="F11" s="8" t="str">
         <f aca="false">INDEX(Pipeline!$G$5:$G$14,MATCH($A11,Pipeline!$Y$5:$Y$14,0))</f>
-        <v>Quoted</v>
+        <v>Engaging customer</v>
       </c>
       <c r="G11" s="8" t="str">
         <f aca="false">INDEX(Pipeline!$Z$5:$Z$14,MATCH($A11,Pipeline!$Y$5:$Y$14,0))&amp;""</f>
@@ -1941,7 +2058,7 @@
       </c>
       <c r="F12" s="8" t="str">
         <f aca="false">INDEX(Pipeline!$G$5:$G$14,MATCH($A12,Pipeline!$Y$5:$Y$14,0))</f>
-        <v>Quoted</v>
+        <v>Not started</v>
       </c>
       <c r="G12" s="8" t="str">
         <f aca="false">INDEX(Pipeline!$Z$5:$Z$14,MATCH($A12,Pipeline!$Y$5:$Y$14,0))&amp;""</f>
@@ -1990,11 +2107,11 @@
       </c>
       <c r="F13" s="8" t="str">
         <f aca="false">INDEX(Pipeline!$G$5:$G$14,MATCH($A13,Pipeline!$Y$5:$Y$14,0))</f>
-        <v>Waiting for PO</v>
+        <v>Billing blocker</v>
       </c>
       <c r="G13" s="8" t="str">
         <f aca="false">INDEX(Pipeline!$Z$5:$Z$14,MATCH($A13,Pipeline!$Y$5:$Y$14,0))&amp;""</f>
-        <v>Auto-renewal with the wrong billing entity; uplift notice due 22 Oct.</v>
+        <v>Auto-renewal with the wrong billing entity; uplift notice due 22 Oct (assumed 30-day notice).</v>
       </c>
       <c r="H13" s="8" t="str">
         <f aca="false">INDEX(Pipeline!$V$5:$V$14,MATCH($A13,Pipeline!$Y$5:$Y$14,0))&amp;""</f>
@@ -2039,11 +2156,11 @@
       </c>
       <c r="F14" s="8" t="str">
         <f aca="false">INDEX(Pipeline!$G$5:$G$14,MATCH($A14,Pipeline!$Y$5:$Y$14,0))</f>
-        <v>Engaging customer</v>
+        <v>At risk: before notice deadline</v>
       </c>
       <c r="G14" s="8" t="str">
         <f aca="false">INDEX(Pipeline!$Z$5:$Z$14,MATCH($A14,Pipeline!$Y$5:$Y$14,0))&amp;""</f>
-        <v>Auto-renewal, usage -20%, Q1 budget cuts, unresponsive. 60 days, but cancellation notice ~19 Nov.</v>
+        <v>Auto-renewal, usage -20%, Q1 budget cuts, unresponsive. 60 days, but the notice deadline is ~19 Nov (assumed 30-day notice).</v>
       </c>
       <c r="H14" s="8" t="str">
         <f aca="false">INDEX(Pipeline!$V$5:$V$14,MATCH($A14,Pipeline!$Y$5:$Y$14,0))&amp;""</f>
@@ -2068,7 +2185,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="C16" s="12" t="str">
         <f aca="false">COUNTIF(L5:L14,"Yes*")&amp;" accounts, "&amp;TEXT(SUMIF(L5:L14,"Yes*",C5:C14),"€#,##0")&amp;" ARR"</f>
@@ -2077,10 +2194,10 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="C17" s="13" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="D17" s="13"/>
       <c r="E17" s="13"/>
@@ -2126,7 +2243,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:AB29"/>
+  <dimension ref="A1:AH34"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="20"/>
@@ -2150,11 +2267,17 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="26" style="0" width="50"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="27" min="27" style="0" width="20"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="28" min="28" style="0" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="29" min="29" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="30" min="30" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="31" min="31" style="0" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="32" min="32" style="0" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="33" min="33" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="34" min="34" style="0" width="14"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2164,99 +2287,123 @@
       <c r="B2" s="14" t="n">
         <v>46315</v>
       </c>
-      <c r="D2" s="5" t="s">
-        <v>39</v>
+      <c r="D2" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="E2" s="14" t="n">
+        <v>46325</v>
+      </c>
+      <c r="G2" s="5" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>40</v>
+        <v>47</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>41</v>
+        <v>48</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>43</v>
+        <v>50</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="I4" s="6" t="s">
-        <v>45</v>
+        <v>52</v>
       </c>
       <c r="J4" s="6" t="s">
-        <v>46</v>
+        <v>53</v>
       </c>
       <c r="K4" s="6" t="s">
-        <v>47</v>
+        <v>54</v>
       </c>
       <c r="L4" s="6" t="s">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="M4" s="6" t="s">
-        <v>49</v>
+        <v>56</v>
       </c>
       <c r="N4" s="6" t="s">
-        <v>50</v>
+        <v>57</v>
       </c>
       <c r="O4" s="6" t="s">
-        <v>51</v>
+        <v>58</v>
       </c>
       <c r="P4" s="6" t="s">
         <v>7</v>
       </c>
       <c r="Q4" s="6" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="R4" s="6" t="s">
-        <v>53</v>
+        <v>60</v>
       </c>
       <c r="S4" s="6" t="s">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="T4" s="6" t="s">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="U4" s="6" t="s">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="V4" s="6" t="s">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="W4" s="6" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="X4" s="6" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="Y4" s="6" t="s">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="Z4" s="6" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="AA4" s="6" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="AB4" s="6" t="s">
-        <v>34</v>
+        <v>40</v>
+      </c>
+      <c r="AC4" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="AD4" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="AE4" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="AF4" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="AG4" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="AH4" s="6" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="15" t="s">
-        <v>57</v>
+        <v>70</v>
       </c>
       <c r="B5" s="16" t="n">
         <v>21000</v>
@@ -2265,19 +2412,19 @@
         <v>46310</v>
       </c>
       <c r="D5" s="18" t="s">
-        <v>58</v>
+        <v>71</v>
       </c>
       <c r="E5" s="19" t="n">
         <v>0</v>
       </c>
       <c r="F5" s="18" t="s">
-        <v>59</v>
+        <v>72</v>
       </c>
       <c r="G5" s="18" t="s">
-        <v>60</v>
+        <v>73</v>
       </c>
       <c r="H5" s="20" t="s">
-        <v>61</v>
+        <v>74</v>
       </c>
       <c r="I5" s="17" t="n">
         <v>46332</v>
@@ -2307,7 +2454,7 @@
         <v>46387</v>
       </c>
       <c r="P5" s="22" t="n">
-        <f aca="false">INDEX(Probability!$B$5:$F$13,MATCH(G5,Probability!$A$5:$A$13,0),MATCH(K5,Probability!$B$4:$F$4,0))</f>
+        <f aca="false">INDEX(Probability!$B$5:$F$19,MATCH(G5,Probability!$A$5:$A$19,0),MATCH(K5,Probability!$B$4:$F$4,0))</f>
         <v>0.5</v>
       </c>
       <c r="Q5" s="15" t="str">
@@ -2327,14 +2474,14 @@
         <v>11025</v>
       </c>
       <c r="U5" s="15" t="str">
-        <f aca="false">IF(G5="Cancelled","Lost",IF(Q5="No","Slips quarter",IF(OR(J5&lt;0,AND(J5&lt;=30,OR(G5="--None--",G5="Not started",G5="Engaging customer",G5="Negotiation"))),"Late","On time")))</f>
+        <f aca="false">IF(G5="Cancelled","Lost",IF(Q5="No","Slips quarter",IF(OR(J5&lt;0,AND(J5&lt;=30,OR(G5="--None--",G5="Not started",G5="Engaging customer",G5="Negotiation",G5="Billing blocker",G5="At risk: before notice deadline",G5="Notice received"))),"Late","On time")))</f>
         <v>Late</v>
       </c>
       <c r="V5" s="20" t="s">
-        <v>62</v>
+        <v>75</v>
       </c>
       <c r="W5" s="18" t="s">
-        <v>63</v>
+        <v>76</v>
       </c>
       <c r="X5" s="17" t="n">
         <v>46316</v>
@@ -2343,18 +2490,38 @@
         <v>2</v>
       </c>
       <c r="Z5" s="20" t="s">
-        <v>64</v>
+        <v>77</v>
       </c>
       <c r="AA5" s="20" t="s">
-        <v>65</v>
+        <v>78</v>
       </c>
       <c r="AB5" s="20" t="s">
-        <v>66</v>
+        <v>79</v>
+      </c>
+      <c r="AC5" s="18"/>
+      <c r="AD5" s="21" t="str">
+        <f aca="false">IF(AC5="","",C5-AC5)</f>
+        <v/>
+      </c>
+      <c r="AE5" s="8" t="str">
+        <f aca="false">IF(E5&gt;=0.2,"Over-usage: upsell line + CSM/Renewals task",IF(E5&lt;=-0.2,"Under-usage: flag CSM"&amp;IF(D5="Auto","; set At risk",""),""))</f>
+        <v/>
+      </c>
+      <c r="AF5" s="20" t="s">
+        <v>80</v>
+      </c>
+      <c r="AG5" s="22" t="n">
+        <f aca="false">IF(I5&lt;=O5,INDEX(Probability!$B$5:$F$19,MATCH(AF5,Probability!$A$5:$A$19,0),MATCH(IF(C5-$E$2&lt;0,"Overdue",IF(C5-$E$2&lt;=30,"0-30",IF(C5-$E$2&lt;=60,"31-60",IF(C5-$E$2&lt;=90,"61-90","&gt;90")))),Probability!$B$4:$F$4,0)),0)</f>
+        <v>0.7</v>
+      </c>
+      <c r="AH5" s="23" t="n">
+        <f aca="false">S5*AG5</f>
+        <v>15435</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="15" t="s">
-        <v>67</v>
+        <v>81</v>
       </c>
       <c r="B6" s="16" t="n">
         <v>48000</v>
@@ -2363,19 +2530,19 @@
         <v>46324</v>
       </c>
       <c r="D6" s="18" t="s">
-        <v>58</v>
+        <v>71</v>
       </c>
       <c r="E6" s="19" t="n">
         <v>0.12</v>
       </c>
       <c r="F6" s="18" t="s">
-        <v>68</v>
+        <v>82</v>
       </c>
       <c r="G6" s="18" t="s">
-        <v>69</v>
+        <v>83</v>
       </c>
       <c r="H6" s="20" t="s">
-        <v>70</v>
+        <v>84</v>
       </c>
       <c r="I6" s="17" t="n">
         <v>46324</v>
@@ -2405,8 +2572,8 @@
         <v>46387</v>
       </c>
       <c r="P6" s="22" t="n">
-        <f aca="false">INDEX(Probability!$B$5:$F$13,MATCH(G6,Probability!$A$5:$A$13,0),MATCH(K6,Probability!$B$4:$F$4,0))</f>
-        <v>0.9</v>
+        <f aca="false">INDEX(Probability!$B$5:$F$19,MATCH(G6,Probability!$A$5:$A$19,0),MATCH(K6,Probability!$B$4:$F$4,0))</f>
+        <v>0.25</v>
       </c>
       <c r="Q6" s="15" t="str">
         <f aca="false">IF(I6&lt;=O6,"Yes","No")</f>
@@ -2414,7 +2581,7 @@
       </c>
       <c r="R6" s="22" t="n">
         <f aca="false">IF(Q6="Yes",P6,0)</f>
-        <v>0.9</v>
+        <v>0.25</v>
       </c>
       <c r="S6" s="23" t="n">
         <f aca="false">SUMIFS(Products!$I:$I,Products!$A:$A,A6)</f>
@@ -2422,17 +2589,17 @@
       </c>
       <c r="T6" s="23" t="n">
         <f aca="false">S6*R6</f>
-        <v>45360</v>
+        <v>12600</v>
       </c>
       <c r="U6" s="15" t="str">
-        <f aca="false">IF(G6="Cancelled","Lost",IF(Q6="No","Slips quarter",IF(OR(J6&lt;0,AND(J6&lt;=30,OR(G6="--None--",G6="Not started",G6="Engaging customer",G6="Negotiation"))),"Late","On time")))</f>
-        <v>On time</v>
+        <f aca="false">IF(G6="Cancelled","Lost",IF(Q6="No","Slips quarter",IF(OR(J6&lt;0,AND(J6&lt;=30,OR(G6="--None--",G6="Not started",G6="Engaging customer",G6="Negotiation",G6="Billing blocker",G6="At risk: before notice deadline",G6="Notice received"))),"Late","On time")))</f>
+        <v>Late</v>
       </c>
       <c r="V6" s="20" t="s">
-        <v>71</v>
+        <v>85</v>
       </c>
       <c r="W6" s="18" t="s">
-        <v>63</v>
+        <v>76</v>
       </c>
       <c r="X6" s="17" t="n">
         <v>46315</v>
@@ -2441,16 +2608,36 @@
         <v>1</v>
       </c>
       <c r="Z6" s="20" t="s">
-        <v>72</v>
+        <v>86</v>
       </c>
       <c r="AA6" s="20" t="s">
-        <v>73</v>
+        <v>87</v>
       </c>
       <c r="AB6" s="20"/>
+      <c r="AC6" s="18"/>
+      <c r="AD6" s="21" t="str">
+        <f aca="false">IF(AC6="","",C6-AC6)</f>
+        <v/>
+      </c>
+      <c r="AE6" s="8" t="str">
+        <f aca="false">IF(E6&gt;=0.2,"Over-usage: upsell line + CSM/Renewals task",IF(E6&lt;=-0.2,"Under-usage: flag CSM"&amp;IF(D6="Auto","; set At risk",""),""))</f>
+        <v/>
+      </c>
+      <c r="AF6" s="20" t="s">
+        <v>88</v>
+      </c>
+      <c r="AG6" s="22" t="n">
+        <f aca="false">IF(I6&lt;=O6,INDEX(Probability!$B$5:$F$19,MATCH(AF6,Probability!$A$5:$A$19,0),MATCH(IF(C6-$E$2&lt;0,"Overdue",IF(C6-$E$2&lt;=30,"0-30",IF(C6-$E$2&lt;=60,"31-60",IF(C6-$E$2&lt;=90,"61-90","&gt;90")))),Probability!$B$4:$F$4,0)),0)</f>
+        <v>0.95</v>
+      </c>
+      <c r="AH6" s="23" t="n">
+        <f aca="false">S6*AG6</f>
+        <v>47880</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="15" t="s">
-        <v>74</v>
+        <v>89</v>
       </c>
       <c r="B7" s="16" t="n">
         <v>26000</v>
@@ -2459,19 +2646,19 @@
         <v>46328</v>
       </c>
       <c r="D7" s="18" t="s">
-        <v>75</v>
+        <v>90</v>
       </c>
       <c r="E7" s="19" t="n">
         <v>0</v>
       </c>
       <c r="F7" s="18" t="s">
-        <v>68</v>
+        <v>82</v>
       </c>
       <c r="G7" s="18" t="s">
-        <v>69</v>
+        <v>91</v>
       </c>
       <c r="H7" s="20" t="s">
-        <v>76</v>
+        <v>92</v>
       </c>
       <c r="I7" s="17" t="n">
         <v>46328</v>
@@ -2501,8 +2688,8 @@
         <v>46387</v>
       </c>
       <c r="P7" s="22" t="n">
-        <f aca="false">INDEX(Probability!$B$5:$F$13,MATCH(G7,Probability!$A$5:$A$13,0),MATCH(K7,Probability!$B$4:$F$4,0))</f>
-        <v>0.9</v>
+        <f aca="false">INDEX(Probability!$B$5:$F$19,MATCH(G7,Probability!$A$5:$A$19,0),MATCH(K7,Probability!$B$4:$F$4,0))</f>
+        <v>0.6</v>
       </c>
       <c r="Q7" s="15" t="str">
         <f aca="false">IF(I7&lt;=O7,"Yes","No")</f>
@@ -2510,7 +2697,7 @@
       </c>
       <c r="R7" s="22" t="n">
         <f aca="false">IF(Q7="Yes",P7,0)</f>
-        <v>0.9</v>
+        <v>0.6</v>
       </c>
       <c r="S7" s="23" t="n">
         <f aca="false">SUMIFS(Products!$I:$I,Products!$A:$A,A7)</f>
@@ -2518,17 +2705,17 @@
       </c>
       <c r="T7" s="23" t="n">
         <f aca="false">S7*R7</f>
-        <v>23400</v>
+        <v>15600</v>
       </c>
       <c r="U7" s="15" t="str">
-        <f aca="false">IF(G7="Cancelled","Lost",IF(Q7="No","Slips quarter",IF(OR(J7&lt;0,AND(J7&lt;=30,OR(G7="--None--",G7="Not started",G7="Engaging customer",G7="Negotiation"))),"Late","On time")))</f>
-        <v>On time</v>
+        <f aca="false">IF(G7="Cancelled","Lost",IF(Q7="No","Slips quarter",IF(OR(J7&lt;0,AND(J7&lt;=30,OR(G7="--None--",G7="Not started",G7="Engaging customer",G7="Negotiation",G7="Billing blocker",G7="At risk: before notice deadline",G7="Notice received"))),"Late","On time")))</f>
+        <v>Late</v>
       </c>
       <c r="V7" s="20" t="s">
-        <v>77</v>
+        <v>93</v>
       </c>
       <c r="W7" s="18" t="s">
-        <v>73</v>
+        <v>87</v>
       </c>
       <c r="X7" s="17" t="n">
         <v>46317</v>
@@ -2537,16 +2724,38 @@
         <v>3</v>
       </c>
       <c r="Z7" s="20" t="s">
-        <v>78</v>
+        <v>94</v>
       </c>
       <c r="AA7" s="20" t="s">
-        <v>79</v>
+        <v>95</v>
       </c>
       <c r="AB7" s="20"/>
+      <c r="AC7" s="18" t="n">
+        <v>30</v>
+      </c>
+      <c r="AD7" s="21" t="n">
+        <f aca="false">IF(AC7="","",C7-AC7)</f>
+        <v>46298</v>
+      </c>
+      <c r="AE7" s="8" t="str">
+        <f aca="false">IF(E7&gt;=0.2,"Over-usage: upsell line + CSM/Renewals task",IF(E7&lt;=-0.2,"Under-usage: flag CSM"&amp;IF(D7="Auto","; set At risk",""),""))</f>
+        <v/>
+      </c>
+      <c r="AF7" s="20" t="s">
+        <v>96</v>
+      </c>
+      <c r="AG7" s="22" t="n">
+        <f aca="false">IF(I7&lt;=O7,INDEX(Probability!$B$5:$F$19,MATCH(AF7,Probability!$A$5:$A$19,0),MATCH(IF(C7-$E$2&lt;0,"Overdue",IF(C7-$E$2&lt;=30,"0-30",IF(C7-$E$2&lt;=60,"31-60",IF(C7-$E$2&lt;=90,"61-90","&gt;90")))),Probability!$B$4:$F$4,0)),0)</f>
+        <v>0.97</v>
+      </c>
+      <c r="AH7" s="23" t="n">
+        <f aca="false">S7*AG7</f>
+        <v>25220</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="15" t="s">
-        <v>80</v>
+        <v>97</v>
       </c>
       <c r="B8" s="16" t="n">
         <v>45000</v>
@@ -2555,19 +2764,19 @@
         <v>46333</v>
       </c>
       <c r="D8" s="18" t="s">
-        <v>58</v>
+        <v>71</v>
       </c>
       <c r="E8" s="19" t="n">
         <v>-0.35</v>
       </c>
       <c r="F8" s="18" t="s">
-        <v>81</v>
+        <v>98</v>
       </c>
       <c r="G8" s="18" t="s">
-        <v>82</v>
+        <v>99</v>
       </c>
       <c r="H8" s="20" t="s">
-        <v>83</v>
+        <v>100</v>
       </c>
       <c r="I8" s="17" t="n">
         <v>46346</v>
@@ -2597,8 +2806,8 @@
         <v>46387</v>
       </c>
       <c r="P8" s="22" t="n">
-        <f aca="false">INDEX(Probability!$B$5:$F$13,MATCH(G8,Probability!$A$5:$A$13,0),MATCH(K8,Probability!$B$4:$F$4,0))</f>
-        <v>0.25</v>
+        <f aca="false">INDEX(Probability!$B$5:$F$19,MATCH(G8,Probability!$A$5:$A$19,0),MATCH(K8,Probability!$B$4:$F$4,0))</f>
+        <v>0.1</v>
       </c>
       <c r="Q8" s="15" t="str">
         <f aca="false">IF(I8&lt;=O8,"Yes","No")</f>
@@ -2606,7 +2815,7 @@
       </c>
       <c r="R8" s="22" t="n">
         <f aca="false">IF(Q8="Yes",P8,0)</f>
-        <v>0.25</v>
+        <v>0.1</v>
       </c>
       <c r="S8" s="23" t="n">
         <f aca="false">SUMIFS(Products!$I:$I,Products!$A:$A,A8)</f>
@@ -2614,17 +2823,17 @@
       </c>
       <c r="T8" s="23" t="n">
         <f aca="false">S8*R8</f>
-        <v>7500</v>
+        <v>3000</v>
       </c>
       <c r="U8" s="15" t="str">
-        <f aca="false">IF(G8="Cancelled","Lost",IF(Q8="No","Slips quarter",IF(OR(J8&lt;0,AND(J8&lt;=30,OR(G8="--None--",G8="Not started",G8="Engaging customer",G8="Negotiation"))),"Late","On time")))</f>
+        <f aca="false">IF(G8="Cancelled","Lost",IF(Q8="No","Slips quarter",IF(OR(J8&lt;0,AND(J8&lt;=30,OR(G8="--None--",G8="Not started",G8="Engaging customer",G8="Negotiation",G8="Billing blocker",G8="At risk: before notice deadline",G8="Notice received"))),"Late","On time")))</f>
         <v>Late</v>
       </c>
       <c r="V8" s="20" t="s">
-        <v>84</v>
+        <v>101</v>
       </c>
       <c r="W8" s="18" t="s">
-        <v>73</v>
+        <v>87</v>
       </c>
       <c r="X8" s="17" t="n">
         <v>46318</v>
@@ -2633,18 +2842,40 @@
         <v>4</v>
       </c>
       <c r="Z8" s="20" t="s">
-        <v>85</v>
+        <v>102</v>
       </c>
       <c r="AA8" s="20" t="s">
-        <v>86</v>
+        <v>103</v>
       </c>
       <c r="AB8" s="20" t="s">
-        <v>87</v>
+        <v>104</v>
+      </c>
+      <c r="AC8" s="18" t="n">
+        <v>30</v>
+      </c>
+      <c r="AD8" s="21" t="n">
+        <f aca="false">IF(AC8="","",C8-AC8)</f>
+        <v>46303</v>
+      </c>
+      <c r="AE8" s="8" t="str">
+        <f aca="false">IF(E8&gt;=0.2,"Over-usage: upsell line + CSM/Renewals task",IF(E8&lt;=-0.2,"Under-usage: flag CSM"&amp;IF(D8="Auto","; set At risk",""),""))</f>
+        <v>Under-usage: flag CSM</v>
+      </c>
+      <c r="AF8" s="20" t="s">
+        <v>83</v>
+      </c>
+      <c r="AG8" s="22" t="n">
+        <f aca="false">IF(I8&lt;=O8,INDEX(Probability!$B$5:$F$19,MATCH(AF8,Probability!$A$5:$A$19,0),MATCH(IF(C8-$E$2&lt;0,"Overdue",IF(C8-$E$2&lt;=30,"0-30",IF(C8-$E$2&lt;=60,"31-60",IF(C8-$E$2&lt;=90,"61-90","&gt;90")))),Probability!$B$4:$F$4,0)),0)</f>
+        <v>0.25</v>
+      </c>
+      <c r="AH8" s="23" t="n">
+        <f aca="false">S8*AG8</f>
+        <v>7500</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="15" t="s">
-        <v>88</v>
+        <v>105</v>
       </c>
       <c r="B9" s="16" t="n">
         <v>36000</v>
@@ -2653,19 +2884,19 @@
         <v>46370</v>
       </c>
       <c r="D9" s="18" t="s">
-        <v>58</v>
+        <v>71</v>
       </c>
       <c r="E9" s="19" t="n">
         <v>-0.1</v>
       </c>
       <c r="F9" s="18" t="s">
-        <v>59</v>
+        <v>72</v>
       </c>
       <c r="G9" s="18" t="s">
-        <v>89</v>
+        <v>106</v>
       </c>
       <c r="H9" s="20" t="s">
-        <v>90</v>
+        <v>107</v>
       </c>
       <c r="I9" s="17" t="n">
         <v>46356</v>
@@ -2695,7 +2926,7 @@
         <v>46387</v>
       </c>
       <c r="P9" s="22" t="n">
-        <f aca="false">INDEX(Probability!$B$5:$F$13,MATCH(G9,Probability!$A$5:$A$13,0),MATCH(K9,Probability!$B$4:$F$4,0))</f>
+        <f aca="false">INDEX(Probability!$B$5:$F$19,MATCH(G9,Probability!$A$5:$A$19,0),MATCH(K9,Probability!$B$4:$F$4,0))</f>
         <v>0.5</v>
       </c>
       <c r="Q9" s="15" t="str">
@@ -2715,14 +2946,14 @@
         <v>16632</v>
       </c>
       <c r="U9" s="15" t="str">
-        <f aca="false">IF(G9="Cancelled","Lost",IF(Q9="No","Slips quarter",IF(OR(J9&lt;0,AND(J9&lt;=30,OR(G9="--None--",G9="Not started",G9="Engaging customer",G9="Negotiation"))),"Late","On time")))</f>
+        <f aca="false">IF(G9="Cancelled","Lost",IF(Q9="No","Slips quarter",IF(OR(J9&lt;0,AND(J9&lt;=30,OR(G9="--None--",G9="Not started",G9="Engaging customer",G9="Negotiation",G9="Billing blocker",G9="At risk: before notice deadline",G9="Notice received"))),"Late","On time")))</f>
         <v>On time</v>
       </c>
       <c r="V9" s="20" t="s">
-        <v>91</v>
+        <v>108</v>
       </c>
       <c r="W9" s="18" t="s">
-        <v>63</v>
+        <v>76</v>
       </c>
       <c r="X9" s="17" t="n">
         <v>46315</v>
@@ -2731,16 +2962,36 @@
         <v>6</v>
       </c>
       <c r="Z9" s="20" t="s">
-        <v>92</v>
+        <v>109</v>
       </c>
       <c r="AA9" s="20" t="s">
-        <v>93</v>
+        <v>110</v>
       </c>
       <c r="AB9" s="20"/>
+      <c r="AC9" s="18"/>
+      <c r="AD9" s="21" t="str">
+        <f aca="false">IF(AC9="","",C9-AC9)</f>
+        <v/>
+      </c>
+      <c r="AE9" s="8" t="str">
+        <f aca="false">IF(E9&gt;=0.2,"Over-usage: upsell line + CSM/Renewals task",IF(E9&lt;=-0.2,"Under-usage: flag CSM"&amp;IF(D9="Auto","; set At risk",""),""))</f>
+        <v/>
+      </c>
+      <c r="AF9" s="20" t="s">
+        <v>106</v>
+      </c>
+      <c r="AG9" s="22" t="n">
+        <f aca="false">IF(I9&lt;=O9,INDEX(Probability!$B$5:$F$19,MATCH(AF9,Probability!$A$5:$A$19,0),MATCH(IF(C9-$E$2&lt;0,"Overdue",IF(C9-$E$2&lt;=30,"0-30",IF(C9-$E$2&lt;=60,"31-60",IF(C9-$E$2&lt;=90,"61-90","&gt;90")))),Probability!$B$4:$F$4,0)),0)</f>
+        <v>0.5</v>
+      </c>
+      <c r="AH9" s="23" t="n">
+        <f aca="false">S9*AG9</f>
+        <v>16632</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="15" t="s">
-        <v>94</v>
+        <v>111</v>
       </c>
       <c r="B10" s="16" t="n">
         <v>50000</v>
@@ -2749,19 +3000,19 @@
         <v>46344</v>
       </c>
       <c r="D10" s="18" t="s">
-        <v>58</v>
+        <v>71</v>
       </c>
       <c r="E10" s="19" t="n">
         <v>0.05</v>
       </c>
       <c r="F10" s="18" t="s">
-        <v>59</v>
+        <v>72</v>
       </c>
       <c r="G10" s="18" t="s">
-        <v>89</v>
+        <v>106</v>
       </c>
       <c r="H10" s="20" t="s">
-        <v>95</v>
+        <v>112</v>
       </c>
       <c r="I10" s="17" t="n">
         <v>46360</v>
@@ -2791,7 +3042,7 @@
         <v>46387</v>
       </c>
       <c r="P10" s="22" t="n">
-        <f aca="false">INDEX(Probability!$B$5:$F$13,MATCH(G10,Probability!$A$5:$A$13,0),MATCH(K10,Probability!$B$4:$F$4,0))</f>
+        <f aca="false">INDEX(Probability!$B$5:$F$19,MATCH(G10,Probability!$A$5:$A$19,0),MATCH(K10,Probability!$B$4:$F$4,0))</f>
         <v>0.4</v>
       </c>
       <c r="Q10" s="15" t="str">
@@ -2811,14 +3062,14 @@
         <v>21000</v>
       </c>
       <c r="U10" s="15" t="str">
-        <f aca="false">IF(G10="Cancelled","Lost",IF(Q10="No","Slips quarter",IF(OR(J10&lt;0,AND(J10&lt;=30,OR(G10="--None--",G10="Not started",G10="Engaging customer",G10="Negotiation"))),"Late","On time")))</f>
+        <f aca="false">IF(G10="Cancelled","Lost",IF(Q10="No","Slips quarter",IF(OR(J10&lt;0,AND(J10&lt;=30,OR(G10="--None--",G10="Not started",G10="Engaging customer",G10="Negotiation",G10="Billing blocker",G10="At risk: before notice deadline",G10="Notice received"))),"Late","On time")))</f>
         <v>Late</v>
       </c>
       <c r="V10" s="20" t="s">
-        <v>96</v>
+        <v>113</v>
       </c>
       <c r="W10" s="18" t="s">
-        <v>97</v>
+        <v>114</v>
       </c>
       <c r="X10" s="17" t="n">
         <v>46318</v>
@@ -2827,18 +3078,38 @@
         <v>5</v>
       </c>
       <c r="Z10" s="20" t="s">
-        <v>98</v>
+        <v>115</v>
       </c>
       <c r="AA10" s="20" t="s">
-        <v>99</v>
+        <v>116</v>
       </c>
       <c r="AB10" s="20" t="s">
-        <v>100</v>
+        <v>117</v>
+      </c>
+      <c r="AC10" s="18"/>
+      <c r="AD10" s="21" t="str">
+        <f aca="false">IF(AC10="","",C10-AC10)</f>
+        <v/>
+      </c>
+      <c r="AE10" s="8" t="str">
+        <f aca="false">IF(E10&gt;=0.2,"Over-usage: upsell line + CSM/Renewals task",IF(E10&lt;=-0.2,"Under-usage: flag CSM"&amp;IF(D10="Auto","; set At risk",""),""))</f>
+        <v/>
+      </c>
+      <c r="AF10" s="20" t="s">
+        <v>73</v>
+      </c>
+      <c r="AG10" s="22" t="n">
+        <f aca="false">IF(I10&lt;=O10,INDEX(Probability!$B$5:$F$19,MATCH(AF10,Probability!$A$5:$A$19,0),MATCH(IF(C10-$E$2&lt;0,"Overdue",IF(C10-$E$2&lt;=30,"0-30",IF(C10-$E$2&lt;=60,"31-60",IF(C10-$E$2&lt;=90,"61-90","&gt;90")))),Probability!$B$4:$F$4,0)),0)</f>
+        <v>0.75</v>
+      </c>
+      <c r="AH10" s="23" t="n">
+        <f aca="false">S10*AG10</f>
+        <v>39375</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="15" t="s">
-        <v>101</v>
+        <v>118</v>
       </c>
       <c r="B11" s="16" t="n">
         <v>28000</v>
@@ -2847,19 +3118,19 @@
         <v>46347</v>
       </c>
       <c r="D11" s="18" t="s">
-        <v>75</v>
+        <v>90</v>
       </c>
       <c r="E11" s="19" t="n">
         <v>0.08</v>
       </c>
       <c r="F11" s="18" t="s">
-        <v>68</v>
+        <v>82</v>
       </c>
       <c r="G11" s="18" t="s">
-        <v>69</v>
+        <v>91</v>
       </c>
       <c r="H11" s="20" t="s">
-        <v>102</v>
+        <v>119</v>
       </c>
       <c r="I11" s="17" t="n">
         <v>46347</v>
@@ -2889,8 +3160,8 @@
         <v>46387</v>
       </c>
       <c r="P11" s="22" t="n">
-        <f aca="false">INDEX(Probability!$B$5:$F$13,MATCH(G11,Probability!$A$5:$A$13,0),MATCH(K11,Probability!$B$4:$F$4,0))</f>
-        <v>0.85</v>
+        <f aca="false">INDEX(Probability!$B$5:$F$19,MATCH(G11,Probability!$A$5:$A$19,0),MATCH(K11,Probability!$B$4:$F$4,0))</f>
+        <v>0.7</v>
       </c>
       <c r="Q11" s="15" t="str">
         <f aca="false">IF(I11&lt;=O11,"Yes","No")</f>
@@ -2898,7 +3169,7 @@
       </c>
       <c r="R11" s="22" t="n">
         <f aca="false">IF(Q11="Yes",P11,0)</f>
-        <v>0.85</v>
+        <v>0.7</v>
       </c>
       <c r="S11" s="23" t="n">
         <f aca="false">SUMIFS(Products!$I:$I,Products!$A:$A,A11)</f>
@@ -2906,17 +3177,17 @@
       </c>
       <c r="T11" s="23" t="n">
         <f aca="false">S11*R11</f>
-        <v>24990</v>
+        <v>20580</v>
       </c>
       <c r="U11" s="15" t="str">
-        <f aca="false">IF(G11="Cancelled","Lost",IF(Q11="No","Slips quarter",IF(OR(J11&lt;0,AND(J11&lt;=30,OR(G11="--None--",G11="Not started",G11="Engaging customer",G11="Negotiation"))),"Late","On time")))</f>
+        <f aca="false">IF(G11="Cancelled","Lost",IF(Q11="No","Slips quarter",IF(OR(J11&lt;0,AND(J11&lt;=30,OR(G11="--None--",G11="Not started",G11="Engaging customer",G11="Negotiation",G11="Billing blocker",G11="At risk: before notice deadline",G11="Notice received"))),"Late","On time")))</f>
         <v>On time</v>
       </c>
       <c r="V11" s="20" t="s">
-        <v>103</v>
+        <v>120</v>
       </c>
       <c r="W11" s="18" t="s">
-        <v>63</v>
+        <v>76</v>
       </c>
       <c r="X11" s="17" t="n">
         <v>46317</v>
@@ -2925,16 +3196,38 @@
         <v>9</v>
       </c>
       <c r="Z11" s="20" t="s">
-        <v>104</v>
+        <v>121</v>
       </c>
       <c r="AA11" s="20" t="s">
-        <v>105</v>
+        <v>122</v>
       </c>
       <c r="AB11" s="20"/>
+      <c r="AC11" s="18" t="n">
+        <v>30</v>
+      </c>
+      <c r="AD11" s="21" t="n">
+        <f aca="false">IF(AC11="","",C11-AC11)</f>
+        <v>46317</v>
+      </c>
+      <c r="AE11" s="8" t="str">
+        <f aca="false">IF(E11&gt;=0.2,"Over-usage: upsell line + CSM/Renewals task",IF(E11&lt;=-0.2,"Under-usage: flag CSM"&amp;IF(D11="Auto","; set At risk",""),""))</f>
+        <v/>
+      </c>
+      <c r="AF11" s="20" t="s">
+        <v>96</v>
+      </c>
+      <c r="AG11" s="22" t="n">
+        <f aca="false">IF(I11&lt;=O11,INDEX(Probability!$B$5:$F$19,MATCH(AF11,Probability!$A$5:$A$19,0),MATCH(IF(C11-$E$2&lt;0,"Overdue",IF(C11-$E$2&lt;=30,"0-30",IF(C11-$E$2&lt;=60,"31-60",IF(C11-$E$2&lt;=90,"61-90","&gt;90")))),Probability!$B$4:$F$4,0)),0)</f>
+        <v>0.97</v>
+      </c>
+      <c r="AH11" s="23" t="n">
+        <f aca="false">S11*AG11</f>
+        <v>28518</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="15" t="s">
-        <v>106</v>
+        <v>123</v>
       </c>
       <c r="B12" s="16" t="n">
         <v>35000</v>
@@ -2943,19 +3236,19 @@
         <v>46354</v>
       </c>
       <c r="D12" s="18" t="s">
-        <v>58</v>
+        <v>71</v>
       </c>
       <c r="E12" s="19" t="n">
         <v>0.4</v>
       </c>
       <c r="F12" s="18" t="s">
-        <v>68</v>
+        <v>82</v>
       </c>
       <c r="G12" s="18" t="s">
-        <v>60</v>
+        <v>99</v>
       </c>
       <c r="H12" s="20" t="s">
-        <v>107</v>
+        <v>124</v>
       </c>
       <c r="I12" s="17" t="n">
         <v>46354</v>
@@ -2985,8 +3278,8 @@
         <v>46387</v>
       </c>
       <c r="P12" s="22" t="n">
-        <f aca="false">INDEX(Probability!$B$5:$F$13,MATCH(G12,Probability!$A$5:$A$13,0),MATCH(K12,Probability!$B$4:$F$4,0))</f>
-        <v>0.7</v>
+        <f aca="false">INDEX(Probability!$B$5:$F$19,MATCH(G12,Probability!$A$5:$A$19,0),MATCH(K12,Probability!$B$4:$F$4,0))</f>
+        <v>0.2</v>
       </c>
       <c r="Q12" s="15" t="str">
         <f aca="false">IF(I12&lt;=O12,"Yes","No")</f>
@@ -2994,7 +3287,7 @@
       </c>
       <c r="R12" s="22" t="n">
         <f aca="false">IF(Q12="Yes",P12,0)</f>
-        <v>0.7</v>
+        <v>0.2</v>
       </c>
       <c r="S12" s="23" t="n">
         <f aca="false">SUMIFS(Products!$I:$I,Products!$A:$A,A12)</f>
@@ -3002,17 +3295,17 @@
       </c>
       <c r="T12" s="23" t="n">
         <f aca="false">S12*R12</f>
-        <v>25725</v>
+        <v>7350</v>
       </c>
       <c r="U12" s="15" t="str">
-        <f aca="false">IF(G12="Cancelled","Lost",IF(Q12="No","Slips quarter",IF(OR(J12&lt;0,AND(J12&lt;=30,OR(G12="--None--",G12="Not started",G12="Engaging customer",G12="Negotiation"))),"Late","On time")))</f>
+        <f aca="false">IF(G12="Cancelled","Lost",IF(Q12="No","Slips quarter",IF(OR(J12&lt;0,AND(J12&lt;=30,OR(G12="--None--",G12="Not started",G12="Engaging customer",G12="Negotiation",G12="Billing blocker",G12="At risk: before notice deadline",G12="Notice received"))),"Late","On time")))</f>
         <v>On time</v>
       </c>
       <c r="V12" s="20" t="s">
-        <v>108</v>
+        <v>125</v>
       </c>
       <c r="W12" s="18" t="s">
-        <v>73</v>
+        <v>87</v>
       </c>
       <c r="X12" s="17" t="n">
         <v>46323</v>
@@ -3021,16 +3314,36 @@
         <v>8</v>
       </c>
       <c r="Z12" s="20" t="s">
-        <v>109</v>
+        <v>126</v>
       </c>
       <c r="AA12" s="20" t="s">
-        <v>63</v>
+        <v>76</v>
       </c>
       <c r="AB12" s="20"/>
+      <c r="AC12" s="18"/>
+      <c r="AD12" s="21" t="str">
+        <f aca="false">IF(AC12="","",C12-AC12)</f>
+        <v/>
+      </c>
+      <c r="AE12" s="8" t="str">
+        <f aca="false">IF(E12&gt;=0.2,"Over-usage: upsell line + CSM/Renewals task",IF(E12&lt;=-0.2,"Under-usage: flag CSM"&amp;IF(D12="Auto","; set At risk",""),""))</f>
+        <v>Over-usage: upsell line + CSM/Renewals task</v>
+      </c>
+      <c r="AF12" s="20" t="s">
+        <v>73</v>
+      </c>
+      <c r="AG12" s="22" t="n">
+        <f aca="false">IF(I12&lt;=O12,INDEX(Probability!$B$5:$F$19,MATCH(AF12,Probability!$A$5:$A$19,0),MATCH(IF(C12-$E$2&lt;0,"Overdue",IF(C12-$E$2&lt;=30,"0-30",IF(C12-$E$2&lt;=60,"31-60",IF(C12-$E$2&lt;=90,"61-90","&gt;90")))),Probability!$B$4:$F$4,0)),0)</f>
+        <v>0.75</v>
+      </c>
+      <c r="AH12" s="23" t="n">
+        <f aca="false">S12*AG12</f>
+        <v>27562.5</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="15" t="s">
-        <v>110</v>
+        <v>127</v>
       </c>
       <c r="B13" s="16" t="n">
         <v>46000</v>
@@ -3039,19 +3352,19 @@
         <v>46365</v>
       </c>
       <c r="D13" s="18" t="s">
-        <v>58</v>
+        <v>71</v>
       </c>
       <c r="E13" s="19" t="n">
         <v>0</v>
       </c>
       <c r="F13" s="18" t="s">
-        <v>59</v>
+        <v>72</v>
       </c>
       <c r="G13" s="18" t="s">
-        <v>60</v>
+        <v>83</v>
       </c>
       <c r="H13" s="20" t="s">
-        <v>111</v>
+        <v>128</v>
       </c>
       <c r="I13" s="17" t="n">
         <v>46365</v>
@@ -3081,8 +3394,8 @@
         <v>46387</v>
       </c>
       <c r="P13" s="22" t="n">
-        <f aca="false">INDEX(Probability!$B$5:$F$13,MATCH(G13,Probability!$A$5:$A$13,0),MATCH(K13,Probability!$B$4:$F$4,0))</f>
-        <v>0.7</v>
+        <f aca="false">INDEX(Probability!$B$5:$F$19,MATCH(G13,Probability!$A$5:$A$19,0),MATCH(K13,Probability!$B$4:$F$4,0))</f>
+        <v>0.35</v>
       </c>
       <c r="Q13" s="15" t="str">
         <f aca="false">IF(I13&lt;=O13,"Yes","No")</f>
@@ -3090,7 +3403,7 @@
       </c>
       <c r="R13" s="22" t="n">
         <f aca="false">IF(Q13="Yes",P13,0)</f>
-        <v>0.7</v>
+        <v>0.35</v>
       </c>
       <c r="S13" s="23" t="n">
         <f aca="false">SUMIFS(Products!$I:$I,Products!$A:$A,A13)</f>
@@ -3098,17 +3411,17 @@
       </c>
       <c r="T13" s="23" t="n">
         <f aca="false">S13*R13</f>
-        <v>33810</v>
+        <v>16905</v>
       </c>
       <c r="U13" s="15" t="str">
-        <f aca="false">IF(G13="Cancelled","Lost",IF(Q13="No","Slips quarter",IF(OR(J13&lt;0,AND(J13&lt;=30,OR(G13="--None--",G13="Not started",G13="Engaging customer",G13="Negotiation"))),"Late","On time")))</f>
+        <f aca="false">IF(G13="Cancelled","Lost",IF(Q13="No","Slips quarter",IF(OR(J13&lt;0,AND(J13&lt;=30,OR(G13="--None--",G13="Not started",G13="Engaging customer",G13="Negotiation",G13="Billing blocker",G13="At risk: before notice deadline",G13="Notice received"))),"Late","On time")))</f>
         <v>On time</v>
       </c>
       <c r="V13" s="20" t="s">
-        <v>112</v>
+        <v>129</v>
       </c>
       <c r="W13" s="18" t="s">
-        <v>63</v>
+        <v>76</v>
       </c>
       <c r="X13" s="17" t="n">
         <v>46322</v>
@@ -3117,16 +3430,36 @@
         <v>7</v>
       </c>
       <c r="Z13" s="20" t="s">
-        <v>113</v>
+        <v>130</v>
       </c>
       <c r="AA13" s="20" t="s">
-        <v>114</v>
+        <v>131</v>
       </c>
       <c r="AB13" s="20"/>
+      <c r="AC13" s="18"/>
+      <c r="AD13" s="21" t="str">
+        <f aca="false">IF(AC13="","",C13-AC13)</f>
+        <v/>
+      </c>
+      <c r="AE13" s="8" t="str">
+        <f aca="false">IF(E13&gt;=0.2,"Over-usage: upsell line + CSM/Renewals task",IF(E13&lt;=-0.2,"Under-usage: flag CSM"&amp;IF(D13="Auto","; set At risk",""),""))</f>
+        <v/>
+      </c>
+      <c r="AF13" s="20" t="s">
+        <v>73</v>
+      </c>
+      <c r="AG13" s="22" t="n">
+        <f aca="false">IF(I13&lt;=O13,INDEX(Probability!$B$5:$F$19,MATCH(AF13,Probability!$A$5:$A$19,0),MATCH(IF(C13-$E$2&lt;0,"Overdue",IF(C13-$E$2&lt;=30,"0-30",IF(C13-$E$2&lt;=60,"31-60",IF(C13-$E$2&lt;=90,"61-90","&gt;90")))),Probability!$B$4:$F$4,0)),0)</f>
+        <v>0.7</v>
+      </c>
+      <c r="AH13" s="23" t="n">
+        <f aca="false">S13*AG13</f>
+        <v>33810</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="15" t="s">
-        <v>115</v>
+        <v>132</v>
       </c>
       <c r="B14" s="16" t="n">
         <v>40000</v>
@@ -3135,19 +3468,19 @@
         <v>46375</v>
       </c>
       <c r="D14" s="18" t="s">
-        <v>75</v>
+        <v>90</v>
       </c>
       <c r="E14" s="19" t="n">
         <v>-0.2</v>
       </c>
       <c r="F14" s="18" t="s">
-        <v>59</v>
+        <v>72</v>
       </c>
       <c r="G14" s="18" t="s">
-        <v>82</v>
+        <v>133</v>
       </c>
       <c r="H14" s="20" t="s">
-        <v>116</v>
+        <v>134</v>
       </c>
       <c r="I14" s="17" t="n">
         <v>46375</v>
@@ -3177,8 +3510,8 @@
         <v>46387</v>
       </c>
       <c r="P14" s="22" t="n">
-        <f aca="false">INDEX(Probability!$B$5:$F$13,MATCH(G14,Probability!$A$5:$A$13,0),MATCH(K14,Probability!$B$4:$F$4,0))</f>
-        <v>0.35</v>
+        <f aca="false">INDEX(Probability!$B$5:$F$19,MATCH(G14,Probability!$A$5:$A$19,0),MATCH(K14,Probability!$B$4:$F$4,0))</f>
+        <v>0.4</v>
       </c>
       <c r="Q14" s="15" t="str">
         <f aca="false">IF(I14&lt;=O14,"Yes","No")</f>
@@ -3186,7 +3519,7 @@
       </c>
       <c r="R14" s="22" t="n">
         <f aca="false">IF(Q14="Yes",P14,0)</f>
-        <v>0.35</v>
+        <v>0.4</v>
       </c>
       <c r="S14" s="23" t="n">
         <f aca="false">SUMIFS(Products!$I:$I,Products!$A:$A,A14)</f>
@@ -3194,17 +3527,17 @@
       </c>
       <c r="T14" s="23" t="n">
         <f aca="false">S14*R14</f>
-        <v>11200</v>
+        <v>12800</v>
       </c>
       <c r="U14" s="15" t="str">
-        <f aca="false">IF(G14="Cancelled","Lost",IF(Q14="No","Slips quarter",IF(OR(J14&lt;0,AND(J14&lt;=30,OR(G14="--None--",G14="Not started",G14="Engaging customer",G14="Negotiation"))),"Late","On time")))</f>
+        <f aca="false">IF(G14="Cancelled","Lost",IF(Q14="No","Slips quarter",IF(OR(J14&lt;0,AND(J14&lt;=30,OR(G14="--None--",G14="Not started",G14="Engaging customer",G14="Negotiation",G14="Billing blocker",G14="At risk: before notice deadline",G14="Notice received"))),"Late","On time")))</f>
         <v>On time</v>
       </c>
       <c r="V14" s="20" t="s">
-        <v>117</v>
+        <v>135</v>
       </c>
       <c r="W14" s="18" t="s">
-        <v>73</v>
+        <v>87</v>
       </c>
       <c r="X14" s="17" t="n">
         <v>46325</v>
@@ -3213,16 +3546,38 @@
         <v>10</v>
       </c>
       <c r="Z14" s="20" t="s">
-        <v>118</v>
+        <v>136</v>
       </c>
       <c r="AA14" s="20" t="s">
-        <v>63</v>
+        <v>76</v>
       </c>
       <c r="AB14" s="20"/>
+      <c r="AC14" s="18" t="n">
+        <v>30</v>
+      </c>
+      <c r="AD14" s="21" t="n">
+        <f aca="false">IF(AC14="","",C14-AC14)</f>
+        <v>46345</v>
+      </c>
+      <c r="AE14" s="8" t="str">
+        <f aca="false">IF(E14&gt;=0.2,"Over-usage: upsell line + CSM/Renewals task",IF(E14&lt;=-0.2,"Under-usage: flag CSM"&amp;IF(D14="Auto","; set At risk",""),""))</f>
+        <v>Under-usage: flag CSM; set At risk</v>
+      </c>
+      <c r="AF14" s="20" t="s">
+        <v>133</v>
+      </c>
+      <c r="AG14" s="22" t="n">
+        <f aca="false">IF(I14&lt;=O14,INDEX(Probability!$B$5:$F$19,MATCH(AF14,Probability!$A$5:$A$19,0),MATCH(IF(C14-$E$2&lt;0,"Overdue",IF(C14-$E$2&lt;=30,"0-30",IF(C14-$E$2&lt;=60,"31-60",IF(C14-$E$2&lt;=90,"61-90","&gt;90")))),Probability!$B$4:$F$4,0)),0)</f>
+        <v>0.4</v>
+      </c>
+      <c r="AH14" s="23" t="n">
+        <f aca="false">S14*AG14</f>
+        <v>12800</v>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>119</v>
+        <v>137</v>
       </c>
       <c r="B15" s="24" t="n">
         <f aca="false">SUM(B5:B14)</f>
@@ -3234,65 +3589,69 @@
       </c>
       <c r="T15" s="24" t="n">
         <f aca="false">SUM(T5:T14)</f>
-        <v>220642</v>
+        <v>137492</v>
+      </c>
+      <c r="AH15" s="24" t="n">
+        <f aca="false">SUM(AH5:AH14)</f>
+        <v>254732.5</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="25" t="s">
-        <v>120</v>
+        <v>138</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="26" t="s">
-        <v>121</v>
+        <v>139</v>
       </c>
       <c r="B19" s="26" t="s">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="C19" s="26" t="s">
-        <v>122</v>
+        <v>140</v>
       </c>
       <c r="D19" s="26" t="s">
-        <v>123</v>
+        <v>141</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="15" t="s">
-        <v>124</v>
+        <v>142</v>
       </c>
       <c r="B20" s="23" t="n">
         <f aca="false">SUMIFS(T5:T14,U5:U14,"On time")</f>
-        <v>181117</v>
+        <v>74267</v>
       </c>
       <c r="C20" s="23" t="n">
         <f aca="false">SUMIFS(S5:S14,U5:U14,"On time")</f>
-        <v>256114</v>
+        <v>179714</v>
       </c>
       <c r="D20" s="15" t="str">
         <f aca="false">COUNTIFS(U5:U14,"On time")&amp;" renewals"</f>
-        <v>7 renewals</v>
+        <v>5 renewals</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="15" t="s">
-        <v>125</v>
+        <v>143</v>
       </c>
       <c r="B21" s="23" t="n">
         <f aca="false">SUMIFS(T5:T14,U5:U14,"Late")</f>
-        <v>39525</v>
+        <v>63225</v>
       </c>
       <c r="C21" s="23" t="n">
         <f aca="false">SUMIFS(S5:S14,U5:U14,"Late")</f>
-        <v>104550</v>
+        <v>180950</v>
       </c>
       <c r="D21" s="15" t="str">
         <f aca="false">COUNTIFS(U5:U14,"Late")&amp;" renewals"</f>
-        <v>3 renewals</v>
+        <v>5 renewals</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="15" t="s">
-        <v>126</v>
+        <v>144</v>
       </c>
       <c r="B22" s="23" t="n">
         <f aca="false">SUMIFS(T5:T14,U5:U14,"Slips quarter")</f>
@@ -3309,11 +3668,11 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="7" t="s">
-        <v>127</v>
+        <v>145</v>
       </c>
       <c r="B23" s="27" t="n">
         <f aca="false">SUM(B20:B22)</f>
-        <v>220642</v>
+        <v>137492</v>
       </c>
       <c r="C23" s="23" t="n">
         <f aca="false">SUM(C20:C22)</f>
@@ -3323,12 +3682,12 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="2" t="s">
-        <v>128</v>
+        <v>146</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="15" t="s">
-        <v>129</v>
+        <v>147</v>
       </c>
       <c r="B25" s="29" t="n">
         <f aca="false">'Opp summary'!E15</f>
@@ -3337,7 +3696,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="15" t="s">
-        <v>130</v>
+        <v>148</v>
       </c>
       <c r="B26" s="29" t="n">
         <f aca="false">'Opp summary'!F15</f>
@@ -3346,7 +3705,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="15" t="s">
-        <v>131</v>
+        <v>149</v>
       </c>
       <c r="B27" s="29" t="n">
         <f aca="false">'Opp summary'!H15</f>
@@ -3355,7 +3714,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="15" t="s">
-        <v>132</v>
+        <v>150</v>
       </c>
       <c r="B28" s="30" t="n">
         <f aca="false">(B15+B25+B27)/B15</f>
@@ -3364,11 +3723,43 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="15" t="s">
-        <v>133</v>
+        <v>151</v>
       </c>
       <c r="B29" s="30" t="n">
         <f aca="false">S15/B15</f>
         <v>0.961770666666667</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="25" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="15" t="s">
+        <v>152</v>
+      </c>
+      <c r="B32" s="27" t="n">
+        <f aca="false">T15</f>
+        <v>137492</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="15" t="s">
+        <v>153</v>
+      </c>
+      <c r="B33" s="27" t="n">
+        <f aca="false">AH15</f>
+        <v>254732.5</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="15" t="s">
+        <v>154</v>
+      </c>
+      <c r="B34" s="27" t="n">
+        <f aca="false">B33-B32</f>
+        <v>117240.5</v>
       </c>
     </row>
   </sheetData>
@@ -3419,9 +3810,36 @@
       <formula>LEFT(AB5,3)="Yes"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="4">
+  <conditionalFormatting sqref="G5:G14">
+    <cfRule type="expression" priority="13" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
+      <formula>AND(G5&lt;&gt;"",INDEX(Probability!$H$5:$H$19,MATCH(G5,Probability!$A$5:$A$19,0))&lt;&gt;"Both",INDEX(Probability!$H$5:$H$19,MATCH(G5,Probability!$A$5:$A$19,0))&lt;&gt;$D5)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AF5:AF14">
+    <cfRule type="expression" priority="14" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
+      <formula>AND(AF5&lt;&gt;"",INDEX(Probability!$H$5:$H$19,MATCH(AF5,Probability!$A$5:$A$19,0))&lt;&gt;"Both",INDEX(Probability!$H$5:$H$19,MATCH(AF5,Probability!$A$5:$A$19,0))&lt;&gt;$D5)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AE5:AE14">
+    <cfRule type="expression" priority="15" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="2">
+      <formula>LEFT(AE5,5)="Under"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="16" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="3">
+      <formula>LEFT(AE5,4)="Over"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AD5:AD14">
+    <cfRule type="expression" priority="17" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
+      <formula>AND(AD5&lt;&gt;"",AD5&lt;$B$2)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="5">
     <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="G5:G14" type="list">
-      <formula1>Probability!$A$5:$A$13</formula1>
+      <formula1>Probability!$A$5:$A$19</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="AF5:AF14" type="list">
+      <formula1>Probability!$A$5:$A$19</formula1>
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="F5:F14" type="list">
@@ -3474,12 +3892,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>134</v>
+        <v>155</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="31" t="s">
-        <v>135</v>
+        <v>156</v>
       </c>
       <c r="B2" s="31"/>
       <c r="C2" s="31"/>
@@ -3500,66 +3918,66 @@
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>136</v>
+        <v>157</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>137</v>
+        <v>158</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>138</v>
+        <v>159</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>139</v>
+        <v>160</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>140</v>
+        <v>161</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>141</v>
+        <v>162</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>142</v>
+        <v>163</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>143</v>
+        <v>164</v>
       </c>
       <c r="I4" s="6" t="s">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="J4" s="6" t="s">
-        <v>144</v>
+        <v>165</v>
       </c>
       <c r="K4" s="6" t="s">
-        <v>145</v>
+        <v>166</v>
       </c>
       <c r="L4" s="6" t="s">
-        <v>146</v>
+        <v>167</v>
       </c>
       <c r="M4" s="6" t="s">
-        <v>147</v>
+        <v>168</v>
       </c>
       <c r="N4" s="6" t="s">
-        <v>148</v>
+        <v>169</v>
       </c>
       <c r="O4" s="6" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="P4" s="6" t="s">
-        <v>149</v>
+        <v>170</v>
       </c>
       <c r="Q4" s="6" t="s">
-        <v>150</v>
+        <v>171</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="15" t="s">
-        <v>57</v>
+        <v>70</v>
       </c>
       <c r="B5" s="15" t="s">
-        <v>151</v>
+        <v>172</v>
       </c>
       <c r="C5" s="18" t="s">
-        <v>152</v>
+        <v>173</v>
       </c>
       <c r="D5" s="18" t="n">
         <v>1</v>
@@ -3606,18 +4024,18 @@
         <v>0</v>
       </c>
       <c r="Q5" s="15" t="s">
-        <v>153</v>
+        <v>174</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="15" t="s">
-        <v>67</v>
+        <v>81</v>
       </c>
       <c r="B6" s="15" t="s">
-        <v>154</v>
+        <v>175</v>
       </c>
       <c r="C6" s="18" t="s">
-        <v>152</v>
+        <v>173</v>
       </c>
       <c r="D6" s="18" t="n">
         <v>1</v>
@@ -3664,18 +4082,18 @@
         <v>0</v>
       </c>
       <c r="Q6" s="15" t="s">
-        <v>155</v>
+        <v>176</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="15" t="s">
-        <v>74</v>
+        <v>89</v>
       </c>
       <c r="B7" s="15" t="s">
-        <v>151</v>
+        <v>172</v>
       </c>
       <c r="C7" s="18" t="s">
-        <v>152</v>
+        <v>173</v>
       </c>
       <c r="D7" s="18" t="n">
         <v>1</v>
@@ -3722,18 +4140,18 @@
         <v>0</v>
       </c>
       <c r="Q7" s="15" t="s">
-        <v>156</v>
+        <v>177</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="15" t="s">
-        <v>80</v>
+        <v>97</v>
       </c>
       <c r="B8" s="15" t="s">
-        <v>157</v>
+        <v>178</v>
       </c>
       <c r="C8" s="18" t="s">
-        <v>158</v>
+        <v>179</v>
       </c>
       <c r="D8" s="18" t="n">
         <v>1</v>
@@ -3780,18 +4198,18 @@
         <v>-15000</v>
       </c>
       <c r="Q8" s="15" t="s">
-        <v>159</v>
+        <v>180</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="15" t="s">
-        <v>88</v>
+        <v>105</v>
       </c>
       <c r="B9" s="15" t="s">
-        <v>160</v>
+        <v>181</v>
       </c>
       <c r="C9" s="18" t="s">
-        <v>152</v>
+        <v>173</v>
       </c>
       <c r="D9" s="18" t="n">
         <v>2</v>
@@ -3838,18 +4256,18 @@
         <v>0</v>
       </c>
       <c r="Q9" s="15" t="s">
-        <v>161</v>
+        <v>182</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="15" t="s">
-        <v>94</v>
+        <v>111</v>
       </c>
       <c r="B10" s="15" t="s">
-        <v>157</v>
+        <v>178</v>
       </c>
       <c r="C10" s="18" t="s">
-        <v>152</v>
+        <v>173</v>
       </c>
       <c r="D10" s="18" t="n">
         <v>1</v>
@@ -3899,13 +4317,13 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="15" t="s">
-        <v>101</v>
+        <v>118</v>
       </c>
       <c r="B11" s="15" t="s">
-        <v>151</v>
+        <v>172</v>
       </c>
       <c r="C11" s="18" t="s">
-        <v>152</v>
+        <v>173</v>
       </c>
       <c r="D11" s="18" t="n">
         <v>1</v>
@@ -3952,18 +4370,18 @@
         <v>0</v>
       </c>
       <c r="Q11" s="15" t="s">
-        <v>162</v>
+        <v>183</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="15" t="s">
-        <v>106</v>
+        <v>123</v>
       </c>
       <c r="B12" s="15" t="s">
-        <v>151</v>
+        <v>172</v>
       </c>
       <c r="C12" s="18" t="s">
-        <v>152</v>
+        <v>173</v>
       </c>
       <c r="D12" s="18" t="n">
         <v>1</v>
@@ -4010,18 +4428,18 @@
         <v>0</v>
       </c>
       <c r="Q12" s="15" t="s">
-        <v>163</v>
+        <v>184</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="15" t="s">
-        <v>106</v>
+        <v>123</v>
       </c>
       <c r="B13" s="15" t="s">
-        <v>164</v>
+        <v>185</v>
       </c>
       <c r="C13" s="18" t="s">
-        <v>165</v>
+        <v>186</v>
       </c>
       <c r="D13" s="18" t="n">
         <v>1</v>
@@ -4068,18 +4486,18 @@
         <v>0</v>
       </c>
       <c r="Q13" s="15" t="s">
-        <v>166</v>
+        <v>187</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="15" t="s">
-        <v>110</v>
+        <v>127</v>
       </c>
       <c r="B14" s="15" t="s">
-        <v>154</v>
+        <v>175</v>
       </c>
       <c r="C14" s="18" t="s">
-        <v>152</v>
+        <v>173</v>
       </c>
       <c r="D14" s="18" t="n">
         <v>1</v>
@@ -4129,13 +4547,13 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="15" t="s">
-        <v>115</v>
+        <v>132</v>
       </c>
       <c r="B15" s="15" t="s">
-        <v>154</v>
+        <v>175</v>
       </c>
       <c r="C15" s="18" t="s">
-        <v>158</v>
+        <v>179</v>
       </c>
       <c r="D15" s="18" t="n">
         <v>1</v>
@@ -4182,12 +4600,12 @@
         <v>-8000</v>
       </c>
       <c r="Q15" s="15" t="s">
-        <v>167</v>
+        <v>188</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>119</v>
+        <v>137</v>
       </c>
       <c r="E17" s="24" t="n">
         <f aca="false">SUM(E5:E15)</f>
@@ -4216,12 +4634,12 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>168</v>
+        <v>189</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="31" t="s">
-        <v>169</v>
+        <v>190</v>
       </c>
       <c r="B20" s="31"/>
       <c r="C20" s="31"/>
@@ -4302,42 +4720,42 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>170</v>
+        <v>191</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="s">
-        <v>136</v>
+        <v>157</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>140</v>
+        <v>161</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>171</v>
+        <v>192</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>172</v>
+        <v>193</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>173</v>
+        <v>194</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>174</v>
+        <v>195</v>
       </c>
       <c r="G3" s="6" t="s">
-        <v>175</v>
+        <v>196</v>
       </c>
       <c r="H3" s="6" t="s">
-        <v>176</v>
+        <v>197</v>
       </c>
       <c r="I3" s="6" t="s">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="J3" s="6" t="s">
-        <v>177</v>
+        <v>198</v>
       </c>
       <c r="K3" s="6" t="s">
-        <v>178</v>
+        <v>199</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4802,7 +5220,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>119</v>
+        <v>137</v>
       </c>
       <c r="B14" s="24" t="n">
         <f aca="false">SUM(B4:B13)</f>
@@ -4847,7 +5265,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="34" t="s">
-        <v>179</v>
+        <v>200</v>
       </c>
       <c r="E15" s="35" t="n">
         <f aca="false">E14</f>
@@ -4864,7 +5282,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="12" t="s">
-        <v>180</v>
+        <v>201</v>
       </c>
       <c r="B17" s="12" t="str">
         <f aca="false">IF(ABS(I14-Pipeline!S15)&lt;1,"OK","MISMATCH")</f>
@@ -4919,47 +5337,47 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>181</v>
+        <v>202</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="s">
-        <v>50</v>
+        <v>57</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>49</v>
+        <v>56</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>182</v>
+        <v>203</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>40</v>
+        <v>47</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>183</v>
+        <v>204</v>
       </c>
       <c r="G3" s="6" t="s">
-        <v>184</v>
+        <v>205</v>
       </c>
       <c r="H3" s="6" t="s">
-        <v>185</v>
+        <v>206</v>
       </c>
       <c r="I3" s="6" t="s">
-        <v>186</v>
+        <v>207</v>
       </c>
       <c r="J3" s="6" t="s">
-        <v>173</v>
+        <v>194</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="15" t="s">
-        <v>187</v>
+        <v>208</v>
       </c>
       <c r="B4" s="15" t="s">
-        <v>188</v>
+        <v>209</v>
       </c>
       <c r="C4" s="15" t="n">
         <f aca="false">COUNTIFS(Pipeline!$M$5:$M$14,B4)</f>
@@ -4975,15 +5393,15 @@
       </c>
       <c r="F4" s="23" t="n">
         <f aca="false">SUMIFS(Pipeline!$T$5:$T$14,Pipeline!$M$5:$M$14,B4)</f>
-        <v>56385</v>
+        <v>23625</v>
       </c>
       <c r="G4" s="23" t="n">
         <f aca="false">SUMIFS(Pipeline!$T$5:$T$14,Pipeline!$M$5:$M$14,B4,Pipeline!$U$5:$U$14,"On time")</f>
-        <v>45360</v>
+        <v>0</v>
       </c>
       <c r="H4" s="23" t="n">
         <f aca="false">SUMIFS(Pipeline!$T$5:$T$14,Pipeline!$M$5:$M$14,B4,Pipeline!$U$5:$U$14,"Late")</f>
-        <v>11025</v>
+        <v>23625</v>
       </c>
       <c r="I4" s="23" t="n">
         <f aca="false">SUMIFS(Pipeline!$B$5:$B$14,Pipeline!$M$5:$M$14,B4,Pipeline!$L$5:$L$14,"YES")</f>
@@ -4996,10 +5414,10 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="15" t="s">
-        <v>187</v>
+        <v>208</v>
       </c>
       <c r="B5" s="15" t="s">
-        <v>189</v>
+        <v>210</v>
       </c>
       <c r="C5" s="15" t="n">
         <f aca="false">COUNTIFS(Pipeline!$M$5:$M$14,B5)</f>
@@ -5015,15 +5433,15 @@
       </c>
       <c r="F5" s="23" t="n">
         <f aca="false">SUMIFS(Pipeline!$T$5:$T$14,Pipeline!$M$5:$M$14,B5)</f>
-        <v>102615</v>
+        <v>67530</v>
       </c>
       <c r="G5" s="23" t="n">
         <f aca="false">SUMIFS(Pipeline!$T$5:$T$14,Pipeline!$M$5:$M$14,B5,Pipeline!$U$5:$U$14,"On time")</f>
-        <v>74115</v>
+        <v>27930</v>
       </c>
       <c r="H5" s="23" t="n">
         <f aca="false">SUMIFS(Pipeline!$T$5:$T$14,Pipeline!$M$5:$M$14,B5,Pipeline!$U$5:$U$14,"Late")</f>
-        <v>28500</v>
+        <v>39600</v>
       </c>
       <c r="I5" s="23" t="n">
         <f aca="false">SUMIFS(Pipeline!$B$5:$B$14,Pipeline!$M$5:$M$14,B5,Pipeline!$L$5:$L$14,"YES")</f>
@@ -5036,10 +5454,10 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="15" t="s">
-        <v>187</v>
+        <v>208</v>
       </c>
       <c r="B6" s="15" t="s">
-        <v>190</v>
+        <v>211</v>
       </c>
       <c r="C6" s="15" t="n">
         <f aca="false">COUNTIFS(Pipeline!$M$5:$M$14,B6)</f>
@@ -5055,11 +5473,11 @@
       </c>
       <c r="F6" s="23" t="n">
         <f aca="false">SUMIFS(Pipeline!$T$5:$T$14,Pipeline!$M$5:$M$14,B6)</f>
-        <v>61642</v>
+        <v>46337</v>
       </c>
       <c r="G6" s="23" t="n">
         <f aca="false">SUMIFS(Pipeline!$T$5:$T$14,Pipeline!$M$5:$M$14,B6,Pipeline!$U$5:$U$14,"On time")</f>
-        <v>61642</v>
+        <v>46337</v>
       </c>
       <c r="H6" s="23" t="n">
         <f aca="false">SUMIFS(Pipeline!$T$5:$T$14,Pipeline!$M$5:$M$14,B6,Pipeline!$U$5:$U$14,"Late")</f>
@@ -5076,7 +5494,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>191</v>
+        <v>212</v>
       </c>
       <c r="C7" s="2" t="n">
         <f aca="false">SUM(C4:C6)</f>
@@ -5092,15 +5510,15 @@
       </c>
       <c r="F7" s="24" t="n">
         <f aca="false">SUM(F4:F6)</f>
-        <v>220642</v>
+        <v>137492</v>
       </c>
       <c r="G7" s="24" t="n">
         <f aca="false">SUM(G4:G6)</f>
-        <v>181117</v>
+        <v>74267</v>
       </c>
       <c r="H7" s="24" t="n">
         <f aca="false">SUM(H4:H6)</f>
-        <v>39525</v>
+        <v>63225</v>
       </c>
       <c r="I7" s="24" t="n">
         <f aca="false">SUM(I4:I6)</f>
@@ -5137,50 +5555,54 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:H27"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="2" style="0" width="11"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="70"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="11"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>192</v>
+        <v>213</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>193</v>
+        <v>214</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>194</v>
+        <v>215</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>195</v>
+        <v>216</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>196</v>
+        <v>217</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>197</v>
+        <v>218</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>198</v>
+        <v>219</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>199</v>
+        <v>220</v>
+      </c>
+      <c r="H4" s="6" t="s">
+        <v>221</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>200</v>
+        <v>222</v>
       </c>
       <c r="B5" s="36" t="n">
         <v>0</v>
@@ -5198,12 +5620,15 @@
         <v>0</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>201</v>
+        <v>223</v>
+      </c>
+      <c r="H5" s="15" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>202</v>
+        <v>99</v>
       </c>
       <c r="B6" s="36" t="n">
         <v>0.05</v>
@@ -5221,12 +5646,15 @@
         <v>0.35</v>
       </c>
       <c r="G6" s="8" t="s">
-        <v>203</v>
+        <v>224</v>
+      </c>
+      <c r="H6" s="15" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B7" s="36" t="n">
         <v>0.1</v>
@@ -5244,12 +5672,15 @@
         <v>0.5</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>204</v>
+        <v>225</v>
+      </c>
+      <c r="H7" s="15" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
-        <v>89</v>
+        <v>106</v>
       </c>
       <c r="B8" s="36" t="n">
         <v>0.2</v>
@@ -5267,12 +5698,15 @@
         <v>0.55</v>
       </c>
       <c r="G8" s="8" t="s">
-        <v>205</v>
+        <v>226</v>
+      </c>
+      <c r="H8" s="15" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>60</v>
+        <v>73</v>
       </c>
       <c r="B9" s="36" t="n">
         <v>0.5</v>
@@ -5290,12 +5724,15 @@
         <v>0.6</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>206</v>
+        <v>227</v>
+      </c>
+      <c r="H9" s="15" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
-        <v>69</v>
+        <v>80</v>
       </c>
       <c r="B10" s="36" t="n">
         <v>0.7</v>
@@ -5313,12 +5750,15 @@
         <v>0.75</v>
       </c>
       <c r="G10" s="8" t="s">
-        <v>207</v>
+        <v>228</v>
+      </c>
+      <c r="H10" s="15" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>208</v>
+        <v>88</v>
       </c>
       <c r="B11" s="36" t="n">
         <v>0.95</v>
@@ -5336,12 +5776,15 @@
         <v>0.9</v>
       </c>
       <c r="G11" s="8" t="s">
-        <v>209</v>
+        <v>229</v>
+      </c>
+      <c r="H11" s="15" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>210</v>
+        <v>230</v>
       </c>
       <c r="B12" s="36" t="n">
         <v>1</v>
@@ -5359,12 +5802,15 @@
         <v>1</v>
       </c>
       <c r="G12" s="8" t="s">
-        <v>211</v>
+        <v>231</v>
+      </c>
+      <c r="H12" s="15" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
-        <v>212</v>
+        <v>232</v>
       </c>
       <c r="B13" s="36" t="n">
         <v>0</v>
@@ -5382,48 +5828,242 @@
         <v>0</v>
       </c>
       <c r="G13" s="8" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B15" s="31" t="s">
-        <v>214</v>
-      </c>
-      <c r="C15" s="31"/>
-      <c r="D15" s="31"/>
-      <c r="E15" s="31"/>
-      <c r="F15" s="31"/>
-      <c r="G15" s="31"/>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B16" s="31"/>
-      <c r="C16" s="31"/>
-      <c r="D16" s="31"/>
-      <c r="E16" s="31"/>
-      <c r="F16" s="31"/>
-      <c r="G16" s="31"/>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B17" s="31"/>
-      <c r="C17" s="31"/>
-      <c r="D17" s="31"/>
-      <c r="E17" s="31"/>
-      <c r="F17" s="31"/>
-      <c r="G17" s="31"/>
+        <v>233</v>
+      </c>
+      <c r="H13" s="15" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="B14" s="36" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="C14" s="36" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="D14" s="36" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="E14" s="36" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="F14" s="36" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="G14" s="8" t="s">
+        <v>235</v>
+      </c>
+      <c r="H14" s="15" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="B15" s="36" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="C15" s="36" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="D15" s="36" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="E15" s="36" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="F15" s="36" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="G15" s="8" t="s">
+        <v>236</v>
+      </c>
+      <c r="H15" s="15" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="7" t="s">
+        <v>133</v>
+      </c>
+      <c r="B16" s="36" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="C16" s="36" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="D16" s="36" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="E16" s="36" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="F16" s="36" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G16" s="8" t="s">
+        <v>237</v>
+      </c>
+      <c r="H16" s="15" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="7" t="s">
+        <v>238</v>
+      </c>
+      <c r="B17" s="36" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C17" s="36" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="D17" s="36" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="E17" s="36" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="F17" s="36" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="G17" s="8" t="s">
+        <v>239</v>
+      </c>
+      <c r="H17" s="15" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="7" t="s">
+        <v>240</v>
+      </c>
+      <c r="B18" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="36" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D18" s="36" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E18" s="36" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F18" s="36" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G18" s="8" t="s">
+        <v>241</v>
+      </c>
+      <c r="H18" s="15" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="7" t="s">
+        <v>242</v>
+      </c>
+      <c r="B19" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="C19" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="D19" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="E19" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="F19" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="G19" s="8" t="s">
+        <v>243</v>
+      </c>
+      <c r="H19" s="15" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B21" s="31" t="s">
+        <v>244</v>
+      </c>
+      <c r="C21" s="31"/>
+      <c r="D21" s="31"/>
+      <c r="E21" s="31"/>
+      <c r="F21" s="31"/>
+      <c r="G21" s="31"/>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B22" s="31"/>
+      <c r="C22" s="31"/>
+      <c r="D22" s="31"/>
+      <c r="E22" s="31"/>
+      <c r="F22" s="31"/>
+      <c r="G22" s="31"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B23" s="31"/>
+      <c r="C23" s="31"/>
+      <c r="D23" s="31"/>
+      <c r="E23" s="31"/>
+      <c r="F23" s="31"/>
+      <c r="G23" s="31"/>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B25" s="31" t="s">
+        <v>245</v>
+      </c>
+      <c r="C25" s="31"/>
+      <c r="D25" s="31"/>
+      <c r="E25" s="31"/>
+      <c r="F25" s="31"/>
+      <c r="G25" s="31"/>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B26" s="31"/>
+      <c r="C26" s="31"/>
+      <c r="D26" s="31"/>
+      <c r="E26" s="31"/>
+      <c r="F26" s="31"/>
+      <c r="G26" s="31"/>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B27" s="31"/>
+      <c r="C27" s="31"/>
+      <c r="D27" s="31"/>
+      <c r="E27" s="31"/>
+      <c r="F27" s="31"/>
+      <c r="G27" s="31"/>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="B15:G17"/>
+  <mergeCells count="2">
+    <mergeCell ref="B21:G23"/>
+    <mergeCell ref="B25:G27"/>
   </mergeCells>
-  <conditionalFormatting sqref="B5:F13">
+  <conditionalFormatting sqref="B5:F19">
     <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="3">
       <formula>B5&gt;=0.8</formula>
     </cfRule>
     <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
       <formula>AND(B5&gt;0,B5&lt;0.4)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H5:H19">
+    <cfRule type="expression" priority="4" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="2">
+      <formula>H5="Auto"</formula>
     </cfRule>
   </conditionalFormatting>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -5450,95 +6090,95 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>215</v>
+        <v>246</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="s">
-        <v>216</v>
+        <v>247</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>217</v>
+        <v>248</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>218</v>
+        <v>249</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>219</v>
+        <v>250</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>220</v>
+        <v>251</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>221</v>
+        <v>252</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>222</v>
+        <v>253</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>223</v>
+        <v>254</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>224</v>
+        <v>255</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>225</v>
+        <v>256</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>226</v>
+        <v>257</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>227</v>
+        <v>258</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>228</v>
+        <v>259</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>229</v>
+        <v>260</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>230</v>
+        <v>261</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>158</v>
+        <v>179</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>231</v>
+        <v>262</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>232</v>
+        <v>263</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="8" t="s">
-        <v>233</v>
+        <v>264</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>234</v>
+        <v>265</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>235</v>
+        <v>266</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="8" t="s">
-        <v>236</v>
+        <v>267</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>237</v>
+        <v>268</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>238</v>
+        <v>269</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Apply CRM design corrections
Renewal opp created on closed won; renewal date is the next term's service
start; uplift communicated in one January notice; year-1 uplift always, price
locked from year 2 only when paid upfront; churn category and reason on the
opportunity; CSM edits only line type and new numbers; upsell opens its own
opportunity; evidence-based status guardrails; reports filter by CSM and region;
Priority replaces a typed rank in the CRM.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CVAHSCDuy4tEBaMUUSRsNB
</commit_message>
<xml_diff>
--- a/n8n-renewals-challenge/renewal_tracker.xlsx
+++ b/n8n-renewals-challenge/renewal_tracker.xlsx
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="386" uniqueCount="270">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="403" uniqueCount="278">
   <si>
     <t xml:space="preserve">Renewal tracker: a mock-up of the CRM renewal model</t>
   </si>
@@ -87,7 +87,7 @@
     <t xml:space="preserve">Usage rule</t>
   </si>
   <si>
-    <t xml:space="preserve">Usage +20%: renew as is plus an Upsell line and task (no automatic charge). Usage -20%: flag the CSM; auto-renewals move to At risk.</t>
+    <t xml:space="preserve">Usage +20%: renew as is plus an Upsell opportunity and task (no automatic charge). Usage -20%: flag the CSM; auto-renewals move to At risk.</t>
   </si>
   <si>
     <t xml:space="preserve">Forecast of the forecast</t>
@@ -111,13 +111,13 @@
     <t xml:space="preserve">Products</t>
   </si>
   <si>
-    <t xml:space="preserve">Each line is Renewal / Upsell / Downgrade / Cross-sell / Churn. Original ARR is kept; new ARR adds the 5% uplift to the renewed base, prices changes at list, then applies the discount. Δ is green or red.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Churn type</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Regrettable = revenue lost to n8n for good. Non-regrettable = a line churns but is replaced by another n8n product (e.g. self-hosted Enterprise moving to n8n Cloud), so the revenue is kept.</t>
+    <t xml:space="preserve">The CSM only sets the line type (Renewal / Upsell / Downgrade / Churn) and the new numbers. Original ARR, uplift, list price, new ARR and Δ (green/red) recalculate. Upsell lines open a linked Upsell opportunity.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Churn</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Set on the opportunity: churned amount (from the lines), category (Regrettable = revenue lost for good; Non-regrettable = revenue kept, e.g. self-hosted moving to n8n Cloud) and a granular reason.</t>
   </si>
   <si>
     <t xml:space="preserve">Colour code</t>
@@ -330,7 +330,7 @@
     <t xml:space="preserve">Card expired; billing contact unknown</t>
   </si>
   <si>
-    <t xml:space="preserve">CSM gets the billing contact today; I send a secure card-update link or switch to invoice; Finance holds dunning. Uplift notice date passed, renews flat.</t>
+    <t xml:space="preserve">CSM gets the billing contact today; I send a secure card-update link or switch to invoice; Finance holds dunning. Renews at €27.3k with the contractual 5% uplift.</t>
   </si>
   <si>
     <t xml:space="preserve">Auto-renewal fails in 13 days on an expired card: involuntary churn on a green account.</t>
@@ -411,10 +411,10 @@
     <t xml:space="preserve">Invoice to a different legal entity</t>
   </si>
   <si>
-    <t xml:space="preserve">Uplift notice by 22 Oct. New entity details; Legal: billing change or assignment; Finance updates billing before the invoice run.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Auto-renewal with the wrong billing entity; uplift notice due 22 Oct (assumed 30-day notice).</t>
+    <t xml:space="preserve">New entity details (name, VAT, address); Legal: billing change or assignment; Finance updates billing before the invoice run. Cancellation deadline 22 Oct (assumed 30 days).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Auto-renewal would invoice the wrong legal entity; cancellation deadline 22 Oct (assumed 30-day notice).</t>
   </si>
   <si>
     <t xml:space="preserve">Finance, Legal</t>
@@ -426,7 +426,7 @@
     <t xml:space="preserve">Close to execution cap</t>
   </si>
   <si>
-    <t xml:space="preserve">CSM usage review; two quotes out: like-for-like (€36.75k) and next execution tier. Upsell is upside.</t>
+    <t xml:space="preserve">CSM usage review; quote like-for-like (€36.75k) and open a linked Upsell opportunity for the next execution tier.</t>
   </si>
   <si>
     <t xml:space="preserve">Usage +40%, near the execution cap: expansion, and a throttling risk.</t>
@@ -516,10 +516,10 @@
     <t xml:space="preserve">Uplift from this week's actions</t>
   </si>
   <si>
-    <t xml:space="preserve">Opportunity products: renewal / upsell / downgrade / cross-sell / churn per line</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Original ARR is kept for comparison. Change at list = +upsell / -downgrade. Uplift applies to the renewed base only. Discount is measured against the uplifted list price (a waived uplift counts as discount). Churn or downgrade replaced by another n8n product (e.g. self-hosted to Cloud) is non-regrettable.</t>
+    <t xml:space="preserve">Opportunity products: the CSM only sets the line type and the new numbers; everything else recalculates</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CSM inputs (yellow): line type and change at list. Original ARR comes from the closed renewal. Uplift is automatic: 5% on every renewal line in year 1. On multi-year deals paid upfront the price is locked from year 2 (no further uplift); paid annually, 5% applies every year. An Upsell line opens a linked Upsell opportunity so expansion is forecast separately. Churn category and reason live on the opportunity.</t>
   </si>
   <si>
     <t xml:space="preserve">Opportunity</t>
@@ -534,34 +534,34 @@
     <t xml:space="preserve">Term (yrs)</t>
   </si>
   <si>
+    <t xml:space="preserve">Payment</t>
+  </si>
+  <si>
     <t xml:space="preserve">Original ARR (€)</t>
   </si>
   <si>
     <t xml:space="preserve">Change at list (€)</t>
   </si>
   <si>
-    <t xml:space="preserve">Uplift %</t>
+    <t xml:space="preserve">Uplift % (yr 1)</t>
   </si>
   <si>
     <t xml:space="preserve">Discount %</t>
   </si>
   <si>
+    <t xml:space="preserve">List renewal price (€)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Δ vs original (€)</t>
   </si>
   <si>
     <t xml:space="preserve">Δ %</t>
   </si>
   <si>
-    <t xml:space="preserve">List renewal price (€)</t>
-  </si>
-  <si>
     <t xml:space="preserve">Approval needed</t>
   </si>
   <si>
-    <t xml:space="preserve">Replaced by (n8n product)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Churn (€)</t>
+    <t xml:space="preserve">Year 2+ uplift</t>
   </si>
   <si>
     <t xml:space="preserve">Note</t>
@@ -573,6 +573,9 @@
     <t xml:space="preserve">Renewal</t>
   </si>
   <si>
+    <t xml:space="preserve">Annual</t>
+  </si>
+  <si>
     <t xml:space="preserve">Quote of 1 Sep includes 5% uplift</t>
   </si>
   <si>
@@ -582,7 +585,7 @@
     <t xml:space="preserve">Usage +12%: check cap next quarter</t>
   </si>
   <si>
-    <t xml:space="preserve">Auto-renewal: uplift notice date passed this cycle</t>
+    <t xml:space="preserve">Uplift is contractual (annual notice in January)</t>
   </si>
   <si>
     <t xml:space="preserve">n8n Enterprise (self-hosted)</t>
@@ -597,7 +600,7 @@
     <t xml:space="preserve">n8n Enterprise</t>
   </si>
   <si>
-    <t xml:space="preserve">Floor: 2 years at Finance max 12%</t>
+    <t xml:space="preserve">Placeholder until Part 2 is agreed</t>
   </si>
   <si>
     <t xml:space="preserve">Bill to new legal entity</t>
@@ -612,69 +615,90 @@
     <t xml:space="preserve">Upsell</t>
   </si>
   <si>
-    <t xml:space="preserve">Fill in when the customer picks a tier (upside)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Budget cut: right-sized in line with -20% usage</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Uplift (indexation)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Default 5% on every 1-year renewal line (policy C). On a 2-year term the uplift can be waived inside the 5% multi-year allowance with no approval. Plan names and downgrade prices are assumptions: n8n does not publish self-hosted Enterprise prices.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Opportunity roll-up: calculated from product lines</t>
+    <t xml:space="preserve">Opens a linked Upsell opportunity (upside)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Right-sized in line with -20% usage</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Assumptions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Plan names and downgrade prices are assumptions: n8n does not publish self-hosted Enterprise prices. A year-1 uplift waiver is an exception (e.g. three years paid upfront) and counts as a discount under policy C.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Opportunity roll-up: calculated from product lines; churn category and reason set on the opportunity</t>
   </si>
   <si>
     <t xml:space="preserve">Uplift (€)</t>
   </si>
   <si>
-    <t xml:space="preserve">Upsell / cross-sell (€)</t>
+    <t xml:space="preserve">Upsell (€) → Upsell opp</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Churned amount (€)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Churn category</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Churn reason</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Price concession below current (€)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Net change (€)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Net change %</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Regrettable</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Low adoption / champion left</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Budget cut</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(linked to Pipeline)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Churn reasons</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Regrettable: Budget cut · Regrettable: Price · Regrettable: Competitor · Regrettable: Moved to free Community edition · Regrettable: Product gaps · Regrettable: Support or service · Regrettable: Low adoption / champion left · Regrettable: Company closed · Non-regrettable: Migrated to another n8n product · Non-regrettable: Consolidated into another n8n contract · Non-regrettable: Moved to another legal entity</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Missing reason</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Check: new ARR ties to Pipeline</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Renewals by quarter and month (by renewal date)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"># renewals</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Weighted (€)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">On time, weighted (€)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Late, weighted (€)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Overdue ARR (€)</t>
   </si>
   <si>
     <t xml:space="preserve">Regrettable churn (€)</t>
   </si>
   <si>
-    <t xml:space="preserve">Non-regrettable churn (€)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Replacement revenue (€)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Price concession below current (€)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Net change (€)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Net change %</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(linked to Pipeline)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Check: new ARR ties to Pipeline</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Renewals by quarter and month (by renewal date)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"># renewals</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Weighted (€)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">On time, weighted (€)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Late, weighted (€)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Overdue ARR (€)</t>
-  </si>
-  <si>
     <t xml:space="preserve">Q4 2026</t>
   </si>
   <si>
@@ -786,7 +810,7 @@
     <t xml:space="preserve">Overdue renewals use the Overdue column and are shown as Late. They still count in the quarter's forecast only if the expected close date is on or before quarter end. If they slip past quarter end they count 0% for that quarter and come back next quarter as a late renewal.</t>
   </si>
   <si>
-    <t xml:space="preserve">n8n prices by workflow executions (users are unlimited). Usage +20% or more: renew as is, add an Upsell line and a CSM + Renewals task; never auto-charge unless the contract has an overage clause. Usage -20% or more: flag the CSM for an adoption plan; on an auto-renewal, set At risk.</t>
+    <t xml:space="preserve">n8n prices by workflow executions (users are unlimited). Usage +20% or more: renew as is, open an Upsell opportunity and a CSM + Renewals task; never auto-charge unless the contract has an overage clause. Usage -20% or more: flag the CSM for an adoption plan; on an auto-renewal, set At risk.</t>
   </si>
   <si>
     <t xml:space="preserve">Commercial policy (section C) and the approval it triggers</t>
@@ -1821,7 +1845,7 @@
       </c>
       <c r="H7" s="8" t="str">
         <f aca="false">INDEX(Pipeline!$V$5:$V$14,MATCH($A7,Pipeline!$Y$5:$Y$14,0))&amp;""</f>
-        <v>CSM gets the billing contact today; I send a secure card-update link or switch to invoice; Finance holds dunning. Uplift notice date passed, renews flat.</v>
+        <v>CSM gets the billing contact today; I send a secure card-update link or switch to invoice; Finance holds dunning. Renews at €27.3k with the contractual 5% uplift.</v>
       </c>
       <c r="I7" s="8" t="str">
         <f aca="false">INDEX(Pipeline!$W$5:$W$14,MATCH($A7,Pipeline!$Y$5:$Y$14,0))</f>
@@ -2066,7 +2090,7 @@
       </c>
       <c r="H12" s="8" t="str">
         <f aca="false">INDEX(Pipeline!$V$5:$V$14,MATCH($A12,Pipeline!$Y$5:$Y$14,0))&amp;""</f>
-        <v>CSM usage review; two quotes out: like-for-like (€36.75k) and next execution tier. Upsell is upside.</v>
+        <v>CSM usage review; quote like-for-like (€36.75k) and open a linked Upsell opportunity for the next execution tier.</v>
       </c>
       <c r="I12" s="8" t="str">
         <f aca="false">INDEX(Pipeline!$W$5:$W$14,MATCH($A12,Pipeline!$Y$5:$Y$14,0))</f>
@@ -2111,11 +2135,11 @@
       </c>
       <c r="G13" s="8" t="str">
         <f aca="false">INDEX(Pipeline!$Z$5:$Z$14,MATCH($A13,Pipeline!$Y$5:$Y$14,0))&amp;""</f>
-        <v>Auto-renewal with the wrong billing entity; uplift notice due 22 Oct (assumed 30-day notice).</v>
+        <v>Auto-renewal would invoice the wrong legal entity; cancellation deadline 22 Oct (assumed 30-day notice).</v>
       </c>
       <c r="H13" s="8" t="str">
         <f aca="false">INDEX(Pipeline!$V$5:$V$14,MATCH($A13,Pipeline!$Y$5:$Y$14,0))&amp;""</f>
-        <v>Uplift notice by 22 Oct. New entity details; Legal: billing change or assignment; Finance updates billing before the invoice run.</v>
+        <v>New entity details (name, VAT, address); Legal: billing change or assignment; Finance updates billing before the invoice run. Cancellation deadline 22 Oct (assumed 30 days).</v>
       </c>
       <c r="I13" s="8" t="str">
         <f aca="false">INDEX(Pipeline!$W$5:$W$14,MATCH($A13,Pipeline!$Y$5:$Y$14,0))</f>
@@ -2466,7 +2490,7 @@
         <v>0.5</v>
       </c>
       <c r="S5" s="23" t="n">
-        <f aca="false">SUMIFS(Products!$I:$I,Products!$A:$A,A5)</f>
+        <f aca="false">SUMIFS(Products!$K:$K,Products!$A:$A,A5)</f>
         <v>22050</v>
       </c>
       <c r="T5" s="23" t="n">
@@ -2504,7 +2528,7 @@
         <v/>
       </c>
       <c r="AE5" s="8" t="str">
-        <f aca="false">IF(E5&gt;=0.2,"Over-usage: upsell line + CSM/Renewals task",IF(E5&lt;=-0.2,"Under-usage: flag CSM"&amp;IF(D5="Auto","; set At risk",""),""))</f>
+        <f aca="false">IF(E5&gt;=0.2,"Over-usage: open Upsell opp + CSM/Renewals task",IF(E5&lt;=-0.2,"Under-usage: flag CSM"&amp;IF(D5="Auto","; set At risk",""),""))</f>
         <v/>
       </c>
       <c r="AF5" s="20" t="s">
@@ -2584,7 +2608,7 @@
         <v>0.25</v>
       </c>
       <c r="S6" s="23" t="n">
-        <f aca="false">SUMIFS(Products!$I:$I,Products!$A:$A,A6)</f>
+        <f aca="false">SUMIFS(Products!$K:$K,Products!$A:$A,A6)</f>
         <v>50400</v>
       </c>
       <c r="T6" s="23" t="n">
@@ -2620,7 +2644,7 @@
         <v/>
       </c>
       <c r="AE6" s="8" t="str">
-        <f aca="false">IF(E6&gt;=0.2,"Over-usage: upsell line + CSM/Renewals task",IF(E6&lt;=-0.2,"Under-usage: flag CSM"&amp;IF(D6="Auto","; set At risk",""),""))</f>
+        <f aca="false">IF(E6&gt;=0.2,"Over-usage: open Upsell opp + CSM/Renewals task",IF(E6&lt;=-0.2,"Under-usage: flag CSM"&amp;IF(D6="Auto","; set At risk",""),""))</f>
         <v/>
       </c>
       <c r="AF6" s="20" t="s">
@@ -2700,12 +2724,12 @@
         <v>0.6</v>
       </c>
       <c r="S7" s="23" t="n">
-        <f aca="false">SUMIFS(Products!$I:$I,Products!$A:$A,A7)</f>
-        <v>26000</v>
+        <f aca="false">SUMIFS(Products!$K:$K,Products!$A:$A,A7)</f>
+        <v>27300</v>
       </c>
       <c r="T7" s="23" t="n">
         <f aca="false">S7*R7</f>
-        <v>15600</v>
+        <v>16380</v>
       </c>
       <c r="U7" s="15" t="str">
         <f aca="false">IF(G7="Cancelled","Lost",IF(Q7="No","Slips quarter",IF(OR(J7&lt;0,AND(J7&lt;=30,OR(G7="--None--",G7="Not started",G7="Engaging customer",G7="Negotiation",G7="Billing blocker",G7="At risk: before notice deadline",G7="Notice received"))),"Late","On time")))</f>
@@ -2738,7 +2762,7 @@
         <v>46298</v>
       </c>
       <c r="AE7" s="8" t="str">
-        <f aca="false">IF(E7&gt;=0.2,"Over-usage: upsell line + CSM/Renewals task",IF(E7&lt;=-0.2,"Under-usage: flag CSM"&amp;IF(D7="Auto","; set At risk",""),""))</f>
+        <f aca="false">IF(E7&gt;=0.2,"Over-usage: open Upsell opp + CSM/Renewals task",IF(E7&lt;=-0.2,"Under-usage: flag CSM"&amp;IF(D7="Auto","; set At risk",""),""))</f>
         <v/>
       </c>
       <c r="AF7" s="20" t="s">
@@ -2750,7 +2774,7 @@
       </c>
       <c r="AH7" s="23" t="n">
         <f aca="false">S7*AG7</f>
-        <v>25220</v>
+        <v>26481</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2818,7 +2842,7 @@
         <v>0.1</v>
       </c>
       <c r="S8" s="23" t="n">
-        <f aca="false">SUMIFS(Products!$I:$I,Products!$A:$A,A8)</f>
+        <f aca="false">SUMIFS(Products!$K:$K,Products!$A:$A,A8)</f>
         <v>30000</v>
       </c>
       <c r="T8" s="23" t="n">
@@ -2858,7 +2882,7 @@
         <v>46303</v>
       </c>
       <c r="AE8" s="8" t="str">
-        <f aca="false">IF(E8&gt;=0.2,"Over-usage: upsell line + CSM/Renewals task",IF(E8&lt;=-0.2,"Under-usage: flag CSM"&amp;IF(D8="Auto","; set At risk",""),""))</f>
+        <f aca="false">IF(E8&gt;=0.2,"Over-usage: open Upsell opp + CSM/Renewals task",IF(E8&lt;=-0.2,"Under-usage: flag CSM"&amp;IF(D8="Auto","; set At risk",""),""))</f>
         <v>Under-usage: flag CSM</v>
       </c>
       <c r="AF8" s="20" t="s">
@@ -2938,7 +2962,7 @@
         <v>0.5</v>
       </c>
       <c r="S9" s="23" t="n">
-        <f aca="false">SUMIFS(Products!$I:$I,Products!$A:$A,A9)</f>
+        <f aca="false">SUMIFS(Products!$K:$K,Products!$A:$A,A9)</f>
         <v>33264</v>
       </c>
       <c r="T9" s="23" t="n">
@@ -2974,7 +2998,7 @@
         <v/>
       </c>
       <c r="AE9" s="8" t="str">
-        <f aca="false">IF(E9&gt;=0.2,"Over-usage: upsell line + CSM/Renewals task",IF(E9&lt;=-0.2,"Under-usage: flag CSM"&amp;IF(D9="Auto","; set At risk",""),""))</f>
+        <f aca="false">IF(E9&gt;=0.2,"Over-usage: open Upsell opp + CSM/Renewals task",IF(E9&lt;=-0.2,"Under-usage: flag CSM"&amp;IF(D9="Auto","; set At risk",""),""))</f>
         <v/>
       </c>
       <c r="AF9" s="20" t="s">
@@ -3054,7 +3078,7 @@
         <v>0.4</v>
       </c>
       <c r="S10" s="23" t="n">
-        <f aca="false">SUMIFS(Products!$I:$I,Products!$A:$A,A10)</f>
+        <f aca="false">SUMIFS(Products!$K:$K,Products!$A:$A,A10)</f>
         <v>52500</v>
       </c>
       <c r="T10" s="23" t="n">
@@ -3092,7 +3116,7 @@
         <v/>
       </c>
       <c r="AE10" s="8" t="str">
-        <f aca="false">IF(E10&gt;=0.2,"Over-usage: upsell line + CSM/Renewals task",IF(E10&lt;=-0.2,"Under-usage: flag CSM"&amp;IF(D10="Auto","; set At risk",""),""))</f>
+        <f aca="false">IF(E10&gt;=0.2,"Over-usage: open Upsell opp + CSM/Renewals task",IF(E10&lt;=-0.2,"Under-usage: flag CSM"&amp;IF(D10="Auto","; set At risk",""),""))</f>
         <v/>
       </c>
       <c r="AF10" s="20" t="s">
@@ -3172,7 +3196,7 @@
         <v>0.7</v>
       </c>
       <c r="S11" s="23" t="n">
-        <f aca="false">SUMIFS(Products!$I:$I,Products!$A:$A,A11)</f>
+        <f aca="false">SUMIFS(Products!$K:$K,Products!$A:$A,A11)</f>
         <v>29400</v>
       </c>
       <c r="T11" s="23" t="n">
@@ -3210,7 +3234,7 @@
         <v>46317</v>
       </c>
       <c r="AE11" s="8" t="str">
-        <f aca="false">IF(E11&gt;=0.2,"Over-usage: upsell line + CSM/Renewals task",IF(E11&lt;=-0.2,"Under-usage: flag CSM"&amp;IF(D11="Auto","; set At risk",""),""))</f>
+        <f aca="false">IF(E11&gt;=0.2,"Over-usage: open Upsell opp + CSM/Renewals task",IF(E11&lt;=-0.2,"Under-usage: flag CSM"&amp;IF(D11="Auto","; set At risk",""),""))</f>
         <v/>
       </c>
       <c r="AF11" s="20" t="s">
@@ -3290,7 +3314,7 @@
         <v>0.2</v>
       </c>
       <c r="S12" s="23" t="n">
-        <f aca="false">SUMIFS(Products!$I:$I,Products!$A:$A,A12)</f>
+        <f aca="false">SUMIFS(Products!$K:$K,Products!$A:$A,A12)</f>
         <v>36750</v>
       </c>
       <c r="T12" s="23" t="n">
@@ -3326,8 +3350,8 @@
         <v/>
       </c>
       <c r="AE12" s="8" t="str">
-        <f aca="false">IF(E12&gt;=0.2,"Over-usage: upsell line + CSM/Renewals task",IF(E12&lt;=-0.2,"Under-usage: flag CSM"&amp;IF(D12="Auto","; set At risk",""),""))</f>
-        <v>Over-usage: upsell line + CSM/Renewals task</v>
+        <f aca="false">IF(E12&gt;=0.2,"Over-usage: open Upsell opp + CSM/Renewals task",IF(E12&lt;=-0.2,"Under-usage: flag CSM"&amp;IF(D12="Auto","; set At risk",""),""))</f>
+        <v>Over-usage: open Upsell opp + CSM/Renewals task</v>
       </c>
       <c r="AF12" s="20" t="s">
         <v>73</v>
@@ -3406,7 +3430,7 @@
         <v>0.35</v>
       </c>
       <c r="S13" s="23" t="n">
-        <f aca="false">SUMIFS(Products!$I:$I,Products!$A:$A,A13)</f>
+        <f aca="false">SUMIFS(Products!$K:$K,Products!$A:$A,A13)</f>
         <v>48300</v>
       </c>
       <c r="T13" s="23" t="n">
@@ -3442,7 +3466,7 @@
         <v/>
       </c>
       <c r="AE13" s="8" t="str">
-        <f aca="false">IF(E13&gt;=0.2,"Over-usage: upsell line + CSM/Renewals task",IF(E13&lt;=-0.2,"Under-usage: flag CSM"&amp;IF(D13="Auto","; set At risk",""),""))</f>
+        <f aca="false">IF(E13&gt;=0.2,"Over-usage: open Upsell opp + CSM/Renewals task",IF(E13&lt;=-0.2,"Under-usage: flag CSM"&amp;IF(D13="Auto","; set At risk",""),""))</f>
         <v/>
       </c>
       <c r="AF13" s="20" t="s">
@@ -3522,7 +3546,7 @@
         <v>0.4</v>
       </c>
       <c r="S14" s="23" t="n">
-        <f aca="false">SUMIFS(Products!$I:$I,Products!$A:$A,A14)</f>
+        <f aca="false">SUMIFS(Products!$K:$K,Products!$A:$A,A14)</f>
         <v>32000</v>
       </c>
       <c r="T14" s="23" t="n">
@@ -3560,7 +3584,7 @@
         <v>46345</v>
       </c>
       <c r="AE14" s="8" t="str">
-        <f aca="false">IF(E14&gt;=0.2,"Over-usage: upsell line + CSM/Renewals task",IF(E14&lt;=-0.2,"Under-usage: flag CSM"&amp;IF(D14="Auto","; set At risk",""),""))</f>
+        <f aca="false">IF(E14&gt;=0.2,"Over-usage: open Upsell opp + CSM/Renewals task",IF(E14&lt;=-0.2,"Under-usage: flag CSM"&amp;IF(D14="Auto","; set At risk",""),""))</f>
         <v>Under-usage: flag CSM; set At risk</v>
       </c>
       <c r="AF14" s="20" t="s">
@@ -3585,15 +3609,15 @@
       </c>
       <c r="S15" s="24" t="n">
         <f aca="false">SUM(S5:S14)</f>
-        <v>360664</v>
+        <v>361964</v>
       </c>
       <c r="T15" s="24" t="n">
         <f aca="false">SUM(T5:T14)</f>
-        <v>137492</v>
+        <v>138272</v>
       </c>
       <c r="AH15" s="24" t="n">
         <f aca="false">SUM(AH5:AH14)</f>
-        <v>254732.5</v>
+        <v>255993.5</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3638,11 +3662,11 @@
       </c>
       <c r="B21" s="23" t="n">
         <f aca="false">SUMIFS(T5:T14,U5:U14,"Late")</f>
-        <v>63225</v>
+        <v>64005</v>
       </c>
       <c r="C21" s="23" t="n">
         <f aca="false">SUMIFS(S5:S14,U5:U14,"Late")</f>
-        <v>180950</v>
+        <v>182250</v>
       </c>
       <c r="D21" s="15" t="str">
         <f aca="false">COUNTIFS(U5:U14,"Late")&amp;" renewals"</f>
@@ -3672,11 +3696,11 @@
       </c>
       <c r="B23" s="27" t="n">
         <f aca="false">SUM(B20:B22)</f>
-        <v>137492</v>
+        <v>138272</v>
       </c>
       <c r="C23" s="23" t="n">
         <f aca="false">SUM(C20:C22)</f>
-        <v>360664</v>
+        <v>361964</v>
       </c>
       <c r="D23" s="28"/>
     </row>
@@ -3727,7 +3751,7 @@
       </c>
       <c r="B29" s="30" t="n">
         <f aca="false">S15/B15</f>
-        <v>0.961770666666667</v>
+        <v>0.965237333333333</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3741,7 +3765,7 @@
       </c>
       <c r="B32" s="27" t="n">
         <f aca="false">T15</f>
-        <v>137492</v>
+        <v>138272</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3750,7 +3774,7 @@
       </c>
       <c r="B33" s="27" t="n">
         <f aca="false">AH15</f>
-        <v>254732.5</v>
+        <v>255993.5</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3759,7 +3783,7 @@
       </c>
       <c r="B34" s="27" t="n">
         <f aca="false">B33-B32</f>
-        <v>117240.5</v>
+        <v>117721.5</v>
       </c>
     </row>
   </sheetData>
@@ -3871,23 +3895,22 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:Q20"/>
+  <dimension ref="A1:P20"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="20"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="28"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="9" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="13" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="0" width="44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="8" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="11" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="44"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3895,7 +3918,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="31" t="s">
         <v>156</v>
       </c>
@@ -3912,9 +3935,6 @@
       <c r="L2" s="31"/>
       <c r="M2" s="31"/>
       <c r="N2" s="31"/>
-      <c r="O2" s="31"/>
-      <c r="P2" s="31"/>
-      <c r="Q2" s="31"/>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
@@ -3942,13 +3962,13 @@
         <v>164</v>
       </c>
       <c r="I4" s="6" t="s">
+        <v>165</v>
+      </c>
+      <c r="J4" s="6" t="s">
+        <v>166</v>
+      </c>
+      <c r="K4" s="6" t="s">
         <v>61</v>
-      </c>
-      <c r="J4" s="6" t="s">
-        <v>165</v>
-      </c>
-      <c r="K4" s="6" t="s">
-        <v>166</v>
       </c>
       <c r="L4" s="6" t="s">
         <v>167</v>
@@ -3960,12 +3980,9 @@
         <v>169</v>
       </c>
       <c r="O4" s="6" t="s">
-        <v>21</v>
+        <v>170</v>
       </c>
       <c r="P4" s="6" t="s">
-        <v>170</v>
-      </c>
-      <c r="Q4" s="6" t="s">
         <v>171</v>
       </c>
     </row>
@@ -3982,49 +3999,48 @@
       <c r="D5" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="E5" s="16" t="n">
+      <c r="E5" s="18" t="s">
+        <v>174</v>
+      </c>
+      <c r="F5" s="23" t="n">
         <v>21000</v>
       </c>
-      <c r="F5" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="G5" s="19" t="n">
+      <c r="G5" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" s="22" t="n">
+        <f aca="false">IF(C5="Renewal",0.05,0)</f>
         <v>0.05</v>
       </c>
-      <c r="H5" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="I5" s="23" t="n">
-        <f aca="false">L5*(1-H5)</f>
+      <c r="I5" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" s="23" t="n">
+        <f aca="false">IF(C5="Churn",0,F5*(1+H5)+G5)</f>
         <v>22050</v>
       </c>
-      <c r="J5" s="23" t="n">
-        <f aca="false">I5-E5</f>
+      <c r="K5" s="23" t="n">
+        <f aca="false">J5*(1-I5)</f>
+        <v>22050</v>
+      </c>
+      <c r="L5" s="23" t="n">
+        <f aca="false">K5-F5</f>
         <v>1050</v>
       </c>
-      <c r="K5" s="22" t="n">
-        <f aca="false">IF(E5=0,"new",J5/E5)</f>
+      <c r="M5" s="22" t="n">
+        <f aca="false">IF(F5=0,"new",L5/F5)</f>
         <v>0.05</v>
       </c>
-      <c r="L5" s="23" t="n">
-        <f aca="false">IF(C5="Churn",0,E5*(1+G5)+F5)</f>
-        <v>22050</v>
-      </c>
-      <c r="M5" s="15" t="str">
-        <f aca="false">IF(H5=0,IF(AND(G5=0,C5="Renewal",D5=1),"Finance (uplift waived)","None"),IF(AND(D5&gt;=2,H5&lt;=0.05),"None (multi-year)",IF(H5&lt;=0.12,"Finance","VP Customer Success")))</f>
+      <c r="N5" s="15" t="str">
+        <f aca="false">IF(I5=0,"None",IF(AND(D5&gt;=2,I5&lt;=0.05),"None (multi-year)",IF(I5&lt;=0.12,"Finance","VP Customer Success")))</f>
         <v>None</v>
       </c>
-      <c r="N5" s="18"/>
       <c r="O5" s="15" t="str">
-        <f aca="false">IF(OR(C5="Churn",C5="Downgrade"),IF(N5&lt;&gt;"","Non-regrettable","Regrettable"),"")</f>
-        <v/>
-      </c>
-      <c r="P5" s="23" t="n">
-        <f aca="false">IF(C5="Churn",-E5,IF(C5="Downgrade",F5,0))</f>
-        <v>0</v>
-      </c>
-      <c r="Q5" s="15" t="s">
-        <v>174</v>
+        <f aca="false">IF(D5&lt;2,"n/a",IF(E5="Upfront","Locked (0%)","5% a year"))</f>
+        <v>n/a</v>
+      </c>
+      <c r="P5" s="15" t="s">
+        <v>175</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4032,7 +4048,7 @@
         <v>81</v>
       </c>
       <c r="B6" s="15" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="C6" s="18" t="s">
         <v>173</v>
@@ -4040,49 +4056,48 @@
       <c r="D6" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="E6" s="16" t="n">
+      <c r="E6" s="18" t="s">
+        <v>174</v>
+      </c>
+      <c r="F6" s="23" t="n">
         <v>48000</v>
       </c>
-      <c r="F6" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="G6" s="19" t="n">
+      <c r="G6" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="22" t="n">
+        <f aca="false">IF(C6="Renewal",0.05,0)</f>
         <v>0.05</v>
       </c>
-      <c r="H6" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="I6" s="23" t="n">
-        <f aca="false">L6*(1-H6)</f>
+      <c r="I6" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" s="23" t="n">
+        <f aca="false">IF(C6="Churn",0,F6*(1+H6)+G6)</f>
         <v>50400</v>
       </c>
-      <c r="J6" s="23" t="n">
-        <f aca="false">I6-E6</f>
+      <c r="K6" s="23" t="n">
+        <f aca="false">J6*(1-I6)</f>
+        <v>50400</v>
+      </c>
+      <c r="L6" s="23" t="n">
+        <f aca="false">K6-F6</f>
         <v>2400</v>
       </c>
-      <c r="K6" s="22" t="n">
-        <f aca="false">IF(E6=0,"new",J6/E6)</f>
+      <c r="M6" s="22" t="n">
+        <f aca="false">IF(F6=0,"new",L6/F6)</f>
         <v>0.05</v>
       </c>
-      <c r="L6" s="23" t="n">
-        <f aca="false">IF(C6="Churn",0,E6*(1+G6)+F6)</f>
-        <v>50400</v>
-      </c>
-      <c r="M6" s="15" t="str">
-        <f aca="false">IF(H6=0,IF(AND(G6=0,C6="Renewal",D6=1),"Finance (uplift waived)","None"),IF(AND(D6&gt;=2,H6&lt;=0.05),"None (multi-year)",IF(H6&lt;=0.12,"Finance","VP Customer Success")))</f>
+      <c r="N6" s="15" t="str">
+        <f aca="false">IF(I6=0,"None",IF(AND(D6&gt;=2,I6&lt;=0.05),"None (multi-year)",IF(I6&lt;=0.12,"Finance","VP Customer Success")))</f>
         <v>None</v>
       </c>
-      <c r="N6" s="18"/>
       <c r="O6" s="15" t="str">
-        <f aca="false">IF(OR(C6="Churn",C6="Downgrade"),IF(N6&lt;&gt;"","Non-regrettable","Regrettable"),"")</f>
-        <v/>
-      </c>
-      <c r="P6" s="23" t="n">
-        <f aca="false">IF(C6="Churn",-E6,IF(C6="Downgrade",F6,0))</f>
-        <v>0</v>
-      </c>
-      <c r="Q6" s="15" t="s">
-        <v>176</v>
+        <f aca="false">IF(D6&lt;2,"n/a",IF(E6="Upfront","Locked (0%)","5% a year"))</f>
+        <v>n/a</v>
+      </c>
+      <c r="P6" s="15" t="s">
+        <v>177</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4098,49 +4113,48 @@
       <c r="D7" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="E7" s="16" t="n">
+      <c r="E7" s="18" t="s">
+        <v>174</v>
+      </c>
+      <c r="F7" s="23" t="n">
         <v>26000</v>
       </c>
-      <c r="F7" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="G7" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="H7" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="I7" s="23" t="n">
-        <f aca="false">L7*(1-H7)</f>
-        <v>26000</v>
+      <c r="G7" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" s="22" t="n">
+        <f aca="false">IF(C7="Renewal",0.05,0)</f>
+        <v>0.05</v>
+      </c>
+      <c r="I7" s="19" t="n">
+        <v>0</v>
       </c>
       <c r="J7" s="23" t="n">
-        <f aca="false">I7-E7</f>
-        <v>0</v>
-      </c>
-      <c r="K7" s="22" t="n">
-        <f aca="false">IF(E7=0,"new",J7/E7)</f>
-        <v>0</v>
+        <f aca="false">IF(C7="Churn",0,F7*(1+H7)+G7)</f>
+        <v>27300</v>
+      </c>
+      <c r="K7" s="23" t="n">
+        <f aca="false">J7*(1-I7)</f>
+        <v>27300</v>
       </c>
       <c r="L7" s="23" t="n">
-        <f aca="false">IF(C7="Churn",0,E7*(1+G7)+F7)</f>
-        <v>26000</v>
-      </c>
-      <c r="M7" s="15" t="str">
-        <f aca="false">IF(H7=0,IF(AND(G7=0,C7="Renewal",D7=1),"Finance (uplift waived)","None"),IF(AND(D7&gt;=2,H7&lt;=0.05),"None (multi-year)",IF(H7&lt;=0.12,"Finance","VP Customer Success")))</f>
-        <v>Finance (uplift waived)</v>
-      </c>
-      <c r="N7" s="18"/>
+        <f aca="false">K7-F7</f>
+        <v>1300</v>
+      </c>
+      <c r="M7" s="22" t="n">
+        <f aca="false">IF(F7=0,"new",L7/F7)</f>
+        <v>0.05</v>
+      </c>
+      <c r="N7" s="15" t="str">
+        <f aca="false">IF(I7=0,"None",IF(AND(D7&gt;=2,I7&lt;=0.05),"None (multi-year)",IF(I7&lt;=0.12,"Finance","VP Customer Success")))</f>
+        <v>None</v>
+      </c>
       <c r="O7" s="15" t="str">
-        <f aca="false">IF(OR(C7="Churn",C7="Downgrade"),IF(N7&lt;&gt;"","Non-regrettable","Regrettable"),"")</f>
-        <v/>
-      </c>
-      <c r="P7" s="23" t="n">
-        <f aca="false">IF(C7="Churn",-E7,IF(C7="Downgrade",F7,0))</f>
-        <v>0</v>
-      </c>
-      <c r="Q7" s="15" t="s">
-        <v>177</v>
+        <f aca="false">IF(D7&lt;2,"n/a",IF(E7="Upfront","Locked (0%)","5% a year"))</f>
+        <v>n/a</v>
+      </c>
+      <c r="P7" s="15" t="s">
+        <v>178</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4148,57 +4162,56 @@
         <v>97</v>
       </c>
       <c r="B8" s="15" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="C8" s="18" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="D8" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="E8" s="16" t="n">
+      <c r="E8" s="18" t="s">
+        <v>174</v>
+      </c>
+      <c r="F8" s="23" t="n">
         <v>45000</v>
       </c>
-      <c r="F8" s="16" t="n">
+      <c r="G8" s="16" t="n">
         <v>-15000</v>
       </c>
-      <c r="G8" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="H8" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="I8" s="23" t="n">
-        <f aca="false">L8*(1-H8)</f>
+      <c r="H8" s="22" t="n">
+        <f aca="false">IF(C8="Renewal",0.05,0)</f>
+        <v>0</v>
+      </c>
+      <c r="I8" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" s="23" t="n">
+        <f aca="false">IF(C8="Churn",0,F8*(1+H8)+G8)</f>
         <v>30000</v>
       </c>
-      <c r="J8" s="23" t="n">
-        <f aca="false">I8-E8</f>
+      <c r="K8" s="23" t="n">
+        <f aca="false">J8*(1-I8)</f>
+        <v>30000</v>
+      </c>
+      <c r="L8" s="23" t="n">
+        <f aca="false">K8-F8</f>
         <v>-15000</v>
       </c>
-      <c r="K8" s="22" t="n">
-        <f aca="false">IF(E8=0,"new",J8/E8)</f>
+      <c r="M8" s="22" t="n">
+        <f aca="false">IF(F8=0,"new",L8/F8)</f>
         <v>-0.333333333333333</v>
       </c>
-      <c r="L8" s="23" t="n">
-        <f aca="false">IF(C8="Churn",0,E8*(1+G8)+F8)</f>
-        <v>30000</v>
-      </c>
-      <c r="M8" s="15" t="str">
-        <f aca="false">IF(H8=0,IF(AND(G8=0,C8="Renewal",D8=1),"Finance (uplift waived)","None"),IF(AND(D8&gt;=2,H8&lt;=0.05),"None (multi-year)",IF(H8&lt;=0.12,"Finance","VP Customer Success")))</f>
+      <c r="N8" s="15" t="str">
+        <f aca="false">IF(I8=0,"None",IF(AND(D8&gt;=2,I8&lt;=0.05),"None (multi-year)",IF(I8&lt;=0.12,"Finance","VP Customer Success")))</f>
         <v>None</v>
       </c>
-      <c r="N8" s="18"/>
       <c r="O8" s="15" t="str">
-        <f aca="false">IF(OR(C8="Churn",C8="Downgrade"),IF(N8&lt;&gt;"","Non-regrettable","Regrettable"),"")</f>
-        <v>Regrettable</v>
-      </c>
-      <c r="P8" s="23" t="n">
-        <f aca="false">IF(C8="Churn",-E8,IF(C8="Downgrade",F8,0))</f>
-        <v>-15000</v>
-      </c>
-      <c r="Q8" s="15" t="s">
-        <v>180</v>
+        <f aca="false">IF(D8&lt;2,"n/a",IF(E8="Upfront","Locked (0%)","5% a year"))</f>
+        <v>n/a</v>
+      </c>
+      <c r="P8" s="15" t="s">
+        <v>181</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4206,7 +4219,7 @@
         <v>105</v>
       </c>
       <c r="B9" s="15" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="C9" s="18" t="s">
         <v>173</v>
@@ -4214,49 +4227,48 @@
       <c r="D9" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="E9" s="16" t="n">
+      <c r="E9" s="18" t="s">
+        <v>174</v>
+      </c>
+      <c r="F9" s="23" t="n">
         <v>36000</v>
       </c>
-      <c r="F9" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="G9" s="19" t="n">
+      <c r="G9" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" s="22" t="n">
+        <f aca="false">IF(C9="Renewal",0.05,0)</f>
         <v>0.05</v>
       </c>
-      <c r="H9" s="19" t="n">
+      <c r="I9" s="19" t="n">
         <v>0.12</v>
       </c>
-      <c r="I9" s="23" t="n">
-        <f aca="false">L9*(1-H9)</f>
+      <c r="J9" s="23" t="n">
+        <f aca="false">IF(C9="Churn",0,F9*(1+H9)+G9)</f>
+        <v>37800</v>
+      </c>
+      <c r="K9" s="23" t="n">
+        <f aca="false">J9*(1-I9)</f>
         <v>33264</v>
       </c>
-      <c r="J9" s="23" t="n">
-        <f aca="false">I9-E9</f>
+      <c r="L9" s="23" t="n">
+        <f aca="false">K9-F9</f>
         <v>-2736</v>
       </c>
-      <c r="K9" s="22" t="n">
-        <f aca="false">IF(E9=0,"new",J9/E9)</f>
+      <c r="M9" s="22" t="n">
+        <f aca="false">IF(F9=0,"new",L9/F9)</f>
         <v>-0.076</v>
       </c>
-      <c r="L9" s="23" t="n">
-        <f aca="false">IF(C9="Churn",0,E9*(1+G9)+F9)</f>
-        <v>37800</v>
-      </c>
-      <c r="M9" s="15" t="str">
-        <f aca="false">IF(H9=0,IF(AND(G9=0,C9="Renewal",D9=1),"Finance (uplift waived)","None"),IF(AND(D9&gt;=2,H9&lt;=0.05),"None (multi-year)",IF(H9&lt;=0.12,"Finance","VP Customer Success")))</f>
+      <c r="N9" s="15" t="str">
+        <f aca="false">IF(I9=0,"None",IF(AND(D9&gt;=2,I9&lt;=0.05),"None (multi-year)",IF(I9&lt;=0.12,"Finance","VP Customer Success")))</f>
         <v>Finance</v>
       </c>
-      <c r="N9" s="18"/>
       <c r="O9" s="15" t="str">
-        <f aca="false">IF(OR(C9="Churn",C9="Downgrade"),IF(N9&lt;&gt;"","Non-regrettable","Regrettable"),"")</f>
-        <v/>
-      </c>
-      <c r="P9" s="23" t="n">
-        <f aca="false">IF(C9="Churn",-E9,IF(C9="Downgrade",F9,0))</f>
-        <v>0</v>
-      </c>
-      <c r="Q9" s="15" t="s">
-        <v>182</v>
+        <f aca="false">IF(D9&lt;2,"n/a",IF(E9="Upfront","Locked (0%)","5% a year"))</f>
+        <v>5% a year</v>
+      </c>
+      <c r="P9" s="15" t="s">
+        <v>183</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4264,7 +4276,7 @@
         <v>111</v>
       </c>
       <c r="B10" s="15" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="C10" s="18" t="s">
         <v>173</v>
@@ -4272,48 +4284,47 @@
       <c r="D10" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="E10" s="16" t="n">
+      <c r="E10" s="18" t="s">
+        <v>174</v>
+      </c>
+      <c r="F10" s="23" t="n">
         <v>50000</v>
       </c>
-      <c r="F10" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="G10" s="19" t="n">
+      <c r="G10" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" s="22" t="n">
+        <f aca="false">IF(C10="Renewal",0.05,0)</f>
         <v>0.05</v>
       </c>
-      <c r="H10" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="I10" s="23" t="n">
-        <f aca="false">L10*(1-H10)</f>
+      <c r="I10" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="J10" s="23" t="n">
+        <f aca="false">IF(C10="Churn",0,F10*(1+H10)+G10)</f>
         <v>52500</v>
       </c>
-      <c r="J10" s="23" t="n">
-        <f aca="false">I10-E10</f>
+      <c r="K10" s="23" t="n">
+        <f aca="false">J10*(1-I10)</f>
+        <v>52500</v>
+      </c>
+      <c r="L10" s="23" t="n">
+        <f aca="false">K10-F10</f>
         <v>2500</v>
       </c>
-      <c r="K10" s="22" t="n">
-        <f aca="false">IF(E10=0,"new",J10/E10)</f>
+      <c r="M10" s="22" t="n">
+        <f aca="false">IF(F10=0,"new",L10/F10)</f>
         <v>0.05</v>
       </c>
-      <c r="L10" s="23" t="n">
-        <f aca="false">IF(C10="Churn",0,E10*(1+G10)+F10)</f>
-        <v>52500</v>
-      </c>
-      <c r="M10" s="15" t="str">
-        <f aca="false">IF(H10=0,IF(AND(G10=0,C10="Renewal",D10=1),"Finance (uplift waived)","None"),IF(AND(D10&gt;=2,H10&lt;=0.05),"None (multi-year)",IF(H10&lt;=0.12,"Finance","VP Customer Success")))</f>
+      <c r="N10" s="15" t="str">
+        <f aca="false">IF(I10=0,"None",IF(AND(D10&gt;=2,I10&lt;=0.05),"None (multi-year)",IF(I10&lt;=0.12,"Finance","VP Customer Success")))</f>
         <v>None</v>
       </c>
-      <c r="N10" s="18"/>
       <c r="O10" s="15" t="str">
-        <f aca="false">IF(OR(C10="Churn",C10="Downgrade"),IF(N10&lt;&gt;"","Non-regrettable","Regrettable"),"")</f>
-        <v/>
-      </c>
-      <c r="P10" s="23" t="n">
-        <f aca="false">IF(C10="Churn",-E10,IF(C10="Downgrade",F10,0))</f>
-        <v>0</v>
-      </c>
-      <c r="Q10" s="15"/>
+        <f aca="false">IF(D10&lt;2,"n/a",IF(E10="Upfront","Locked (0%)","5% a year"))</f>
+        <v>n/a</v>
+      </c>
+      <c r="P10" s="15"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="15" t="s">
@@ -4328,49 +4339,48 @@
       <c r="D11" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="E11" s="16" t="n">
+      <c r="E11" s="18" t="s">
+        <v>174</v>
+      </c>
+      <c r="F11" s="23" t="n">
         <v>28000</v>
       </c>
-      <c r="F11" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="G11" s="19" t="n">
+      <c r="G11" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" s="22" t="n">
+        <f aca="false">IF(C11="Renewal",0.05,0)</f>
         <v>0.05</v>
       </c>
-      <c r="H11" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="I11" s="23" t="n">
-        <f aca="false">L11*(1-H11)</f>
+      <c r="I11" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" s="23" t="n">
+        <f aca="false">IF(C11="Churn",0,F11*(1+H11)+G11)</f>
         <v>29400</v>
       </c>
-      <c r="J11" s="23" t="n">
-        <f aca="false">I11-E11</f>
+      <c r="K11" s="23" t="n">
+        <f aca="false">J11*(1-I11)</f>
+        <v>29400</v>
+      </c>
+      <c r="L11" s="23" t="n">
+        <f aca="false">K11-F11</f>
         <v>1400</v>
       </c>
-      <c r="K11" s="22" t="n">
-        <f aca="false">IF(E11=0,"new",J11/E11)</f>
+      <c r="M11" s="22" t="n">
+        <f aca="false">IF(F11=0,"new",L11/F11)</f>
         <v>0.05</v>
       </c>
-      <c r="L11" s="23" t="n">
-        <f aca="false">IF(C11="Churn",0,E11*(1+G11)+F11)</f>
-        <v>29400</v>
-      </c>
-      <c r="M11" s="15" t="str">
-        <f aca="false">IF(H11=0,IF(AND(G11=0,C11="Renewal",D11=1),"Finance (uplift waived)","None"),IF(AND(D11&gt;=2,H11&lt;=0.05),"None (multi-year)",IF(H11&lt;=0.12,"Finance","VP Customer Success")))</f>
+      <c r="N11" s="15" t="str">
+        <f aca="false">IF(I11=0,"None",IF(AND(D11&gt;=2,I11&lt;=0.05),"None (multi-year)",IF(I11&lt;=0.12,"Finance","VP Customer Success")))</f>
         <v>None</v>
       </c>
-      <c r="N11" s="18"/>
       <c r="O11" s="15" t="str">
-        <f aca="false">IF(OR(C11="Churn",C11="Downgrade"),IF(N11&lt;&gt;"","Non-regrettable","Regrettable"),"")</f>
-        <v/>
-      </c>
-      <c r="P11" s="23" t="n">
-        <f aca="false">IF(C11="Churn",-E11,IF(C11="Downgrade",F11,0))</f>
-        <v>0</v>
-      </c>
-      <c r="Q11" s="15" t="s">
-        <v>183</v>
+        <f aca="false">IF(D11&lt;2,"n/a",IF(E11="Upfront","Locked (0%)","5% a year"))</f>
+        <v>n/a</v>
+      </c>
+      <c r="P11" s="15" t="s">
+        <v>184</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4386,49 +4396,48 @@
       <c r="D12" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="E12" s="16" t="n">
+      <c r="E12" s="18" t="s">
+        <v>174</v>
+      </c>
+      <c r="F12" s="23" t="n">
         <v>35000</v>
       </c>
-      <c r="F12" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="G12" s="19" t="n">
+      <c r="G12" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" s="22" t="n">
+        <f aca="false">IF(C12="Renewal",0.05,0)</f>
         <v>0.05</v>
       </c>
-      <c r="H12" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="I12" s="23" t="n">
-        <f aca="false">L12*(1-H12)</f>
+      <c r="I12" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="J12" s="23" t="n">
+        <f aca="false">IF(C12="Churn",0,F12*(1+H12)+G12)</f>
         <v>36750</v>
       </c>
-      <c r="J12" s="23" t="n">
-        <f aca="false">I12-E12</f>
+      <c r="K12" s="23" t="n">
+        <f aca="false">J12*(1-I12)</f>
+        <v>36750</v>
+      </c>
+      <c r="L12" s="23" t="n">
+        <f aca="false">K12-F12</f>
         <v>1750</v>
       </c>
-      <c r="K12" s="22" t="n">
-        <f aca="false">IF(E12=0,"new",J12/E12)</f>
+      <c r="M12" s="22" t="n">
+        <f aca="false">IF(F12=0,"new",L12/F12)</f>
         <v>0.05</v>
       </c>
-      <c r="L12" s="23" t="n">
-        <f aca="false">IF(C12="Churn",0,E12*(1+G12)+F12)</f>
-        <v>36750</v>
-      </c>
-      <c r="M12" s="15" t="str">
-        <f aca="false">IF(H12=0,IF(AND(G12=0,C12="Renewal",D12=1),"Finance (uplift waived)","None"),IF(AND(D12&gt;=2,H12&lt;=0.05),"None (multi-year)",IF(H12&lt;=0.12,"Finance","VP Customer Success")))</f>
+      <c r="N12" s="15" t="str">
+        <f aca="false">IF(I12=0,"None",IF(AND(D12&gt;=2,I12&lt;=0.05),"None (multi-year)",IF(I12&lt;=0.12,"Finance","VP Customer Success")))</f>
         <v>None</v>
       </c>
-      <c r="N12" s="18"/>
       <c r="O12" s="15" t="str">
-        <f aca="false">IF(OR(C12="Churn",C12="Downgrade"),IF(N12&lt;&gt;"","Non-regrettable","Regrettable"),"")</f>
-        <v/>
-      </c>
-      <c r="P12" s="23" t="n">
-        <f aca="false">IF(C12="Churn",-E12,IF(C12="Downgrade",F12,0))</f>
-        <v>0</v>
-      </c>
-      <c r="Q12" s="15" t="s">
-        <v>184</v>
+        <f aca="false">IF(D12&lt;2,"n/a",IF(E12="Upfront","Locked (0%)","5% a year"))</f>
+        <v>n/a</v>
+      </c>
+      <c r="P12" s="15" t="s">
+        <v>185</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4436,57 +4445,56 @@
         <v>123</v>
       </c>
       <c r="B13" s="15" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="C13" s="18" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="D13" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="E13" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="F13" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="G13" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="H13" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="I13" s="23" t="n">
-        <f aca="false">L13*(1-H13)</f>
+      <c r="E13" s="18" t="s">
+        <v>174</v>
+      </c>
+      <c r="F13" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" s="22" t="n">
+        <f aca="false">IF(C13="Renewal",0.05,0)</f>
+        <v>0</v>
+      </c>
+      <c r="I13" s="19" t="n">
         <v>0</v>
       </c>
       <c r="J13" s="23" t="n">
-        <f aca="false">I13-E13</f>
-        <v>0</v>
-      </c>
-      <c r="K13" s="22" t="str">
-        <f aca="false">IF(E13=0,"new",J13/E13)</f>
+        <f aca="false">IF(C13="Churn",0,F13*(1+H13)+G13)</f>
+        <v>0</v>
+      </c>
+      <c r="K13" s="23" t="n">
+        <f aca="false">J13*(1-I13)</f>
+        <v>0</v>
+      </c>
+      <c r="L13" s="23" t="n">
+        <f aca="false">K13-F13</f>
+        <v>0</v>
+      </c>
+      <c r="M13" s="22" t="str">
+        <f aca="false">IF(F13=0,"new",L13/F13)</f>
         <v>new</v>
       </c>
-      <c r="L13" s="23" t="n">
-        <f aca="false">IF(C13="Churn",0,E13*(1+G13)+F13)</f>
-        <v>0</v>
-      </c>
-      <c r="M13" s="15" t="str">
-        <f aca="false">IF(H13=0,IF(AND(G13=0,C13="Renewal",D13=1),"Finance (uplift waived)","None"),IF(AND(D13&gt;=2,H13&lt;=0.05),"None (multi-year)",IF(H13&lt;=0.12,"Finance","VP Customer Success")))</f>
+      <c r="N13" s="15" t="str">
+        <f aca="false">IF(I13=0,"None",IF(AND(D13&gt;=2,I13&lt;=0.05),"None (multi-year)",IF(I13&lt;=0.12,"Finance","VP Customer Success")))</f>
         <v>None</v>
       </c>
-      <c r="N13" s="18"/>
       <c r="O13" s="15" t="str">
-        <f aca="false">IF(OR(C13="Churn",C13="Downgrade"),IF(N13&lt;&gt;"","Non-regrettable","Regrettable"),"")</f>
-        <v/>
-      </c>
-      <c r="P13" s="23" t="n">
-        <f aca="false">IF(C13="Churn",-E13,IF(C13="Downgrade",F13,0))</f>
-        <v>0</v>
-      </c>
-      <c r="Q13" s="15" t="s">
-        <v>187</v>
+        <f aca="false">IF(D13&lt;2,"n/a",IF(E13="Upfront","Locked (0%)","5% a year"))</f>
+        <v>n/a</v>
+      </c>
+      <c r="P13" s="15" t="s">
+        <v>188</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4494,7 +4502,7 @@
         <v>127</v>
       </c>
       <c r="B14" s="15" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="C14" s="18" t="s">
         <v>173</v>
@@ -4502,144 +4510,138 @@
       <c r="D14" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="E14" s="16" t="n">
+      <c r="E14" s="18" t="s">
+        <v>174</v>
+      </c>
+      <c r="F14" s="23" t="n">
         <v>46000</v>
       </c>
-      <c r="F14" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="G14" s="19" t="n">
+      <c r="G14" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" s="22" t="n">
+        <f aca="false">IF(C14="Renewal",0.05,0)</f>
         <v>0.05</v>
       </c>
-      <c r="H14" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="I14" s="23" t="n">
-        <f aca="false">L14*(1-H14)</f>
+      <c r="I14" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="J14" s="23" t="n">
+        <f aca="false">IF(C14="Churn",0,F14*(1+H14)+G14)</f>
         <v>48300</v>
       </c>
-      <c r="J14" s="23" t="n">
-        <f aca="false">I14-E14</f>
+      <c r="K14" s="23" t="n">
+        <f aca="false">J14*(1-I14)</f>
+        <v>48300</v>
+      </c>
+      <c r="L14" s="23" t="n">
+        <f aca="false">K14-F14</f>
         <v>2300</v>
       </c>
-      <c r="K14" s="22" t="n">
-        <f aca="false">IF(E14=0,"new",J14/E14)</f>
+      <c r="M14" s="22" t="n">
+        <f aca="false">IF(F14=0,"new",L14/F14)</f>
         <v>0.05</v>
       </c>
-      <c r="L14" s="23" t="n">
-        <f aca="false">IF(C14="Churn",0,E14*(1+G14)+F14)</f>
-        <v>48300</v>
-      </c>
-      <c r="M14" s="15" t="str">
-        <f aca="false">IF(H14=0,IF(AND(G14=0,C14="Renewal",D14=1),"Finance (uplift waived)","None"),IF(AND(D14&gt;=2,H14&lt;=0.05),"None (multi-year)",IF(H14&lt;=0.12,"Finance","VP Customer Success")))</f>
+      <c r="N14" s="15" t="str">
+        <f aca="false">IF(I14=0,"None",IF(AND(D14&gt;=2,I14&lt;=0.05),"None (multi-year)",IF(I14&lt;=0.12,"Finance","VP Customer Success")))</f>
         <v>None</v>
       </c>
-      <c r="N14" s="18"/>
       <c r="O14" s="15" t="str">
-        <f aca="false">IF(OR(C14="Churn",C14="Downgrade"),IF(N14&lt;&gt;"","Non-regrettable","Regrettable"),"")</f>
-        <v/>
-      </c>
-      <c r="P14" s="23" t="n">
-        <f aca="false">IF(C14="Churn",-E14,IF(C14="Downgrade",F14,0))</f>
-        <v>0</v>
-      </c>
-      <c r="Q14" s="15"/>
+        <f aca="false">IF(D14&lt;2,"n/a",IF(E14="Upfront","Locked (0%)","5% a year"))</f>
+        <v>n/a</v>
+      </c>
+      <c r="P14" s="15"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="15" t="s">
         <v>132</v>
       </c>
       <c r="B15" s="15" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="C15" s="18" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="D15" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="E15" s="16" t="n">
+      <c r="E15" s="18" t="s">
+        <v>174</v>
+      </c>
+      <c r="F15" s="23" t="n">
         <v>40000</v>
       </c>
-      <c r="F15" s="16" t="n">
+      <c r="G15" s="16" t="n">
         <v>-8000</v>
       </c>
-      <c r="G15" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="H15" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="I15" s="23" t="n">
-        <f aca="false">L15*(1-H15)</f>
+      <c r="H15" s="22" t="n">
+        <f aca="false">IF(C15="Renewal",0.05,0)</f>
+        <v>0</v>
+      </c>
+      <c r="I15" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="J15" s="23" t="n">
+        <f aca="false">IF(C15="Churn",0,F15*(1+H15)+G15)</f>
         <v>32000</v>
       </c>
-      <c r="J15" s="23" t="n">
-        <f aca="false">I15-E15</f>
+      <c r="K15" s="23" t="n">
+        <f aca="false">J15*(1-I15)</f>
+        <v>32000</v>
+      </c>
+      <c r="L15" s="23" t="n">
+        <f aca="false">K15-F15</f>
         <v>-8000</v>
       </c>
-      <c r="K15" s="22" t="n">
-        <f aca="false">IF(E15=0,"new",J15/E15)</f>
+      <c r="M15" s="22" t="n">
+        <f aca="false">IF(F15=0,"new",L15/F15)</f>
         <v>-0.2</v>
       </c>
-      <c r="L15" s="23" t="n">
-        <f aca="false">IF(C15="Churn",0,E15*(1+G15)+F15)</f>
-        <v>32000</v>
-      </c>
-      <c r="M15" s="15" t="str">
-        <f aca="false">IF(H15=0,IF(AND(G15=0,C15="Renewal",D15=1),"Finance (uplift waived)","None"),IF(AND(D15&gt;=2,H15&lt;=0.05),"None (multi-year)",IF(H15&lt;=0.12,"Finance","VP Customer Success")))</f>
+      <c r="N15" s="15" t="str">
+        <f aca="false">IF(I15=0,"None",IF(AND(D15&gt;=2,I15&lt;=0.05),"None (multi-year)",IF(I15&lt;=0.12,"Finance","VP Customer Success")))</f>
         <v>None</v>
       </c>
-      <c r="N15" s="18"/>
       <c r="O15" s="15" t="str">
-        <f aca="false">IF(OR(C15="Churn",C15="Downgrade"),IF(N15&lt;&gt;"","Non-regrettable","Regrettable"),"")</f>
-        <v>Regrettable</v>
-      </c>
-      <c r="P15" s="23" t="n">
-        <f aca="false">IF(C15="Churn",-E15,IF(C15="Downgrade",F15,0))</f>
-        <v>-8000</v>
-      </c>
-      <c r="Q15" s="15" t="s">
-        <v>188</v>
+        <f aca="false">IF(D15&lt;2,"n/a",IF(E15="Upfront","Locked (0%)","5% a year"))</f>
+        <v>n/a</v>
+      </c>
+      <c r="P15" s="15" t="s">
+        <v>189</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="E17" s="24" t="n">
-        <f aca="false">SUM(E5:E15)</f>
-        <v>375000</v>
-      </c>
       <c r="F17" s="24" t="n">
         <f aca="false">SUM(F5:F15)</f>
+        <v>375000</v>
+      </c>
+      <c r="G17" s="24" t="n">
+        <f aca="false">SUM(G5:G15)</f>
         <v>-23000</v>
-      </c>
-      <c r="I17" s="24" t="n">
-        <f aca="false">SUM(I5:I15)</f>
-        <v>360664</v>
       </c>
       <c r="J17" s="24" t="n">
         <f aca="false">SUM(J5:J15)</f>
-        <v>-14336</v>
+        <v>366500</v>
+      </c>
+      <c r="K17" s="24" t="n">
+        <f aca="false">SUM(K5:K15)</f>
+        <v>361964</v>
       </c>
       <c r="L17" s="24" t="n">
         <f aca="false">SUM(L5:L15)</f>
-        <v>365200</v>
-      </c>
-      <c r="P17" s="24" t="n">
-        <f aca="false">SUM(P5:P15)</f>
-        <v>-23000</v>
+        <v>-13036</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="31" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B20" s="31"/>
       <c r="C20" s="31"/>
@@ -4656,37 +4658,32 @@
       <c r="N20" s="31"/>
       <c r="O20" s="31"/>
       <c r="P20" s="31"/>
-      <c r="Q20" s="31"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A2:Q2"/>
-    <mergeCell ref="A20:Q20"/>
+    <mergeCell ref="A2:N2"/>
+    <mergeCell ref="A20:P20"/>
   </mergeCells>
-  <conditionalFormatting sqref="J5:K55">
+  <conditionalFormatting sqref="L5:M55">
     <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="4">
-      <formula>AND(ISNUMBER(J5),J5&gt;0)</formula>
+      <formula>AND(ISNUMBER(L5),L5&gt;0)</formula>
     </cfRule>
     <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
-      <formula>AND(ISNUMBER(J5),J5&lt;0)</formula>
+      <formula>AND(ISNUMBER(L5),L5&lt;0)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M5:M55">
+  <conditionalFormatting sqref="N5:N55">
     <cfRule type="expression" priority="4" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="2">
-      <formula>LEFT(M5,4)&lt;&gt;"None"</formula>
+      <formula>LEFT(N5,4)&lt;&gt;"None"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="O5:O55">
-    <cfRule type="expression" priority="5" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
-      <formula>O5="Regrettable"</formula>
-    </cfRule>
-    <cfRule type="expression" priority="6" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="3">
-      <formula>O5="Non-regrettable"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <dataValidations count="1">
+  <dataValidations count="2">
     <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C5:C55" type="list">
-      <formula1>"Renewal,Upsell,Downgrade,Cross-sell,Churn"</formula1>
+      <formula1>"Renewal,Upsell,Downgrade,Churn"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E5:E55" type="list">
+      <formula1>"Annual,Upfront"</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
@@ -4705,22 +4702,24 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K17"/>
+  <dimension ref="A1:K18"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="20"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="7" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="16"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="9" style="0" width="13"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="11"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4728,34 +4727,34 @@
         <v>157</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="G3" s="6" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="H3" s="6" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="I3" s="6" t="s">
         <v>61</v>
       </c>
       <c r="J3" s="6" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="K3" s="6" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4764,35 +4763,29 @@
         <v>Vantage Freight</v>
       </c>
       <c r="B4" s="23" t="n">
-        <f aca="false">SUMIFS(Products!$E:$E,Products!$A:$A,$A4)</f>
+        <f aca="false">SUMIFS(Products!$F:$F,Products!$A:$A,$A4)</f>
         <v>21000</v>
       </c>
       <c r="C4" s="23" t="n">
-        <f aca="false">SUMPRODUCT((Products!$A$5:$A$200=$A4)*(Products!$C$5:$C$200="Renewal")*Products!$E$5:$E$200*Products!$G$5:$G$200)</f>
+        <f aca="false">SUMPRODUCT((Products!$A$5:$A$200=$A4)*Products!$F$5:$F$200*Products!$H$5:$H$200)</f>
         <v>1050</v>
       </c>
       <c r="D4" s="23" t="n">
-        <f aca="false">SUMIFS(Products!$F:$F,Products!$A:$A,$A4,Products!$C:$C,"Upsell")+SUMIFS(Products!$F:$F,Products!$A:$A,$A4,Products!$C:$C,"Cross-sell")</f>
+        <f aca="false">SUMIFS(Products!$G:$G,Products!$A:$A,$A4,Products!$C:$C,"Upsell")</f>
         <v>0</v>
       </c>
       <c r="E4" s="23" t="n">
-        <f aca="false">SUMIFS(Products!$P:$P,Products!$A:$A,$A4,Products!$O:$O,"Regrettable")</f>
-        <v>0</v>
-      </c>
-      <c r="F4" s="23" t="n">
-        <f aca="false">SUMIFS(Products!$P:$P,Products!$A:$A,$A4,Products!$O:$O,"Non-regrettable")</f>
-        <v>0</v>
-      </c>
-      <c r="G4" s="23" t="n">
-        <f aca="false">-F4</f>
-        <v>-0</v>
-      </c>
+        <f aca="false">SUMIFS(Products!$G:$G,Products!$A:$A,$A4,Products!$C:$C,"Downgrade")-SUMIFS(Products!$F:$F,Products!$A:$A,$A4,Products!$C:$C,"Churn")</f>
+        <v>0</v>
+      </c>
+      <c r="F4" s="18"/>
+      <c r="G4" s="18"/>
       <c r="H4" s="23" t="n">
-        <f aca="false">MIN(0,C4-(SUMIFS(Products!$L:$L,Products!$A:$A,$A4)-SUMIFS(Products!$I:$I,Products!$A:$A,$A4)))</f>
+        <f aca="false">MIN(0,C4-(SUMIFS(Products!$J:$J,Products!$A:$A,$A4)-SUMIFS(Products!$K:$K,Products!$A:$A,$A4)))</f>
         <v>0</v>
       </c>
       <c r="I4" s="23" t="n">
-        <f aca="false">SUMIFS(Products!$I:$I,Products!$A:$A,$A4)</f>
+        <f aca="false">SUMIFS(Products!$K:$K,Products!$A:$A,$A4)</f>
         <v>22050</v>
       </c>
       <c r="J4" s="23" t="n">
@@ -4810,35 +4803,29 @@
         <v>Northwind Logistics</v>
       </c>
       <c r="B5" s="23" t="n">
-        <f aca="false">SUMIFS(Products!$E:$E,Products!$A:$A,$A5)</f>
+        <f aca="false">SUMIFS(Products!$F:$F,Products!$A:$A,$A5)</f>
         <v>48000</v>
       </c>
       <c r="C5" s="23" t="n">
-        <f aca="false">SUMPRODUCT((Products!$A$5:$A$200=$A5)*(Products!$C$5:$C$200="Renewal")*Products!$E$5:$E$200*Products!$G$5:$G$200)</f>
+        <f aca="false">SUMPRODUCT((Products!$A$5:$A$200=$A5)*Products!$F$5:$F$200*Products!$H$5:$H$200)</f>
         <v>2400</v>
       </c>
       <c r="D5" s="23" t="n">
-        <f aca="false">SUMIFS(Products!$F:$F,Products!$A:$A,$A5,Products!$C:$C,"Upsell")+SUMIFS(Products!$F:$F,Products!$A:$A,$A5,Products!$C:$C,"Cross-sell")</f>
+        <f aca="false">SUMIFS(Products!$G:$G,Products!$A:$A,$A5,Products!$C:$C,"Upsell")</f>
         <v>0</v>
       </c>
       <c r="E5" s="23" t="n">
-        <f aca="false">SUMIFS(Products!$P:$P,Products!$A:$A,$A5,Products!$O:$O,"Regrettable")</f>
-        <v>0</v>
-      </c>
-      <c r="F5" s="23" t="n">
-        <f aca="false">SUMIFS(Products!$P:$P,Products!$A:$A,$A5,Products!$O:$O,"Non-regrettable")</f>
-        <v>0</v>
-      </c>
-      <c r="G5" s="23" t="n">
-        <f aca="false">-F5</f>
-        <v>-0</v>
-      </c>
+        <f aca="false">SUMIFS(Products!$G:$G,Products!$A:$A,$A5,Products!$C:$C,"Downgrade")-SUMIFS(Products!$F:$F,Products!$A:$A,$A5,Products!$C:$C,"Churn")</f>
+        <v>0</v>
+      </c>
+      <c r="F5" s="18"/>
+      <c r="G5" s="18"/>
       <c r="H5" s="23" t="n">
-        <f aca="false">MIN(0,C5-(SUMIFS(Products!$L:$L,Products!$A:$A,$A5)-SUMIFS(Products!$I:$I,Products!$A:$A,$A5)))</f>
+        <f aca="false">MIN(0,C5-(SUMIFS(Products!$J:$J,Products!$A:$A,$A5)-SUMIFS(Products!$K:$K,Products!$A:$A,$A5)))</f>
         <v>0</v>
       </c>
       <c r="I5" s="23" t="n">
-        <f aca="false">SUMIFS(Products!$I:$I,Products!$A:$A,$A5)</f>
+        <f aca="false">SUMIFS(Products!$K:$K,Products!$A:$A,$A5)</f>
         <v>50400</v>
       </c>
       <c r="J5" s="23" t="n">
@@ -4856,44 +4843,38 @@
         <v>Pixelforge</v>
       </c>
       <c r="B6" s="23" t="n">
-        <f aca="false">SUMIFS(Products!$E:$E,Products!$A:$A,$A6)</f>
+        <f aca="false">SUMIFS(Products!$F:$F,Products!$A:$A,$A6)</f>
         <v>26000</v>
       </c>
       <c r="C6" s="23" t="n">
-        <f aca="false">SUMPRODUCT((Products!$A$5:$A$200=$A6)*(Products!$C$5:$C$200="Renewal")*Products!$E$5:$E$200*Products!$G$5:$G$200)</f>
-        <v>0</v>
+        <f aca="false">SUMPRODUCT((Products!$A$5:$A$200=$A6)*Products!$F$5:$F$200*Products!$H$5:$H$200)</f>
+        <v>1300</v>
       </c>
       <c r="D6" s="23" t="n">
-        <f aca="false">SUMIFS(Products!$F:$F,Products!$A:$A,$A6,Products!$C:$C,"Upsell")+SUMIFS(Products!$F:$F,Products!$A:$A,$A6,Products!$C:$C,"Cross-sell")</f>
+        <f aca="false">SUMIFS(Products!$G:$G,Products!$A:$A,$A6,Products!$C:$C,"Upsell")</f>
         <v>0</v>
       </c>
       <c r="E6" s="23" t="n">
-        <f aca="false">SUMIFS(Products!$P:$P,Products!$A:$A,$A6,Products!$O:$O,"Regrettable")</f>
-        <v>0</v>
-      </c>
-      <c r="F6" s="23" t="n">
-        <f aca="false">SUMIFS(Products!$P:$P,Products!$A:$A,$A6,Products!$O:$O,"Non-regrettable")</f>
-        <v>0</v>
-      </c>
-      <c r="G6" s="23" t="n">
-        <f aca="false">-F6</f>
-        <v>-0</v>
-      </c>
+        <f aca="false">SUMIFS(Products!$G:$G,Products!$A:$A,$A6,Products!$C:$C,"Downgrade")-SUMIFS(Products!$F:$F,Products!$A:$A,$A6,Products!$C:$C,"Churn")</f>
+        <v>0</v>
+      </c>
+      <c r="F6" s="18"/>
+      <c r="G6" s="18"/>
       <c r="H6" s="23" t="n">
-        <f aca="false">MIN(0,C6-(SUMIFS(Products!$L:$L,Products!$A:$A,$A6)-SUMIFS(Products!$I:$I,Products!$A:$A,$A6)))</f>
+        <f aca="false">MIN(0,C6-(SUMIFS(Products!$J:$J,Products!$A:$A,$A6)-SUMIFS(Products!$K:$K,Products!$A:$A,$A6)))</f>
         <v>0</v>
       </c>
       <c r="I6" s="23" t="n">
-        <f aca="false">SUMIFS(Products!$I:$I,Products!$A:$A,$A6)</f>
-        <v>26000</v>
+        <f aca="false">SUMIFS(Products!$K:$K,Products!$A:$A,$A6)</f>
+        <v>27300</v>
       </c>
       <c r="J6" s="23" t="n">
         <f aca="false">I6-B6</f>
-        <v>0</v>
+        <v>1300</v>
       </c>
       <c r="K6" s="22" t="n">
         <f aca="false">IF(B6=0,0,J6/B6)</f>
-        <v>0</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4902,35 +4883,33 @@
         <v>Halden Health</v>
       </c>
       <c r="B7" s="23" t="n">
-        <f aca="false">SUMIFS(Products!$E:$E,Products!$A:$A,$A7)</f>
+        <f aca="false">SUMIFS(Products!$F:$F,Products!$A:$A,$A7)</f>
         <v>45000</v>
       </c>
       <c r="C7" s="23" t="n">
-        <f aca="false">SUMPRODUCT((Products!$A$5:$A$200=$A7)*(Products!$C$5:$C$200="Renewal")*Products!$E$5:$E$200*Products!$G$5:$G$200)</f>
+        <f aca="false">SUMPRODUCT((Products!$A$5:$A$200=$A7)*Products!$F$5:$F$200*Products!$H$5:$H$200)</f>
         <v>0</v>
       </c>
       <c r="D7" s="23" t="n">
-        <f aca="false">SUMIFS(Products!$F:$F,Products!$A:$A,$A7,Products!$C:$C,"Upsell")+SUMIFS(Products!$F:$F,Products!$A:$A,$A7,Products!$C:$C,"Cross-sell")</f>
+        <f aca="false">SUMIFS(Products!$G:$G,Products!$A:$A,$A7,Products!$C:$C,"Upsell")</f>
         <v>0</v>
       </c>
       <c r="E7" s="23" t="n">
-        <f aca="false">SUMIFS(Products!$P:$P,Products!$A:$A,$A7,Products!$O:$O,"Regrettable")</f>
+        <f aca="false">SUMIFS(Products!$G:$G,Products!$A:$A,$A7,Products!$C:$C,"Downgrade")-SUMIFS(Products!$F:$F,Products!$A:$A,$A7,Products!$C:$C,"Churn")</f>
         <v>-15000</v>
       </c>
-      <c r="F7" s="23" t="n">
-        <f aca="false">SUMIFS(Products!$P:$P,Products!$A:$A,$A7,Products!$O:$O,"Non-regrettable")</f>
-        <v>0</v>
-      </c>
-      <c r="G7" s="23" t="n">
-        <f aca="false">-F7</f>
-        <v>-0</v>
+      <c r="F7" s="18" t="s">
+        <v>201</v>
+      </c>
+      <c r="G7" s="18" t="s">
+        <v>202</v>
       </c>
       <c r="H7" s="23" t="n">
-        <f aca="false">MIN(0,C7-(SUMIFS(Products!$L:$L,Products!$A:$A,$A7)-SUMIFS(Products!$I:$I,Products!$A:$A,$A7)))</f>
+        <f aca="false">MIN(0,C7-(SUMIFS(Products!$J:$J,Products!$A:$A,$A7)-SUMIFS(Products!$K:$K,Products!$A:$A,$A7)))</f>
         <v>0</v>
       </c>
       <c r="I7" s="23" t="n">
-        <f aca="false">SUMIFS(Products!$I:$I,Products!$A:$A,$A7)</f>
+        <f aca="false">SUMIFS(Products!$K:$K,Products!$A:$A,$A7)</f>
         <v>30000</v>
       </c>
       <c r="J7" s="23" t="n">
@@ -4948,35 +4927,29 @@
         <v>Brightloop</v>
       </c>
       <c r="B8" s="23" t="n">
-        <f aca="false">SUMIFS(Products!$E:$E,Products!$A:$A,$A8)</f>
+        <f aca="false">SUMIFS(Products!$F:$F,Products!$A:$A,$A8)</f>
         <v>36000</v>
       </c>
       <c r="C8" s="23" t="n">
-        <f aca="false">SUMPRODUCT((Products!$A$5:$A$200=$A8)*(Products!$C$5:$C$200="Renewal")*Products!$E$5:$E$200*Products!$G$5:$G$200)</f>
+        <f aca="false">SUMPRODUCT((Products!$A$5:$A$200=$A8)*Products!$F$5:$F$200*Products!$H$5:$H$200)</f>
         <v>1800</v>
       </c>
       <c r="D8" s="23" t="n">
-        <f aca="false">SUMIFS(Products!$F:$F,Products!$A:$A,$A8,Products!$C:$C,"Upsell")+SUMIFS(Products!$F:$F,Products!$A:$A,$A8,Products!$C:$C,"Cross-sell")</f>
+        <f aca="false">SUMIFS(Products!$G:$G,Products!$A:$A,$A8,Products!$C:$C,"Upsell")</f>
         <v>0</v>
       </c>
       <c r="E8" s="23" t="n">
-        <f aca="false">SUMIFS(Products!$P:$P,Products!$A:$A,$A8,Products!$O:$O,"Regrettable")</f>
-        <v>0</v>
-      </c>
-      <c r="F8" s="23" t="n">
-        <f aca="false">SUMIFS(Products!$P:$P,Products!$A:$A,$A8,Products!$O:$O,"Non-regrettable")</f>
-        <v>0</v>
-      </c>
-      <c r="G8" s="23" t="n">
-        <f aca="false">-F8</f>
-        <v>-0</v>
-      </c>
+        <f aca="false">SUMIFS(Products!$G:$G,Products!$A:$A,$A8,Products!$C:$C,"Downgrade")-SUMIFS(Products!$F:$F,Products!$A:$A,$A8,Products!$C:$C,"Churn")</f>
+        <v>0</v>
+      </c>
+      <c r="F8" s="18"/>
+      <c r="G8" s="18"/>
       <c r="H8" s="23" t="n">
-        <f aca="false">MIN(0,C8-(SUMIFS(Products!$L:$L,Products!$A:$A,$A8)-SUMIFS(Products!$I:$I,Products!$A:$A,$A8)))</f>
+        <f aca="false">MIN(0,C8-(SUMIFS(Products!$J:$J,Products!$A:$A,$A8)-SUMIFS(Products!$K:$K,Products!$A:$A,$A8)))</f>
         <v>-2736</v>
       </c>
       <c r="I8" s="23" t="n">
-        <f aca="false">SUMIFS(Products!$I:$I,Products!$A:$A,$A8)</f>
+        <f aca="false">SUMIFS(Products!$K:$K,Products!$A:$A,$A8)</f>
         <v>33264</v>
       </c>
       <c r="J8" s="23" t="n">
@@ -4994,35 +4967,29 @@
         <v>Tessera Finance</v>
       </c>
       <c r="B9" s="23" t="n">
-        <f aca="false">SUMIFS(Products!$E:$E,Products!$A:$A,$A9)</f>
+        <f aca="false">SUMIFS(Products!$F:$F,Products!$A:$A,$A9)</f>
         <v>50000</v>
       </c>
       <c r="C9" s="23" t="n">
-        <f aca="false">SUMPRODUCT((Products!$A$5:$A$200=$A9)*(Products!$C$5:$C$200="Renewal")*Products!$E$5:$E$200*Products!$G$5:$G$200)</f>
+        <f aca="false">SUMPRODUCT((Products!$A$5:$A$200=$A9)*Products!$F$5:$F$200*Products!$H$5:$H$200)</f>
         <v>2500</v>
       </c>
       <c r="D9" s="23" t="n">
-        <f aca="false">SUMIFS(Products!$F:$F,Products!$A:$A,$A9,Products!$C:$C,"Upsell")+SUMIFS(Products!$F:$F,Products!$A:$A,$A9,Products!$C:$C,"Cross-sell")</f>
+        <f aca="false">SUMIFS(Products!$G:$G,Products!$A:$A,$A9,Products!$C:$C,"Upsell")</f>
         <v>0</v>
       </c>
       <c r="E9" s="23" t="n">
-        <f aca="false">SUMIFS(Products!$P:$P,Products!$A:$A,$A9,Products!$O:$O,"Regrettable")</f>
-        <v>0</v>
-      </c>
-      <c r="F9" s="23" t="n">
-        <f aca="false">SUMIFS(Products!$P:$P,Products!$A:$A,$A9,Products!$O:$O,"Non-regrettable")</f>
-        <v>0</v>
-      </c>
-      <c r="G9" s="23" t="n">
-        <f aca="false">-F9</f>
-        <v>-0</v>
-      </c>
+        <f aca="false">SUMIFS(Products!$G:$G,Products!$A:$A,$A9,Products!$C:$C,"Downgrade")-SUMIFS(Products!$F:$F,Products!$A:$A,$A9,Products!$C:$C,"Churn")</f>
+        <v>0</v>
+      </c>
+      <c r="F9" s="18"/>
+      <c r="G9" s="18"/>
       <c r="H9" s="23" t="n">
-        <f aca="false">MIN(0,C9-(SUMIFS(Products!$L:$L,Products!$A:$A,$A9)-SUMIFS(Products!$I:$I,Products!$A:$A,$A9)))</f>
+        <f aca="false">MIN(0,C9-(SUMIFS(Products!$J:$J,Products!$A:$A,$A9)-SUMIFS(Products!$K:$K,Products!$A:$A,$A9)))</f>
         <v>0</v>
       </c>
       <c r="I9" s="23" t="n">
-        <f aca="false">SUMIFS(Products!$I:$I,Products!$A:$A,$A9)</f>
+        <f aca="false">SUMIFS(Products!$K:$K,Products!$A:$A,$A9)</f>
         <v>52500</v>
       </c>
       <c r="J9" s="23" t="n">
@@ -5040,35 +5007,29 @@
         <v>Lumen Retail</v>
       </c>
       <c r="B10" s="23" t="n">
-        <f aca="false">SUMIFS(Products!$E:$E,Products!$A:$A,$A10)</f>
+        <f aca="false">SUMIFS(Products!$F:$F,Products!$A:$A,$A10)</f>
         <v>28000</v>
       </c>
       <c r="C10" s="23" t="n">
-        <f aca="false">SUMPRODUCT((Products!$A$5:$A$200=$A10)*(Products!$C$5:$C$200="Renewal")*Products!$E$5:$E$200*Products!$G$5:$G$200)</f>
+        <f aca="false">SUMPRODUCT((Products!$A$5:$A$200=$A10)*Products!$F$5:$F$200*Products!$H$5:$H$200)</f>
         <v>1400</v>
       </c>
       <c r="D10" s="23" t="n">
-        <f aca="false">SUMIFS(Products!$F:$F,Products!$A:$A,$A10,Products!$C:$C,"Upsell")+SUMIFS(Products!$F:$F,Products!$A:$A,$A10,Products!$C:$C,"Cross-sell")</f>
+        <f aca="false">SUMIFS(Products!$G:$G,Products!$A:$A,$A10,Products!$C:$C,"Upsell")</f>
         <v>0</v>
       </c>
       <c r="E10" s="23" t="n">
-        <f aca="false">SUMIFS(Products!$P:$P,Products!$A:$A,$A10,Products!$O:$O,"Regrettable")</f>
-        <v>0</v>
-      </c>
-      <c r="F10" s="23" t="n">
-        <f aca="false">SUMIFS(Products!$P:$P,Products!$A:$A,$A10,Products!$O:$O,"Non-regrettable")</f>
-        <v>0</v>
-      </c>
-      <c r="G10" s="23" t="n">
-        <f aca="false">-F10</f>
-        <v>-0</v>
-      </c>
+        <f aca="false">SUMIFS(Products!$G:$G,Products!$A:$A,$A10,Products!$C:$C,"Downgrade")-SUMIFS(Products!$F:$F,Products!$A:$A,$A10,Products!$C:$C,"Churn")</f>
+        <v>0</v>
+      </c>
+      <c r="F10" s="18"/>
+      <c r="G10" s="18"/>
       <c r="H10" s="23" t="n">
-        <f aca="false">MIN(0,C10-(SUMIFS(Products!$L:$L,Products!$A:$A,$A10)-SUMIFS(Products!$I:$I,Products!$A:$A,$A10)))</f>
+        <f aca="false">MIN(0,C10-(SUMIFS(Products!$J:$J,Products!$A:$A,$A10)-SUMIFS(Products!$K:$K,Products!$A:$A,$A10)))</f>
         <v>0</v>
       </c>
       <c r="I10" s="23" t="n">
-        <f aca="false">SUMIFS(Products!$I:$I,Products!$A:$A,$A10)</f>
+        <f aca="false">SUMIFS(Products!$K:$K,Products!$A:$A,$A10)</f>
         <v>29400</v>
       </c>
       <c r="J10" s="23" t="n">
@@ -5086,35 +5047,29 @@
         <v>Kestrel Analytics</v>
       </c>
       <c r="B11" s="23" t="n">
-        <f aca="false">SUMIFS(Products!$E:$E,Products!$A:$A,$A11)</f>
+        <f aca="false">SUMIFS(Products!$F:$F,Products!$A:$A,$A11)</f>
         <v>35000</v>
       </c>
       <c r="C11" s="23" t="n">
-        <f aca="false">SUMPRODUCT((Products!$A$5:$A$200=$A11)*(Products!$C$5:$C$200="Renewal")*Products!$E$5:$E$200*Products!$G$5:$G$200)</f>
+        <f aca="false">SUMPRODUCT((Products!$A$5:$A$200=$A11)*Products!$F$5:$F$200*Products!$H$5:$H$200)</f>
         <v>1750</v>
       </c>
       <c r="D11" s="23" t="n">
-        <f aca="false">SUMIFS(Products!$F:$F,Products!$A:$A,$A11,Products!$C:$C,"Upsell")+SUMIFS(Products!$F:$F,Products!$A:$A,$A11,Products!$C:$C,"Cross-sell")</f>
+        <f aca="false">SUMIFS(Products!$G:$G,Products!$A:$A,$A11,Products!$C:$C,"Upsell")</f>
         <v>0</v>
       </c>
       <c r="E11" s="23" t="n">
-        <f aca="false">SUMIFS(Products!$P:$P,Products!$A:$A,$A11,Products!$O:$O,"Regrettable")</f>
-        <v>0</v>
-      </c>
-      <c r="F11" s="23" t="n">
-        <f aca="false">SUMIFS(Products!$P:$P,Products!$A:$A,$A11,Products!$O:$O,"Non-regrettable")</f>
-        <v>0</v>
-      </c>
-      <c r="G11" s="23" t="n">
-        <f aca="false">-F11</f>
-        <v>-0</v>
-      </c>
+        <f aca="false">SUMIFS(Products!$G:$G,Products!$A:$A,$A11,Products!$C:$C,"Downgrade")-SUMIFS(Products!$F:$F,Products!$A:$A,$A11,Products!$C:$C,"Churn")</f>
+        <v>0</v>
+      </c>
+      <c r="F11" s="18"/>
+      <c r="G11" s="18"/>
       <c r="H11" s="23" t="n">
-        <f aca="false">MIN(0,C11-(SUMIFS(Products!$L:$L,Products!$A:$A,$A11)-SUMIFS(Products!$I:$I,Products!$A:$A,$A11)))</f>
+        <f aca="false">MIN(0,C11-(SUMIFS(Products!$J:$J,Products!$A:$A,$A11)-SUMIFS(Products!$K:$K,Products!$A:$A,$A11)))</f>
         <v>0</v>
       </c>
       <c r="I11" s="23" t="n">
-        <f aca="false">SUMIFS(Products!$I:$I,Products!$A:$A,$A11)</f>
+        <f aca="false">SUMIFS(Products!$K:$K,Products!$A:$A,$A11)</f>
         <v>36750</v>
       </c>
       <c r="J11" s="23" t="n">
@@ -5132,35 +5087,29 @@
         <v>Marlowe Insurance</v>
       </c>
       <c r="B12" s="23" t="n">
-        <f aca="false">SUMIFS(Products!$E:$E,Products!$A:$A,$A12)</f>
+        <f aca="false">SUMIFS(Products!$F:$F,Products!$A:$A,$A12)</f>
         <v>46000</v>
       </c>
       <c r="C12" s="23" t="n">
-        <f aca="false">SUMPRODUCT((Products!$A$5:$A$200=$A12)*(Products!$C$5:$C$200="Renewal")*Products!$E$5:$E$200*Products!$G$5:$G$200)</f>
+        <f aca="false">SUMPRODUCT((Products!$A$5:$A$200=$A12)*Products!$F$5:$F$200*Products!$H$5:$H$200)</f>
         <v>2300</v>
       </c>
       <c r="D12" s="23" t="n">
-        <f aca="false">SUMIFS(Products!$F:$F,Products!$A:$A,$A12,Products!$C:$C,"Upsell")+SUMIFS(Products!$F:$F,Products!$A:$A,$A12,Products!$C:$C,"Cross-sell")</f>
+        <f aca="false">SUMIFS(Products!$G:$G,Products!$A:$A,$A12,Products!$C:$C,"Upsell")</f>
         <v>0</v>
       </c>
       <c r="E12" s="23" t="n">
-        <f aca="false">SUMIFS(Products!$P:$P,Products!$A:$A,$A12,Products!$O:$O,"Regrettable")</f>
-        <v>0</v>
-      </c>
-      <c r="F12" s="23" t="n">
-        <f aca="false">SUMIFS(Products!$P:$P,Products!$A:$A,$A12,Products!$O:$O,"Non-regrettable")</f>
-        <v>0</v>
-      </c>
-      <c r="G12" s="23" t="n">
-        <f aca="false">-F12</f>
-        <v>-0</v>
-      </c>
+        <f aca="false">SUMIFS(Products!$G:$G,Products!$A:$A,$A12,Products!$C:$C,"Downgrade")-SUMIFS(Products!$F:$F,Products!$A:$A,$A12,Products!$C:$C,"Churn")</f>
+        <v>0</v>
+      </c>
+      <c r="F12" s="18"/>
+      <c r="G12" s="18"/>
       <c r="H12" s="23" t="n">
-        <f aca="false">MIN(0,C12-(SUMIFS(Products!$L:$L,Products!$A:$A,$A12)-SUMIFS(Products!$I:$I,Products!$A:$A,$A12)))</f>
+        <f aca="false">MIN(0,C12-(SUMIFS(Products!$J:$J,Products!$A:$A,$A12)-SUMIFS(Products!$K:$K,Products!$A:$A,$A12)))</f>
         <v>0</v>
       </c>
       <c r="I12" s="23" t="n">
-        <f aca="false">SUMIFS(Products!$I:$I,Products!$A:$A,$A12)</f>
+        <f aca="false">SUMIFS(Products!$K:$K,Products!$A:$A,$A12)</f>
         <v>48300</v>
       </c>
       <c r="J12" s="23" t="n">
@@ -5178,35 +5127,33 @@
         <v>Quanta Labs</v>
       </c>
       <c r="B13" s="23" t="n">
-        <f aca="false">SUMIFS(Products!$E:$E,Products!$A:$A,$A13)</f>
+        <f aca="false">SUMIFS(Products!$F:$F,Products!$A:$A,$A13)</f>
         <v>40000</v>
       </c>
       <c r="C13" s="23" t="n">
-        <f aca="false">SUMPRODUCT((Products!$A$5:$A$200=$A13)*(Products!$C$5:$C$200="Renewal")*Products!$E$5:$E$200*Products!$G$5:$G$200)</f>
+        <f aca="false">SUMPRODUCT((Products!$A$5:$A$200=$A13)*Products!$F$5:$F$200*Products!$H$5:$H$200)</f>
         <v>0</v>
       </c>
       <c r="D13" s="23" t="n">
-        <f aca="false">SUMIFS(Products!$F:$F,Products!$A:$A,$A13,Products!$C:$C,"Upsell")+SUMIFS(Products!$F:$F,Products!$A:$A,$A13,Products!$C:$C,"Cross-sell")</f>
+        <f aca="false">SUMIFS(Products!$G:$G,Products!$A:$A,$A13,Products!$C:$C,"Upsell")</f>
         <v>0</v>
       </c>
       <c r="E13" s="23" t="n">
-        <f aca="false">SUMIFS(Products!$P:$P,Products!$A:$A,$A13,Products!$O:$O,"Regrettable")</f>
+        <f aca="false">SUMIFS(Products!$G:$G,Products!$A:$A,$A13,Products!$C:$C,"Downgrade")-SUMIFS(Products!$F:$F,Products!$A:$A,$A13,Products!$C:$C,"Churn")</f>
         <v>-8000</v>
       </c>
-      <c r="F13" s="23" t="n">
-        <f aca="false">SUMIFS(Products!$P:$P,Products!$A:$A,$A13,Products!$O:$O,"Non-regrettable")</f>
-        <v>0</v>
-      </c>
-      <c r="G13" s="23" t="n">
-        <f aca="false">-F13</f>
-        <v>-0</v>
+      <c r="F13" s="18" t="s">
+        <v>201</v>
+      </c>
+      <c r="G13" s="18" t="s">
+        <v>203</v>
       </c>
       <c r="H13" s="23" t="n">
-        <f aca="false">MIN(0,C13-(SUMIFS(Products!$L:$L,Products!$A:$A,$A13)-SUMIFS(Products!$I:$I,Products!$A:$A,$A13)))</f>
+        <f aca="false">MIN(0,C13-(SUMIFS(Products!$J:$J,Products!$A:$A,$A13)-SUMIFS(Products!$K:$K,Products!$A:$A,$A13)))</f>
         <v>0</v>
       </c>
       <c r="I13" s="23" t="n">
-        <f aca="false">SUMIFS(Products!$I:$I,Products!$A:$A,$A13)</f>
+        <f aca="false">SUMIFS(Products!$K:$K,Products!$A:$A,$A13)</f>
         <v>32000</v>
       </c>
       <c r="J13" s="23" t="n">
@@ -5228,7 +5175,7 @@
       </c>
       <c r="C14" s="24" t="n">
         <f aca="false">SUM(C4:C13)</f>
-        <v>13200</v>
+        <v>14500</v>
       </c>
       <c r="D14" s="24" t="n">
         <f aca="false">SUM(D4:D13)</f>
@@ -5238,41 +5185,33 @@
         <f aca="false">SUM(E4:E13)</f>
         <v>-23000</v>
       </c>
-      <c r="F14" s="24" t="n">
-        <f aca="false">SUM(F4:F13)</f>
-        <v>0</v>
-      </c>
-      <c r="G14" s="24" t="n">
-        <f aca="false">SUM(G4:G13)</f>
-        <v>0</v>
-      </c>
       <c r="H14" s="24" t="n">
         <f aca="false">SUM(H4:H13)</f>
         <v>-2736</v>
       </c>
       <c r="I14" s="24" t="n">
         <f aca="false">SUM(I4:I13)</f>
-        <v>360664</v>
+        <v>361964</v>
       </c>
       <c r="J14" s="24" t="n">
         <f aca="false">SUM(J4:J13)</f>
-        <v>-14336</v>
+        <v>-13036</v>
       </c>
       <c r="K14" s="33" t="n">
         <f aca="false">IF(B14=0,0,J14/B14)</f>
-        <v>-0.0382293333333333</v>
+        <v>-0.0347626666666667</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="34" t="s">
-        <v>200</v>
+        <v>204</v>
       </c>
       <c r="E15" s="35" t="n">
-        <f aca="false">E14</f>
+        <f aca="false">SUMIFS(E4:E13,F4:F13,"Regrettable")</f>
         <v>-23000</v>
       </c>
       <c r="F15" s="35" t="n">
-        <f aca="false">F14</f>
+        <f aca="false">SUMIFS(E4:E13,F4:F13,"Non-regrettable")</f>
         <v>0</v>
       </c>
       <c r="H15" s="35" t="n">
@@ -5280,16 +5219,45 @@
         <v>-2736</v>
       </c>
     </row>
+    <row r="16" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="2" t="s">
+        <v>205</v>
+      </c>
+      <c r="B16" s="31" t="s">
+        <v>206</v>
+      </c>
+      <c r="C16" s="31"/>
+      <c r="D16" s="31"/>
+      <c r="E16" s="31"/>
+      <c r="F16" s="31"/>
+      <c r="G16" s="31"/>
+      <c r="H16" s="31"/>
+      <c r="I16" s="31"/>
+      <c r="J16" s="31"/>
+      <c r="K16" s="31"/>
+    </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="12" t="s">
-        <v>201</v>
+      <c r="A17" s="2" t="s">
+        <v>207</v>
       </c>
       <c r="B17" s="12" t="str">
+        <f aca="false">COUNTIFS(E4:E13,"&lt;0",F4:F13,"")&amp;" opportunities with churn but no category"</f>
+        <v>0 opportunities with churn but no category</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="12" t="s">
+        <v>208</v>
+      </c>
+      <c r="B18" s="12" t="str">
         <f aca="false">IF(ABS(I14-Pipeline!S15)&lt;1,"OK","MISMATCH")</f>
         <v>OK</v>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B16:K16"/>
+  </mergeCells>
   <conditionalFormatting sqref="J4:K14">
     <cfRule type="cellIs" priority="2" operator="greaterThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="4">
       <formula>0</formula>
@@ -5303,11 +5271,17 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F4:F14">
-    <cfRule type="cellIs" priority="5" operator="lessThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="2">
-      <formula>0</formula>
+  <conditionalFormatting sqref="F4:F13">
+    <cfRule type="expression" priority="5" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
+      <formula>AND(E4&lt;0,F4="")</formula>
     </cfRule>
   </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="F4:F13" type="list">
+      <formula1>"Regrettable,Non-regrettable"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+  </dataValidations>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -5337,7 +5311,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>202</v>
+        <v>209</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5348,7 +5322,7 @@
         <v>56</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>203</v>
+        <v>210</v>
       </c>
       <c r="D3" s="6" t="s">
         <v>47</v>
@@ -5357,27 +5331,27 @@
         <v>61</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>204</v>
+        <v>211</v>
       </c>
       <c r="G3" s="6" t="s">
-        <v>205</v>
+        <v>212</v>
       </c>
       <c r="H3" s="6" t="s">
-        <v>206</v>
+        <v>213</v>
       </c>
       <c r="I3" s="6" t="s">
-        <v>207</v>
+        <v>214</v>
       </c>
       <c r="J3" s="6" t="s">
-        <v>194</v>
+        <v>215</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="15" t="s">
-        <v>208</v>
+        <v>216</v>
       </c>
       <c r="B4" s="15" t="s">
-        <v>209</v>
+        <v>217</v>
       </c>
       <c r="C4" s="15" t="n">
         <f aca="false">COUNTIFS(Pipeline!$M$5:$M$14,B4)</f>
@@ -5408,16 +5382,16 @@
         <v>21000</v>
       </c>
       <c r="J4" s="23" t="n">
-        <f aca="false">SUMPRODUCT((TEXT(Pipeline!$C$5:$C$14,"yyyy-mm")=B4)*'Opp summary'!$E$4:$E$13)</f>
+        <f aca="false">SUMPRODUCT((TEXT(Pipeline!$C$5:$C$14,"yyyy-mm")=B4)*('Opp summary'!$F$4:$F$13="Regrettable")*'Opp summary'!$E$4:$E$13)</f>
         <v>0</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="15" t="s">
-        <v>208</v>
+        <v>216</v>
       </c>
       <c r="B5" s="15" t="s">
-        <v>210</v>
+        <v>218</v>
       </c>
       <c r="C5" s="15" t="n">
         <f aca="false">COUNTIFS(Pipeline!$M$5:$M$14,B5)</f>
@@ -5429,11 +5403,11 @@
       </c>
       <c r="E5" s="23" t="n">
         <f aca="false">SUMIFS(Pipeline!$S$5:$S$14,Pipeline!$M$5:$M$14,B5)</f>
-        <v>174650</v>
+        <v>175950</v>
       </c>
       <c r="F5" s="23" t="n">
         <f aca="false">SUMIFS(Pipeline!$T$5:$T$14,Pipeline!$M$5:$M$14,B5)</f>
-        <v>67530</v>
+        <v>68310</v>
       </c>
       <c r="G5" s="23" t="n">
         <f aca="false">SUMIFS(Pipeline!$T$5:$T$14,Pipeline!$M$5:$M$14,B5,Pipeline!$U$5:$U$14,"On time")</f>
@@ -5441,23 +5415,23 @@
       </c>
       <c r="H5" s="23" t="n">
         <f aca="false">SUMIFS(Pipeline!$T$5:$T$14,Pipeline!$M$5:$M$14,B5,Pipeline!$U$5:$U$14,"Late")</f>
-        <v>39600</v>
+        <v>40380</v>
       </c>
       <c r="I5" s="23" t="n">
         <f aca="false">SUMIFS(Pipeline!$B$5:$B$14,Pipeline!$M$5:$M$14,B5,Pipeline!$L$5:$L$14,"YES")</f>
         <v>0</v>
       </c>
       <c r="J5" s="23" t="n">
-        <f aca="false">SUMPRODUCT((TEXT(Pipeline!$C$5:$C$14,"yyyy-mm")=B5)*'Opp summary'!$E$4:$E$13)</f>
+        <f aca="false">SUMPRODUCT((TEXT(Pipeline!$C$5:$C$14,"yyyy-mm")=B5)*('Opp summary'!$F$4:$F$13="Regrettable")*'Opp summary'!$E$4:$E$13)</f>
         <v>-15000</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="15" t="s">
-        <v>208</v>
+        <v>216</v>
       </c>
       <c r="B6" s="15" t="s">
-        <v>211</v>
+        <v>219</v>
       </c>
       <c r="C6" s="15" t="n">
         <f aca="false">COUNTIFS(Pipeline!$M$5:$M$14,B6)</f>
@@ -5488,13 +5462,13 @@
         <v>0</v>
       </c>
       <c r="J6" s="23" t="n">
-        <f aca="false">SUMPRODUCT((TEXT(Pipeline!$C$5:$C$14,"yyyy-mm")=B6)*'Opp summary'!$E$4:$E$13)</f>
+        <f aca="false">SUMPRODUCT((TEXT(Pipeline!$C$5:$C$14,"yyyy-mm")=B6)*('Opp summary'!$F$4:$F$13="Regrettable")*'Opp summary'!$E$4:$E$13)</f>
         <v>-8000</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>212</v>
+        <v>220</v>
       </c>
       <c r="C7" s="2" t="n">
         <f aca="false">SUM(C4:C6)</f>
@@ -5506,11 +5480,11 @@
       </c>
       <c r="E7" s="24" t="n">
         <f aca="false">SUM(E4:E6)</f>
-        <v>360664</v>
+        <v>361964</v>
       </c>
       <c r="F7" s="24" t="n">
         <f aca="false">SUM(F4:F6)</f>
-        <v>137492</v>
+        <v>138272</v>
       </c>
       <c r="G7" s="24" t="n">
         <f aca="false">SUM(G4:G6)</f>
@@ -5518,7 +5492,7 @@
       </c>
       <c r="H7" s="24" t="n">
         <f aca="false">SUM(H4:H6)</f>
-        <v>63225</v>
+        <v>64005</v>
       </c>
       <c r="I7" s="24" t="n">
         <f aca="false">SUM(I4:I6)</f>
@@ -5566,12 +5540,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>213</v>
+        <v>221</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>214</v>
+        <v>222</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5579,30 +5553,30 @@
         <v>34</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>215</v>
+        <v>223</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>216</v>
+        <v>224</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>217</v>
+        <v>225</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>218</v>
+        <v>226</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>219</v>
+        <v>227</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>220</v>
+        <v>228</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>221</v>
+        <v>229</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>222</v>
+        <v>230</v>
       </c>
       <c r="B5" s="36" t="n">
         <v>0</v>
@@ -5620,7 +5594,7 @@
         <v>0</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>223</v>
+        <v>231</v>
       </c>
       <c r="H5" s="15" t="s">
         <v>71</v>
@@ -5646,7 +5620,7 @@
         <v>0.35</v>
       </c>
       <c r="G6" s="8" t="s">
-        <v>224</v>
+        <v>232</v>
       </c>
       <c r="H6" s="15" t="s">
         <v>71</v>
@@ -5672,7 +5646,7 @@
         <v>0.5</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>225</v>
+        <v>233</v>
       </c>
       <c r="H7" s="15" t="s">
         <v>71</v>
@@ -5698,7 +5672,7 @@
         <v>0.55</v>
       </c>
       <c r="G8" s="8" t="s">
-        <v>226</v>
+        <v>234</v>
       </c>
       <c r="H8" s="15" t="s">
         <v>71</v>
@@ -5724,7 +5698,7 @@
         <v>0.6</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>227</v>
+        <v>235</v>
       </c>
       <c r="H9" s="15" t="s">
         <v>71</v>
@@ -5750,7 +5724,7 @@
         <v>0.75</v>
       </c>
       <c r="G10" s="8" t="s">
-        <v>228</v>
+        <v>236</v>
       </c>
       <c r="H10" s="15" t="s">
         <v>71</v>
@@ -5776,7 +5750,7 @@
         <v>0.9</v>
       </c>
       <c r="G11" s="8" t="s">
-        <v>229</v>
+        <v>237</v>
       </c>
       <c r="H11" s="15" t="s">
         <v>71</v>
@@ -5784,7 +5758,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>230</v>
+        <v>238</v>
       </c>
       <c r="B12" s="36" t="n">
         <v>1</v>
@@ -5802,7 +5776,7 @@
         <v>1</v>
       </c>
       <c r="G12" s="8" t="s">
-        <v>231</v>
+        <v>239</v>
       </c>
       <c r="H12" s="15" t="s">
         <v>71</v>
@@ -5810,7 +5784,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
-        <v>232</v>
+        <v>240</v>
       </c>
       <c r="B13" s="36" t="n">
         <v>0</v>
@@ -5828,10 +5802,10 @@
         <v>0</v>
       </c>
       <c r="G13" s="8" t="s">
-        <v>233</v>
+        <v>241</v>
       </c>
       <c r="H13" s="15" t="s">
-        <v>234</v>
+        <v>242</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5854,7 +5828,7 @@
         <v>0.9</v>
       </c>
       <c r="G14" s="8" t="s">
-        <v>235</v>
+        <v>243</v>
       </c>
       <c r="H14" s="15" t="s">
         <v>90</v>
@@ -5880,7 +5854,7 @@
         <v>0.8</v>
       </c>
       <c r="G15" s="8" t="s">
-        <v>236</v>
+        <v>244</v>
       </c>
       <c r="H15" s="15" t="s">
         <v>90</v>
@@ -5906,7 +5880,7 @@
         <v>0.5</v>
       </c>
       <c r="G16" s="8" t="s">
-        <v>237</v>
+        <v>245</v>
       </c>
       <c r="H16" s="15" t="s">
         <v>90</v>
@@ -5914,7 +5888,7 @@
     </row>
     <row r="17" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="s">
-        <v>238</v>
+        <v>246</v>
       </c>
       <c r="B17" s="36" t="n">
         <v>0.5</v>
@@ -5932,7 +5906,7 @@
         <v>0.8</v>
       </c>
       <c r="G17" s="8" t="s">
-        <v>239</v>
+        <v>247</v>
       </c>
       <c r="H17" s="15" t="s">
         <v>90</v>
@@ -5940,7 +5914,7 @@
     </row>
     <row r="18" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="7" t="s">
-        <v>240</v>
+        <v>248</v>
       </c>
       <c r="B18" s="36" t="n">
         <v>0</v>
@@ -5958,7 +5932,7 @@
         <v>0.1</v>
       </c>
       <c r="G18" s="8" t="s">
-        <v>241</v>
+        <v>249</v>
       </c>
       <c r="H18" s="15" t="s">
         <v>90</v>
@@ -5966,7 +5940,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="s">
-        <v>242</v>
+        <v>250</v>
       </c>
       <c r="B19" s="36" t="n">
         <v>1</v>
@@ -5984,7 +5958,7 @@
         <v>1</v>
       </c>
       <c r="G19" s="8" t="s">
-        <v>243</v>
+        <v>251</v>
       </c>
       <c r="H19" s="15" t="s">
         <v>90</v>
@@ -5995,7 +5969,7 @@
         <v>15</v>
       </c>
       <c r="B21" s="31" t="s">
-        <v>244</v>
+        <v>252</v>
       </c>
       <c r="C21" s="31"/>
       <c r="D21" s="31"/>
@@ -6024,7 +5998,7 @@
         <v>11</v>
       </c>
       <c r="B25" s="31" t="s">
-        <v>245</v>
+        <v>253</v>
       </c>
       <c r="C25" s="31"/>
       <c r="D25" s="31"/>
@@ -6090,95 +6064,95 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>246</v>
+        <v>254</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="s">
-        <v>247</v>
+        <v>255</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>248</v>
+        <v>256</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>249</v>
+        <v>257</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>250</v>
+        <v>258</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>251</v>
+        <v>259</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>252</v>
+        <v>260</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>253</v>
+        <v>261</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>254</v>
+        <v>262</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>255</v>
+        <v>263</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>256</v>
+        <v>264</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>257</v>
+        <v>265</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>258</v>
+        <v>266</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>259</v>
+        <v>267</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>260</v>
+        <v>268</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>261</v>
+        <v>269</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>262</v>
+        <v>270</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>263</v>
+        <v>271</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="8" t="s">
-        <v>264</v>
+        <v>272</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>265</v>
+        <v>273</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>266</v>
+        <v>274</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="8" t="s">
-        <v>267</v>
+        <v>275</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>268</v>
+        <v>276</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>269</v>
+        <v>277</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Product lines are maintained by the Renewals Manager, not the CSM
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CVAHSCDuy4tEBaMUUSRsNB
</commit_message>
<xml_diff>
--- a/n8n-renewals-challenge/renewal_tracker.xlsx
+++ b/n8n-renewals-challenge/renewal_tracker.xlsx
@@ -111,7 +111,7 @@
     <t xml:space="preserve">Products</t>
   </si>
   <si>
-    <t xml:space="preserve">The CSM only sets the line type (Renewal / Upsell / Downgrade / Churn) and the new numbers. Original ARR, uplift, list price, new ARR and Δ (green/red) recalculate. Upsell lines open a linked Upsell opportunity.</t>
+    <t xml:space="preserve">The Renewals Manager only sets the line type (Renewal / Upsell / Downgrade / Churn) and the new numbers. Original ARR, uplift, list price, new ARR and Δ (green/red) recalculate. Upsell lines open a linked Upsell opportunity.</t>
   </si>
   <si>
     <t xml:space="preserve">Churn</t>
@@ -516,10 +516,10 @@
     <t xml:space="preserve">Uplift from this week's actions</t>
   </si>
   <si>
-    <t xml:space="preserve">Opportunity products: the CSM only sets the line type and the new numbers; everything else recalculates</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CSM inputs (yellow): line type and change at list. Original ARR comes from the closed renewal. Uplift is automatic: 5% on every renewal line in year 1. On multi-year deals paid upfront the price is locked from year 2 (no further uplift); paid annually, 5% applies every year. An Upsell line opens a linked Upsell opportunity so expansion is forecast separately. Churn category and reason live on the opportunity.</t>
+    <t xml:space="preserve">Opportunity products: the Renewals Manager only sets the line type and the new numbers; everything else recalculates</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Renewals Manager inputs (yellow): line type and change at list. Original ARR comes from the closed renewal. Uplift is automatic: 5% on every renewal line in year 1. On multi-year deals paid upfront the price is locked from year 2 (no further uplift); paid annually, 5% applies every year. An Upsell line opens a linked Upsell opportunity so expansion is forecast separately. Churn category and reason live on the opportunity.</t>
   </si>
   <si>
     <t xml:space="preserve">Opportunity</t>

</xml_diff>

<commit_message>
Treat renewal ARR as uplift-included across tracker, docs, one-pager and web page
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CVAHSCDuy4tEBaMUUSRsNB
</commit_message>
<xml_diff>
--- a/n8n-renewals-challenge/renewal_tracker.xlsx
+++ b/n8n-renewals-challenge/renewal_tracker.xlsx
@@ -111,7 +111,7 @@
     <t xml:space="preserve">Products</t>
   </si>
   <si>
-    <t xml:space="preserve">The Renewals Manager only sets the line type (Renewal / Upsell / Downgrade / Churn) and the new numbers. Original ARR, uplift, list price, new ARR and Δ (green/red) recalculate. Upsell lines open a linked Upsell opportunity.</t>
+    <t xml:space="preserve">The Renewals Manager only sets the line type (Renewal / Upsell / Downgrade / Churn) and the new numbers. Original ARR, list price, new ARR and Δ (green/red) recalculate; the renewal value already includes the uplift. Upsell lines open a linked Upsell opportunity.</t>
   </si>
   <si>
     <t xml:space="preserve">Churn</t>
@@ -306,7 +306,7 @@
     <t xml:space="preserve">No quote sent; signatory unknown; signed 3 days late last year</t>
   </si>
   <si>
-    <t xml:space="preserve">Quote and order form out today at €50.4k for e-signature; champion confirms signatory and PO need; signature booked for 27 Oct.</t>
+    <t xml:space="preserve">Quote and order form out today at €48k for e-signature; champion confirms signatory and PO need; signature booked for 27 Oct.</t>
   </si>
   <si>
     <t xml:space="preserve">Biggest near-term ARR, 9 days out, no quote, signed 3 days late last year. One hour of work removes most of the risk.</t>
@@ -330,7 +330,7 @@
     <t xml:space="preserve">Card expired; billing contact unknown</t>
   </si>
   <si>
-    <t xml:space="preserve">CSM gets the billing contact today; I send a secure card-update link or switch to invoice; Finance holds dunning. Renews at €27.3k with the contractual 5% uplift.</t>
+    <t xml:space="preserve">CSM gets the billing contact today; I send a secure card-update link or switch to invoice; Finance holds dunning. Renews at €26k (renewal value).</t>
   </si>
   <si>
     <t xml:space="preserve">Auto-renewal fails in 13 days on an expired card: involuntary churn on a green account.</t>
@@ -426,7 +426,7 @@
     <t xml:space="preserve">Close to execution cap</t>
   </si>
   <si>
-    <t xml:space="preserve">CSM usage review; quote like-for-like (€36.75k) and open a linked Upsell opportunity for the next execution tier.</t>
+    <t xml:space="preserve">CSM usage review; quote like-for-like (€35k) and open a linked Upsell opportunity for the next execution tier.</t>
   </si>
   <si>
     <t xml:space="preserve">Usage +40%, near the execution cap: expansion, and a throttling risk.</t>
@@ -504,7 +504,7 @@
     <t xml:space="preserve">Gross retention (base less regrettable churn and concessions)</t>
   </si>
   <si>
-    <t xml:space="preserve">Net retention (new ARR / base, incl. 5% uplift)</t>
+    <t xml:space="preserve">Net retention (new ARR / base)</t>
   </si>
   <si>
     <t xml:space="preserve">Weighted today (statuses from what we know)</t>
@@ -513,13 +513,13 @@
     <t xml:space="preserve">Weighted by 30 Oct, if this week's actions land</t>
   </si>
   <si>
-    <t xml:space="preserve">Uplift from this week's actions</t>
+    <t xml:space="preserve">Gain from this week's actions</t>
   </si>
   <si>
     <t xml:space="preserve">Opportunity products: the Renewals Manager only sets the line type and the new numbers; everything else recalculates</t>
   </si>
   <si>
-    <t xml:space="preserve">Renewals Manager inputs (yellow): line type and change at list. Original ARR comes from the closed renewal. Uplift is automatic: 5% on every renewal line in year 1. On multi-year deals paid upfront the price is locked from year 2 (no further uplift); paid annually, 5% applies every year. An Upsell line opens a linked Upsell opportunity so expansion is forecast separately. Churn category and reason live on the opportunity.</t>
+    <t xml:space="preserve">Renewals Manager inputs (yellow): line type and change at list. Original ARR is the renewal value and already includes the 5% uplift (applied when the renewal opportunity is created), so nothing is added on top. On multi-year deals paid upfront the price is locked from year 2 (no further uplift); paid annually, 5% applies every year. An Upsell line opens a linked Upsell opportunity so expansion is forecast separately. Churn category and reason live on the opportunity.</t>
   </si>
   <si>
     <t xml:space="preserve">Opportunity</t>
@@ -543,7 +543,7 @@
     <t xml:space="preserve">Change at list (€)</t>
   </si>
   <si>
-    <t xml:space="preserve">Uplift % (yr 1)</t>
+    <t xml:space="preserve">Extra uplift %</t>
   </si>
   <si>
     <t xml:space="preserve">Discount %</t>
@@ -576,7 +576,7 @@
     <t xml:space="preserve">Annual</t>
   </si>
   <si>
-    <t xml:space="preserve">Quote of 1 Sep includes 5% uplift</t>
+    <t xml:space="preserve">Quote of 1 Sep at the renewal value</t>
   </si>
   <si>
     <t xml:space="preserve">n8n Cloud Enterprise</t>
@@ -585,7 +585,7 @@
     <t xml:space="preserve">Usage +12%: check cap next quarter</t>
   </si>
   <si>
-    <t xml:space="preserve">Uplift is contractual (annual notice in January)</t>
+    <t xml:space="preserve">Renewal value; the contractual uplift is already in it</t>
   </si>
   <si>
     <t xml:space="preserve">n8n Enterprise (self-hosted)</t>
@@ -600,7 +600,7 @@
     <t xml:space="preserve">n8n Enterprise</t>
   </si>
   <si>
-    <t xml:space="preserve">Placeholder until Part 2 is agreed</t>
+    <t xml:space="preserve">Ramp year 1: 10% off; year 2 €35,910</t>
   </si>
   <si>
     <t xml:space="preserve">Bill to new legal entity</t>
@@ -780,7 +780,7 @@
     <t xml:space="preserve">Both</t>
   </si>
   <si>
-    <t xml:space="preserve">Valid payment method, correct billing entity, uplift notice sent, usage stable or growing. (Overdue = payment failed: move to Billing blocker.)</t>
+    <t xml:space="preserve">Valid payment method, correct billing entity, usage stable or growing. (Overdue = payment failed: move to Billing blocker.)</t>
   </si>
   <si>
     <t xml:space="preserve">Expired card, wrong legal entity, PO required. Admin fix, usually recoverable.</t>
@@ -1747,7 +1747,7 @@
       </c>
       <c r="H5" s="8" t="str">
         <f aca="false">INDEX(Pipeline!$V$5:$V$14,MATCH($A5,Pipeline!$Y$5:$Y$14,0))&amp;""</f>
-        <v>Quote and order form out today at €50.4k for e-signature; champion confirms signatory and PO need; signature booked for 27 Oct.</v>
+        <v>Quote and order form out today at €48k for e-signature; champion confirms signatory and PO need; signature booked for 27 Oct.</v>
       </c>
       <c r="I5" s="8" t="str">
         <f aca="false">INDEX(Pipeline!$W$5:$W$14,MATCH($A5,Pipeline!$Y$5:$Y$14,0))</f>
@@ -1845,7 +1845,7 @@
       </c>
       <c r="H7" s="8" t="str">
         <f aca="false">INDEX(Pipeline!$V$5:$V$14,MATCH($A7,Pipeline!$Y$5:$Y$14,0))&amp;""</f>
-        <v>CSM gets the billing contact today; I send a secure card-update link or switch to invoice; Finance holds dunning. Renews at €27.3k with the contractual 5% uplift.</v>
+        <v>CSM gets the billing contact today; I send a secure card-update link or switch to invoice; Finance holds dunning. Renews at €26k (renewal value).</v>
       </c>
       <c r="I7" s="8" t="str">
         <f aca="false">INDEX(Pipeline!$W$5:$W$14,MATCH($A7,Pipeline!$Y$5:$Y$14,0))</f>
@@ -2090,7 +2090,7 @@
       </c>
       <c r="H12" s="8" t="str">
         <f aca="false">INDEX(Pipeline!$V$5:$V$14,MATCH($A12,Pipeline!$Y$5:$Y$14,0))&amp;""</f>
-        <v>CSM usage review; quote like-for-like (€36.75k) and open a linked Upsell opportunity for the next execution tier.</v>
+        <v>CSM usage review; quote like-for-like (€35k) and open a linked Upsell opportunity for the next execution tier.</v>
       </c>
       <c r="I12" s="8" t="str">
         <f aca="false">INDEX(Pipeline!$W$5:$W$14,MATCH($A12,Pipeline!$Y$5:$Y$14,0))</f>
@@ -2491,11 +2491,11 @@
       </c>
       <c r="S5" s="23" t="n">
         <f aca="false">SUMIFS(Products!$K:$K,Products!$A:$A,A5)</f>
-        <v>22050</v>
+        <v>21000</v>
       </c>
       <c r="T5" s="23" t="n">
         <f aca="false">S5*R5</f>
-        <v>11025</v>
+        <v>10500</v>
       </c>
       <c r="U5" s="15" t="str">
         <f aca="false">IF(G5="Cancelled","Lost",IF(Q5="No","Slips quarter",IF(OR(J5&lt;0,AND(J5&lt;=30,OR(G5="--None--",G5="Not started",G5="Engaging customer",G5="Negotiation",G5="Billing blocker",G5="At risk: before notice deadline",G5="Notice received"))),"Late","On time")))</f>
@@ -2540,7 +2540,7 @@
       </c>
       <c r="AH5" s="23" t="n">
         <f aca="false">S5*AG5</f>
-        <v>15435</v>
+        <v>14700</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2609,11 +2609,11 @@
       </c>
       <c r="S6" s="23" t="n">
         <f aca="false">SUMIFS(Products!$K:$K,Products!$A:$A,A6)</f>
-        <v>50400</v>
+        <v>48000</v>
       </c>
       <c r="T6" s="23" t="n">
         <f aca="false">S6*R6</f>
-        <v>12600</v>
+        <v>12000</v>
       </c>
       <c r="U6" s="15" t="str">
         <f aca="false">IF(G6="Cancelled","Lost",IF(Q6="No","Slips quarter",IF(OR(J6&lt;0,AND(J6&lt;=30,OR(G6="--None--",G6="Not started",G6="Engaging customer",G6="Negotiation",G6="Billing blocker",G6="At risk: before notice deadline",G6="Notice received"))),"Late","On time")))</f>
@@ -2656,7 +2656,7 @@
       </c>
       <c r="AH6" s="23" t="n">
         <f aca="false">S6*AG6</f>
-        <v>47880</v>
+        <v>45600</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2725,11 +2725,11 @@
       </c>
       <c r="S7" s="23" t="n">
         <f aca="false">SUMIFS(Products!$K:$K,Products!$A:$A,A7)</f>
-        <v>27300</v>
+        <v>26000</v>
       </c>
       <c r="T7" s="23" t="n">
         <f aca="false">S7*R7</f>
-        <v>16380</v>
+        <v>15600</v>
       </c>
       <c r="U7" s="15" t="str">
         <f aca="false">IF(G7="Cancelled","Lost",IF(Q7="No","Slips quarter",IF(OR(J7&lt;0,AND(J7&lt;=30,OR(G7="--None--",G7="Not started",G7="Engaging customer",G7="Negotiation",G7="Billing blocker",G7="At risk: before notice deadline",G7="Notice received"))),"Late","On time")))</f>
@@ -2774,7 +2774,7 @@
       </c>
       <c r="AH7" s="23" t="n">
         <f aca="false">S7*AG7</f>
-        <v>26481</v>
+        <v>25220</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2963,11 +2963,11 @@
       </c>
       <c r="S9" s="23" t="n">
         <f aca="false">SUMIFS(Products!$K:$K,Products!$A:$A,A9)</f>
-        <v>33264</v>
+        <v>32400</v>
       </c>
       <c r="T9" s="23" t="n">
         <f aca="false">S9*R9</f>
-        <v>16632</v>
+        <v>16200</v>
       </c>
       <c r="U9" s="15" t="str">
         <f aca="false">IF(G9="Cancelled","Lost",IF(Q9="No","Slips quarter",IF(OR(J9&lt;0,AND(J9&lt;=30,OR(G9="--None--",G9="Not started",G9="Engaging customer",G9="Negotiation",G9="Billing blocker",G9="At risk: before notice deadline",G9="Notice received"))),"Late","On time")))</f>
@@ -3010,7 +3010,7 @@
       </c>
       <c r="AH9" s="23" t="n">
         <f aca="false">S9*AG9</f>
-        <v>16632</v>
+        <v>16200</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3079,11 +3079,11 @@
       </c>
       <c r="S10" s="23" t="n">
         <f aca="false">SUMIFS(Products!$K:$K,Products!$A:$A,A10)</f>
-        <v>52500</v>
+        <v>50000</v>
       </c>
       <c r="T10" s="23" t="n">
         <f aca="false">S10*R10</f>
-        <v>21000</v>
+        <v>20000</v>
       </c>
       <c r="U10" s="15" t="str">
         <f aca="false">IF(G10="Cancelled","Lost",IF(Q10="No","Slips quarter",IF(OR(J10&lt;0,AND(J10&lt;=30,OR(G10="--None--",G10="Not started",G10="Engaging customer",G10="Negotiation",G10="Billing blocker",G10="At risk: before notice deadline",G10="Notice received"))),"Late","On time")))</f>
@@ -3128,7 +3128,7 @@
       </c>
       <c r="AH10" s="23" t="n">
         <f aca="false">S10*AG10</f>
-        <v>39375</v>
+        <v>37500</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3197,11 +3197,11 @@
       </c>
       <c r="S11" s="23" t="n">
         <f aca="false">SUMIFS(Products!$K:$K,Products!$A:$A,A11)</f>
-        <v>29400</v>
+        <v>28000</v>
       </c>
       <c r="T11" s="23" t="n">
         <f aca="false">S11*R11</f>
-        <v>20580</v>
+        <v>19600</v>
       </c>
       <c r="U11" s="15" t="str">
         <f aca="false">IF(G11="Cancelled","Lost",IF(Q11="No","Slips quarter",IF(OR(J11&lt;0,AND(J11&lt;=30,OR(G11="--None--",G11="Not started",G11="Engaging customer",G11="Negotiation",G11="Billing blocker",G11="At risk: before notice deadline",G11="Notice received"))),"Late","On time")))</f>
@@ -3246,7 +3246,7 @@
       </c>
       <c r="AH11" s="23" t="n">
         <f aca="false">S11*AG11</f>
-        <v>28518</v>
+        <v>27160</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3315,11 +3315,11 @@
       </c>
       <c r="S12" s="23" t="n">
         <f aca="false">SUMIFS(Products!$K:$K,Products!$A:$A,A12)</f>
-        <v>36750</v>
+        <v>35000</v>
       </c>
       <c r="T12" s="23" t="n">
         <f aca="false">S12*R12</f>
-        <v>7350</v>
+        <v>7000</v>
       </c>
       <c r="U12" s="15" t="str">
         <f aca="false">IF(G12="Cancelled","Lost",IF(Q12="No","Slips quarter",IF(OR(J12&lt;0,AND(J12&lt;=30,OR(G12="--None--",G12="Not started",G12="Engaging customer",G12="Negotiation",G12="Billing blocker",G12="At risk: before notice deadline",G12="Notice received"))),"Late","On time")))</f>
@@ -3362,7 +3362,7 @@
       </c>
       <c r="AH12" s="23" t="n">
         <f aca="false">S12*AG12</f>
-        <v>27562.5</v>
+        <v>26250</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3431,11 +3431,11 @@
       </c>
       <c r="S13" s="23" t="n">
         <f aca="false">SUMIFS(Products!$K:$K,Products!$A:$A,A13)</f>
-        <v>48300</v>
+        <v>46000</v>
       </c>
       <c r="T13" s="23" t="n">
         <f aca="false">S13*R13</f>
-        <v>16905</v>
+        <v>16100</v>
       </c>
       <c r="U13" s="15" t="str">
         <f aca="false">IF(G13="Cancelled","Lost",IF(Q13="No","Slips quarter",IF(OR(J13&lt;0,AND(J13&lt;=30,OR(G13="--None--",G13="Not started",G13="Engaging customer",G13="Negotiation",G13="Billing blocker",G13="At risk: before notice deadline",G13="Notice received"))),"Late","On time")))</f>
@@ -3478,7 +3478,7 @@
       </c>
       <c r="AH13" s="23" t="n">
         <f aca="false">S13*AG13</f>
-        <v>33810</v>
+        <v>32200</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3609,15 +3609,15 @@
       </c>
       <c r="S15" s="24" t="n">
         <f aca="false">SUM(S5:S14)</f>
-        <v>361964</v>
+        <v>348400</v>
       </c>
       <c r="T15" s="24" t="n">
         <f aca="false">SUM(T5:T14)</f>
-        <v>138272</v>
+        <v>132800</v>
       </c>
       <c r="AH15" s="24" t="n">
         <f aca="false">SUM(AH5:AH14)</f>
-        <v>255993.5</v>
+        <v>245130</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3645,11 +3645,11 @@
       </c>
       <c r="B20" s="23" t="n">
         <f aca="false">SUMIFS(T5:T14,U5:U14,"On time")</f>
-        <v>74267</v>
+        <v>71700</v>
       </c>
       <c r="C20" s="23" t="n">
         <f aca="false">SUMIFS(S5:S14,U5:U14,"On time")</f>
-        <v>179714</v>
+        <v>173400</v>
       </c>
       <c r="D20" s="15" t="str">
         <f aca="false">COUNTIFS(U5:U14,"On time")&amp;" renewals"</f>
@@ -3662,11 +3662,11 @@
       </c>
       <c r="B21" s="23" t="n">
         <f aca="false">SUMIFS(T5:T14,U5:U14,"Late")</f>
-        <v>64005</v>
+        <v>61100</v>
       </c>
       <c r="C21" s="23" t="n">
         <f aca="false">SUMIFS(S5:S14,U5:U14,"Late")</f>
-        <v>182250</v>
+        <v>175000</v>
       </c>
       <c r="D21" s="15" t="str">
         <f aca="false">COUNTIFS(U5:U14,"Late")&amp;" renewals"</f>
@@ -3696,11 +3696,11 @@
       </c>
       <c r="B23" s="27" t="n">
         <f aca="false">SUM(B20:B22)</f>
-        <v>138272</v>
+        <v>132800</v>
       </c>
       <c r="C23" s="23" t="n">
         <f aca="false">SUM(C20:C22)</f>
-        <v>361964</v>
+        <v>348400</v>
       </c>
       <c r="D23" s="28"/>
     </row>
@@ -3733,7 +3733,7 @@
       </c>
       <c r="B27" s="29" t="n">
         <f aca="false">'Opp summary'!H15</f>
-        <v>-2736</v>
+        <v>-3600</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3742,7 +3742,7 @@
       </c>
       <c r="B28" s="30" t="n">
         <f aca="false">(B15+B25+B27)/B15</f>
-        <v>0.931370666666667</v>
+        <v>0.929066666666667</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3751,7 +3751,7 @@
       </c>
       <c r="B29" s="30" t="n">
         <f aca="false">S15/B15</f>
-        <v>0.965237333333333</v>
+        <v>0.929066666666667</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3765,7 +3765,7 @@
       </c>
       <c r="B32" s="27" t="n">
         <f aca="false">T15</f>
-        <v>138272</v>
+        <v>132800</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3774,7 +3774,7 @@
       </c>
       <c r="B33" s="27" t="n">
         <f aca="false">AH15</f>
-        <v>255993.5</v>
+        <v>245130</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3783,7 +3783,7 @@
       </c>
       <c r="B34" s="27" t="n">
         <f aca="false">B33-B32</f>
-        <v>117721.5</v>
+        <v>112330</v>
       </c>
     </row>
   </sheetData>
@@ -4009,27 +4009,26 @@
         <v>0</v>
       </c>
       <c r="H5" s="22" t="n">
-        <f aca="false">IF(C5="Renewal",0.05,0)</f>
-        <v>0.05</v>
+        <v>0</v>
       </c>
       <c r="I5" s="19" t="n">
         <v>0</v>
       </c>
       <c r="J5" s="23" t="n">
         <f aca="false">IF(C5="Churn",0,F5*(1+H5)+G5)</f>
-        <v>22050</v>
+        <v>21000</v>
       </c>
       <c r="K5" s="23" t="n">
         <f aca="false">J5*(1-I5)</f>
-        <v>22050</v>
+        <v>21000</v>
       </c>
       <c r="L5" s="23" t="n">
         <f aca="false">K5-F5</f>
-        <v>1050</v>
+        <v>0</v>
       </c>
       <c r="M5" s="22" t="n">
         <f aca="false">IF(F5=0,"new",L5/F5)</f>
-        <v>0.05</v>
+        <v>0</v>
       </c>
       <c r="N5" s="15" t="str">
         <f aca="false">IF(I5=0,"None",IF(AND(D5&gt;=2,I5&lt;=0.05),"None (multi-year)",IF(I5&lt;=0.12,"Finance","VP Customer Success")))</f>
@@ -4066,27 +4065,26 @@
         <v>0</v>
       </c>
       <c r="H6" s="22" t="n">
-        <f aca="false">IF(C6="Renewal",0.05,0)</f>
-        <v>0.05</v>
+        <v>0</v>
       </c>
       <c r="I6" s="19" t="n">
         <v>0</v>
       </c>
       <c r="J6" s="23" t="n">
         <f aca="false">IF(C6="Churn",0,F6*(1+H6)+G6)</f>
-        <v>50400</v>
+        <v>48000</v>
       </c>
       <c r="K6" s="23" t="n">
         <f aca="false">J6*(1-I6)</f>
-        <v>50400</v>
+        <v>48000</v>
       </c>
       <c r="L6" s="23" t="n">
         <f aca="false">K6-F6</f>
-        <v>2400</v>
+        <v>0</v>
       </c>
       <c r="M6" s="22" t="n">
         <f aca="false">IF(F6=0,"new",L6/F6)</f>
-        <v>0.05</v>
+        <v>0</v>
       </c>
       <c r="N6" s="15" t="str">
         <f aca="false">IF(I6=0,"None",IF(AND(D6&gt;=2,I6&lt;=0.05),"None (multi-year)",IF(I6&lt;=0.12,"Finance","VP Customer Success")))</f>
@@ -4123,27 +4121,26 @@
         <v>0</v>
       </c>
       <c r="H7" s="22" t="n">
-        <f aca="false">IF(C7="Renewal",0.05,0)</f>
-        <v>0.05</v>
+        <v>0</v>
       </c>
       <c r="I7" s="19" t="n">
         <v>0</v>
       </c>
       <c r="J7" s="23" t="n">
         <f aca="false">IF(C7="Churn",0,F7*(1+H7)+G7)</f>
-        <v>27300</v>
+        <v>26000</v>
       </c>
       <c r="K7" s="23" t="n">
         <f aca="false">J7*(1-I7)</f>
-        <v>27300</v>
+        <v>26000</v>
       </c>
       <c r="L7" s="23" t="n">
         <f aca="false">K7-F7</f>
-        <v>1300</v>
+        <v>0</v>
       </c>
       <c r="M7" s="22" t="n">
         <f aca="false">IF(F7=0,"new",L7/F7)</f>
-        <v>0.05</v>
+        <v>0</v>
       </c>
       <c r="N7" s="15" t="str">
         <f aca="false">IF(I7=0,"None",IF(AND(D7&gt;=2,I7&lt;=0.05),"None (multi-year)",IF(I7&lt;=0.12,"Finance","VP Customer Success")))</f>
@@ -4180,7 +4177,6 @@
         <v>-15000</v>
       </c>
       <c r="H8" s="22" t="n">
-        <f aca="false">IF(C8="Renewal",0.05,0)</f>
         <v>0</v>
       </c>
       <c r="I8" s="19" t="n">
@@ -4237,27 +4233,26 @@
         <v>0</v>
       </c>
       <c r="H9" s="22" t="n">
-        <f aca="false">IF(C9="Renewal",0.05,0)</f>
-        <v>0.05</v>
+        <v>0</v>
       </c>
       <c r="I9" s="19" t="n">
-        <v>0.12</v>
+        <v>0.1</v>
       </c>
       <c r="J9" s="23" t="n">
         <f aca="false">IF(C9="Churn",0,F9*(1+H9)+G9)</f>
-        <v>37800</v>
+        <v>36000</v>
       </c>
       <c r="K9" s="23" t="n">
         <f aca="false">J9*(1-I9)</f>
-        <v>33264</v>
+        <v>32400</v>
       </c>
       <c r="L9" s="23" t="n">
         <f aca="false">K9-F9</f>
-        <v>-2736</v>
+        <v>-3600</v>
       </c>
       <c r="M9" s="22" t="n">
         <f aca="false">IF(F9=0,"new",L9/F9)</f>
-        <v>-0.076</v>
+        <v>-0.1</v>
       </c>
       <c r="N9" s="15" t="str">
         <f aca="false">IF(I9=0,"None",IF(AND(D9&gt;=2,I9&lt;=0.05),"None (multi-year)",IF(I9&lt;=0.12,"Finance","VP Customer Success")))</f>
@@ -4294,27 +4289,26 @@
         <v>0</v>
       </c>
       <c r="H10" s="22" t="n">
-        <f aca="false">IF(C10="Renewal",0.05,0)</f>
-        <v>0.05</v>
+        <v>0</v>
       </c>
       <c r="I10" s="19" t="n">
         <v>0</v>
       </c>
       <c r="J10" s="23" t="n">
         <f aca="false">IF(C10="Churn",0,F10*(1+H10)+G10)</f>
-        <v>52500</v>
+        <v>50000</v>
       </c>
       <c r="K10" s="23" t="n">
         <f aca="false">J10*(1-I10)</f>
-        <v>52500</v>
+        <v>50000</v>
       </c>
       <c r="L10" s="23" t="n">
         <f aca="false">K10-F10</f>
-        <v>2500</v>
+        <v>0</v>
       </c>
       <c r="M10" s="22" t="n">
         <f aca="false">IF(F10=0,"new",L10/F10)</f>
-        <v>0.05</v>
+        <v>0</v>
       </c>
       <c r="N10" s="15" t="str">
         <f aca="false">IF(I10=0,"None",IF(AND(D10&gt;=2,I10&lt;=0.05),"None (multi-year)",IF(I10&lt;=0.12,"Finance","VP Customer Success")))</f>
@@ -4349,27 +4343,26 @@
         <v>0</v>
       </c>
       <c r="H11" s="22" t="n">
-        <f aca="false">IF(C11="Renewal",0.05,0)</f>
-        <v>0.05</v>
+        <v>0</v>
       </c>
       <c r="I11" s="19" t="n">
         <v>0</v>
       </c>
       <c r="J11" s="23" t="n">
         <f aca="false">IF(C11="Churn",0,F11*(1+H11)+G11)</f>
-        <v>29400</v>
+        <v>28000</v>
       </c>
       <c r="K11" s="23" t="n">
         <f aca="false">J11*(1-I11)</f>
-        <v>29400</v>
+        <v>28000</v>
       </c>
       <c r="L11" s="23" t="n">
         <f aca="false">K11-F11</f>
-        <v>1400</v>
+        <v>0</v>
       </c>
       <c r="M11" s="22" t="n">
         <f aca="false">IF(F11=0,"new",L11/F11)</f>
-        <v>0.05</v>
+        <v>0</v>
       </c>
       <c r="N11" s="15" t="str">
         <f aca="false">IF(I11=0,"None",IF(AND(D11&gt;=2,I11&lt;=0.05),"None (multi-year)",IF(I11&lt;=0.12,"Finance","VP Customer Success")))</f>
@@ -4406,27 +4399,26 @@
         <v>0</v>
       </c>
       <c r="H12" s="22" t="n">
-        <f aca="false">IF(C12="Renewal",0.05,0)</f>
-        <v>0.05</v>
+        <v>0</v>
       </c>
       <c r="I12" s="19" t="n">
         <v>0</v>
       </c>
       <c r="J12" s="23" t="n">
         <f aca="false">IF(C12="Churn",0,F12*(1+H12)+G12)</f>
-        <v>36750</v>
+        <v>35000</v>
       </c>
       <c r="K12" s="23" t="n">
         <f aca="false">J12*(1-I12)</f>
-        <v>36750</v>
+        <v>35000</v>
       </c>
       <c r="L12" s="23" t="n">
         <f aca="false">K12-F12</f>
-        <v>1750</v>
+        <v>0</v>
       </c>
       <c r="M12" s="22" t="n">
         <f aca="false">IF(F12=0,"new",L12/F12)</f>
-        <v>0.05</v>
+        <v>0</v>
       </c>
       <c r="N12" s="15" t="str">
         <f aca="false">IF(I12=0,"None",IF(AND(D12&gt;=2,I12&lt;=0.05),"None (multi-year)",IF(I12&lt;=0.12,"Finance","VP Customer Success")))</f>
@@ -4463,7 +4455,6 @@
         <v>0</v>
       </c>
       <c r="H13" s="22" t="n">
-        <f aca="false">IF(C13="Renewal",0.05,0)</f>
         <v>0</v>
       </c>
       <c r="I13" s="19" t="n">
@@ -4520,27 +4511,26 @@
         <v>0</v>
       </c>
       <c r="H14" s="22" t="n">
-        <f aca="false">IF(C14="Renewal",0.05,0)</f>
-        <v>0.05</v>
+        <v>0</v>
       </c>
       <c r="I14" s="19" t="n">
         <v>0</v>
       </c>
       <c r="J14" s="23" t="n">
         <f aca="false">IF(C14="Churn",0,F14*(1+H14)+G14)</f>
-        <v>48300</v>
+        <v>46000</v>
       </c>
       <c r="K14" s="23" t="n">
         <f aca="false">J14*(1-I14)</f>
-        <v>48300</v>
+        <v>46000</v>
       </c>
       <c r="L14" s="23" t="n">
         <f aca="false">K14-F14</f>
-        <v>2300</v>
+        <v>0</v>
       </c>
       <c r="M14" s="22" t="n">
         <f aca="false">IF(F14=0,"new",L14/F14)</f>
-        <v>0.05</v>
+        <v>0</v>
       </c>
       <c r="N14" s="15" t="str">
         <f aca="false">IF(I14=0,"None",IF(AND(D14&gt;=2,I14&lt;=0.05),"None (multi-year)",IF(I14&lt;=0.12,"Finance","VP Customer Success")))</f>
@@ -4575,7 +4565,6 @@
         <v>-8000</v>
       </c>
       <c r="H15" s="22" t="n">
-        <f aca="false">IF(C15="Renewal",0.05,0)</f>
         <v>0</v>
       </c>
       <c r="I15" s="19" t="n">
@@ -4623,15 +4612,15 @@
       </c>
       <c r="J17" s="24" t="n">
         <f aca="false">SUM(J5:J15)</f>
-        <v>366500</v>
+        <v>352000</v>
       </c>
       <c r="K17" s="24" t="n">
         <f aca="false">SUM(K5:K15)</f>
-        <v>361964</v>
+        <v>348400</v>
       </c>
       <c r="L17" s="24" t="n">
         <f aca="false">SUM(L5:L15)</f>
-        <v>-13036</v>
+        <v>-26600</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4768,7 +4757,7 @@
       </c>
       <c r="C4" s="23" t="n">
         <f aca="false">SUMPRODUCT((Products!$A$5:$A$200=$A4)*Products!$F$5:$F$200*Products!$H$5:$H$200)</f>
-        <v>1050</v>
+        <v>0</v>
       </c>
       <c r="D4" s="23" t="n">
         <f aca="false">SUMIFS(Products!$G:$G,Products!$A:$A,$A4,Products!$C:$C,"Upsell")</f>
@@ -4786,15 +4775,15 @@
       </c>
       <c r="I4" s="23" t="n">
         <f aca="false">SUMIFS(Products!$K:$K,Products!$A:$A,$A4)</f>
-        <v>22050</v>
+        <v>21000</v>
       </c>
       <c r="J4" s="23" t="n">
         <f aca="false">I4-B4</f>
-        <v>1050</v>
+        <v>0</v>
       </c>
       <c r="K4" s="22" t="n">
         <f aca="false">IF(B4=0,0,J4/B4)</f>
-        <v>0.05</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4808,7 +4797,7 @@
       </c>
       <c r="C5" s="23" t="n">
         <f aca="false">SUMPRODUCT((Products!$A$5:$A$200=$A5)*Products!$F$5:$F$200*Products!$H$5:$H$200)</f>
-        <v>2400</v>
+        <v>0</v>
       </c>
       <c r="D5" s="23" t="n">
         <f aca="false">SUMIFS(Products!$G:$G,Products!$A:$A,$A5,Products!$C:$C,"Upsell")</f>
@@ -4826,15 +4815,15 @@
       </c>
       <c r="I5" s="23" t="n">
         <f aca="false">SUMIFS(Products!$K:$K,Products!$A:$A,$A5)</f>
-        <v>50400</v>
+        <v>48000</v>
       </c>
       <c r="J5" s="23" t="n">
         <f aca="false">I5-B5</f>
-        <v>2400</v>
+        <v>0</v>
       </c>
       <c r="K5" s="22" t="n">
         <f aca="false">IF(B5=0,0,J5/B5)</f>
-        <v>0.05</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4848,7 +4837,7 @@
       </c>
       <c r="C6" s="23" t="n">
         <f aca="false">SUMPRODUCT((Products!$A$5:$A$200=$A6)*Products!$F$5:$F$200*Products!$H$5:$H$200)</f>
-        <v>1300</v>
+        <v>0</v>
       </c>
       <c r="D6" s="23" t="n">
         <f aca="false">SUMIFS(Products!$G:$G,Products!$A:$A,$A6,Products!$C:$C,"Upsell")</f>
@@ -4866,15 +4855,15 @@
       </c>
       <c r="I6" s="23" t="n">
         <f aca="false">SUMIFS(Products!$K:$K,Products!$A:$A,$A6)</f>
-        <v>27300</v>
+        <v>26000</v>
       </c>
       <c r="J6" s="23" t="n">
         <f aca="false">I6-B6</f>
-        <v>1300</v>
+        <v>0</v>
       </c>
       <c r="K6" s="22" t="n">
         <f aca="false">IF(B6=0,0,J6/B6)</f>
-        <v>0.05</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4932,7 +4921,7 @@
       </c>
       <c r="C8" s="23" t="n">
         <f aca="false">SUMPRODUCT((Products!$A$5:$A$200=$A8)*Products!$F$5:$F$200*Products!$H$5:$H$200)</f>
-        <v>1800</v>
+        <v>0</v>
       </c>
       <c r="D8" s="23" t="n">
         <f aca="false">SUMIFS(Products!$G:$G,Products!$A:$A,$A8,Products!$C:$C,"Upsell")</f>
@@ -4946,19 +4935,19 @@
       <c r="G8" s="18"/>
       <c r="H8" s="23" t="n">
         <f aca="false">MIN(0,C8-(SUMIFS(Products!$J:$J,Products!$A:$A,$A8)-SUMIFS(Products!$K:$K,Products!$A:$A,$A8)))</f>
-        <v>-2736</v>
+        <v>-3600</v>
       </c>
       <c r="I8" s="23" t="n">
         <f aca="false">SUMIFS(Products!$K:$K,Products!$A:$A,$A8)</f>
-        <v>33264</v>
+        <v>32400</v>
       </c>
       <c r="J8" s="23" t="n">
         <f aca="false">I8-B8</f>
-        <v>-2736</v>
+        <v>-3600</v>
       </c>
       <c r="K8" s="22" t="n">
         <f aca="false">IF(B8=0,0,J8/B8)</f>
-        <v>-0.076</v>
+        <v>-0.1</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4972,7 +4961,7 @@
       </c>
       <c r="C9" s="23" t="n">
         <f aca="false">SUMPRODUCT((Products!$A$5:$A$200=$A9)*Products!$F$5:$F$200*Products!$H$5:$H$200)</f>
-        <v>2500</v>
+        <v>0</v>
       </c>
       <c r="D9" s="23" t="n">
         <f aca="false">SUMIFS(Products!$G:$G,Products!$A:$A,$A9,Products!$C:$C,"Upsell")</f>
@@ -4990,15 +4979,15 @@
       </c>
       <c r="I9" s="23" t="n">
         <f aca="false">SUMIFS(Products!$K:$K,Products!$A:$A,$A9)</f>
-        <v>52500</v>
+        <v>50000</v>
       </c>
       <c r="J9" s="23" t="n">
         <f aca="false">I9-B9</f>
-        <v>2500</v>
+        <v>0</v>
       </c>
       <c r="K9" s="22" t="n">
         <f aca="false">IF(B9=0,0,J9/B9)</f>
-        <v>0.05</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5012,7 +5001,7 @@
       </c>
       <c r="C10" s="23" t="n">
         <f aca="false">SUMPRODUCT((Products!$A$5:$A$200=$A10)*Products!$F$5:$F$200*Products!$H$5:$H$200)</f>
-        <v>1400</v>
+        <v>0</v>
       </c>
       <c r="D10" s="23" t="n">
         <f aca="false">SUMIFS(Products!$G:$G,Products!$A:$A,$A10,Products!$C:$C,"Upsell")</f>
@@ -5030,15 +5019,15 @@
       </c>
       <c r="I10" s="23" t="n">
         <f aca="false">SUMIFS(Products!$K:$K,Products!$A:$A,$A10)</f>
-        <v>29400</v>
+        <v>28000</v>
       </c>
       <c r="J10" s="23" t="n">
         <f aca="false">I10-B10</f>
-        <v>1400</v>
+        <v>0</v>
       </c>
       <c r="K10" s="22" t="n">
         <f aca="false">IF(B10=0,0,J10/B10)</f>
-        <v>0.05</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5052,7 +5041,7 @@
       </c>
       <c r="C11" s="23" t="n">
         <f aca="false">SUMPRODUCT((Products!$A$5:$A$200=$A11)*Products!$F$5:$F$200*Products!$H$5:$H$200)</f>
-        <v>1750</v>
+        <v>0</v>
       </c>
       <c r="D11" s="23" t="n">
         <f aca="false">SUMIFS(Products!$G:$G,Products!$A:$A,$A11,Products!$C:$C,"Upsell")</f>
@@ -5070,15 +5059,15 @@
       </c>
       <c r="I11" s="23" t="n">
         <f aca="false">SUMIFS(Products!$K:$K,Products!$A:$A,$A11)</f>
-        <v>36750</v>
+        <v>35000</v>
       </c>
       <c r="J11" s="23" t="n">
         <f aca="false">I11-B11</f>
-        <v>1750</v>
+        <v>0</v>
       </c>
       <c r="K11" s="22" t="n">
         <f aca="false">IF(B11=0,0,J11/B11)</f>
-        <v>0.05</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5092,7 +5081,7 @@
       </c>
       <c r="C12" s="23" t="n">
         <f aca="false">SUMPRODUCT((Products!$A$5:$A$200=$A12)*Products!$F$5:$F$200*Products!$H$5:$H$200)</f>
-        <v>2300</v>
+        <v>0</v>
       </c>
       <c r="D12" s="23" t="n">
         <f aca="false">SUMIFS(Products!$G:$G,Products!$A:$A,$A12,Products!$C:$C,"Upsell")</f>
@@ -5110,15 +5099,15 @@
       </c>
       <c r="I12" s="23" t="n">
         <f aca="false">SUMIFS(Products!$K:$K,Products!$A:$A,$A12)</f>
-        <v>48300</v>
+        <v>46000</v>
       </c>
       <c r="J12" s="23" t="n">
         <f aca="false">I12-B12</f>
-        <v>2300</v>
+        <v>0</v>
       </c>
       <c r="K12" s="22" t="n">
         <f aca="false">IF(B12=0,0,J12/B12)</f>
-        <v>0.05</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5175,7 +5164,7 @@
       </c>
       <c r="C14" s="24" t="n">
         <f aca="false">SUM(C4:C13)</f>
-        <v>14500</v>
+        <v>0</v>
       </c>
       <c r="D14" s="24" t="n">
         <f aca="false">SUM(D4:D13)</f>
@@ -5187,19 +5176,19 @@
       </c>
       <c r="H14" s="24" t="n">
         <f aca="false">SUM(H4:H13)</f>
-        <v>-2736</v>
+        <v>-3600</v>
       </c>
       <c r="I14" s="24" t="n">
         <f aca="false">SUM(I4:I13)</f>
-        <v>361964</v>
+        <v>348400</v>
       </c>
       <c r="J14" s="24" t="n">
         <f aca="false">SUM(J4:J13)</f>
-        <v>-13036</v>
+        <v>-26600</v>
       </c>
       <c r="K14" s="33" t="n">
         <f aca="false">IF(B14=0,0,J14/B14)</f>
-        <v>-0.0347626666666667</v>
+        <v>-0.0709333333333333</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5216,7 +5205,7 @@
       </c>
       <c r="H15" s="35" t="n">
         <f aca="false">H14</f>
-        <v>-2736</v>
+        <v>-3600</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5363,11 +5352,11 @@
       </c>
       <c r="E4" s="23" t="n">
         <f aca="false">SUMIFS(Pipeline!$S$5:$S$14,Pipeline!$M$5:$M$14,B4)</f>
-        <v>72450</v>
+        <v>69000</v>
       </c>
       <c r="F4" s="23" t="n">
         <f aca="false">SUMIFS(Pipeline!$T$5:$T$14,Pipeline!$M$5:$M$14,B4)</f>
-        <v>23625</v>
+        <v>22500</v>
       </c>
       <c r="G4" s="23" t="n">
         <f aca="false">SUMIFS(Pipeline!$T$5:$T$14,Pipeline!$M$5:$M$14,B4,Pipeline!$U$5:$U$14,"On time")</f>
@@ -5375,7 +5364,7 @@
       </c>
       <c r="H4" s="23" t="n">
         <f aca="false">SUMIFS(Pipeline!$T$5:$T$14,Pipeline!$M$5:$M$14,B4,Pipeline!$U$5:$U$14,"Late")</f>
-        <v>23625</v>
+        <v>22500</v>
       </c>
       <c r="I4" s="23" t="n">
         <f aca="false">SUMIFS(Pipeline!$B$5:$B$14,Pipeline!$M$5:$M$14,B4,Pipeline!$L$5:$L$14,"YES")</f>
@@ -5403,19 +5392,19 @@
       </c>
       <c r="E5" s="23" t="n">
         <f aca="false">SUMIFS(Pipeline!$S$5:$S$14,Pipeline!$M$5:$M$14,B5)</f>
-        <v>175950</v>
+        <v>169000</v>
       </c>
       <c r="F5" s="23" t="n">
         <f aca="false">SUMIFS(Pipeline!$T$5:$T$14,Pipeline!$M$5:$M$14,B5)</f>
-        <v>68310</v>
+        <v>65200</v>
       </c>
       <c r="G5" s="23" t="n">
         <f aca="false">SUMIFS(Pipeline!$T$5:$T$14,Pipeline!$M$5:$M$14,B5,Pipeline!$U$5:$U$14,"On time")</f>
-        <v>27930</v>
+        <v>26600</v>
       </c>
       <c r="H5" s="23" t="n">
         <f aca="false">SUMIFS(Pipeline!$T$5:$T$14,Pipeline!$M$5:$M$14,B5,Pipeline!$U$5:$U$14,"Late")</f>
-        <v>40380</v>
+        <v>38600</v>
       </c>
       <c r="I5" s="23" t="n">
         <f aca="false">SUMIFS(Pipeline!$B$5:$B$14,Pipeline!$M$5:$M$14,B5,Pipeline!$L$5:$L$14,"YES")</f>
@@ -5443,15 +5432,15 @@
       </c>
       <c r="E6" s="23" t="n">
         <f aca="false">SUMIFS(Pipeline!$S$5:$S$14,Pipeline!$M$5:$M$14,B6)</f>
-        <v>113564</v>
+        <v>110400</v>
       </c>
       <c r="F6" s="23" t="n">
         <f aca="false">SUMIFS(Pipeline!$T$5:$T$14,Pipeline!$M$5:$M$14,B6)</f>
-        <v>46337</v>
+        <v>45100</v>
       </c>
       <c r="G6" s="23" t="n">
         <f aca="false">SUMIFS(Pipeline!$T$5:$T$14,Pipeline!$M$5:$M$14,B6,Pipeline!$U$5:$U$14,"On time")</f>
-        <v>46337</v>
+        <v>45100</v>
       </c>
       <c r="H6" s="23" t="n">
         <f aca="false">SUMIFS(Pipeline!$T$5:$T$14,Pipeline!$M$5:$M$14,B6,Pipeline!$U$5:$U$14,"Late")</f>
@@ -5480,19 +5469,19 @@
       </c>
       <c r="E7" s="24" t="n">
         <f aca="false">SUM(E4:E6)</f>
-        <v>361964</v>
+        <v>348400</v>
       </c>
       <c r="F7" s="24" t="n">
         <f aca="false">SUM(F4:F6)</f>
-        <v>138272</v>
+        <v>132800</v>
       </c>
       <c r="G7" s="24" t="n">
         <f aca="false">SUM(G4:G6)</f>
-        <v>74267</v>
+        <v>71700</v>
       </c>
       <c r="H7" s="24" t="n">
         <f aca="false">SUM(H4:H6)</f>
-        <v>64005</v>
+        <v>61100</v>
       </c>
       <c r="I7" s="24" t="n">
         <f aca="false">SUM(I4:I6)</f>

</xml_diff>

<commit_message>
Show the 30 Oct forecast with actions (green) and with no action (red)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CVAHSCDuy4tEBaMUUSRsNB
</commit_message>
<xml_diff>
--- a/n8n-renewals-challenge/renewal_tracker.xlsx
+++ b/n8n-renewals-challenge/renewal_tracker.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <fileVersion appName="Calc"/>
-  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
+  <workbookPr backupFile="false" showObjects="all" dateCompatibility="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="600" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Read me" sheetId="1" state="visible" r:id="rId3"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/comments3.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:v2="http://schemas.openxmlformats.org/spreadsheetml/2006/main/v2" mc:Ignorable="v2">
   <authors>
     <author>Unknown Author</author>
   </authors>
@@ -43,13 +43,34 @@
           <t xml:space="preserve">Exercise date: Tue 20 Oct 2026, so Vantage is overdue and the other nine fall inside 60 days. Use =TODAY() in live use.</t>
         </r>
       </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>4</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>75</xdr:colOff>
+                <xdr:row>3</xdr:row>
+                <xdr:rowOff>39</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
     </comment>
   </commentList>
 </comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="403" uniqueCount="278">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="408" uniqueCount="283">
   <si>
     <t xml:space="preserve">Renewal tracker: a mock-up of the CRM renewal model</t>
   </si>
@@ -189,7 +210,7 @@
     <t xml:space="preserve">Target date</t>
   </si>
   <si>
-    <t xml:space="preserve">Blue on yellow = input. Everything else is a formula. Columns AF-AH: the forecast after this week's actions.</t>
+    <t xml:space="preserve">Blue on yellow = input. Everything else is a formula. Columns AF-AJ: the forecast on 30 Oct, with this week's actions (green) and with no action (red).</t>
   </si>
   <si>
     <t xml:space="preserve">Base ARR (€)</t>
@@ -261,6 +282,12 @@
     <t xml:space="preserve">Weighted after actions (€)</t>
   </si>
   <si>
+    <t xml:space="preserve">No-action prob. (30 Oct)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Weighted, no action (€)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Vantage Freight</t>
   </si>
   <si>
@@ -516,6 +543,15 @@
     <t xml:space="preserve">Gain from this week's actions</t>
   </si>
   <si>
+    <t xml:space="preserve">Weighted by 30 Oct with no action (statuses stay, the countdown runs)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cost of doing nothing (vs today)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Action power: with actions vs no action on 30 Oct</t>
+  </si>
+  <si>
     <t xml:space="preserve">Opportunity products: the Renewals Manager only sets the line type and the new numbers; everything else recalculates</t>
   </si>
   <si>
@@ -630,7 +666,7 @@
     <t xml:space="preserve">Opportunity roll-up: calculated from product lines; churn category and reason set on the opportunity</t>
   </si>
   <si>
-    <t xml:space="preserve">Uplift (€)</t>
+    <t xml:space="preserve">Extra uplift (€)</t>
   </si>
   <si>
     <t xml:space="preserve">Upsell (€) → Upsell opp</t>
@@ -891,9 +927,9 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="7">
     <numFmt numFmtId="164" formatCode="General"/>
-    <numFmt numFmtId="165" formatCode="\€#,##0;[RED]&quot;-€&quot;#,##0;\-"/>
-    <numFmt numFmtId="166" formatCode="dd\ mmm\ yyyy"/>
-    <numFmt numFmtId="167" formatCode="General"/>
+    <numFmt numFmtId="165" formatCode="General"/>
+    <numFmt numFmtId="166" formatCode="\€#,##0;[RED]&quot;-€&quot;#,##0;\-"/>
+    <numFmt numFmtId="167" formatCode="dd\ mmm\ yyyy"/>
     <numFmt numFmtId="168" formatCode="0%;[RED]\-0%;\-"/>
     <numFmt numFmtId="169" formatCode="0.0%"/>
     <numFmt numFmtId="170" formatCode="0%"/>
@@ -999,7 +1035,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1016,6 +1052,18 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFFF2CC"/>
         <bgColor rgb="FFFFF3CD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD4EDDA"/>
+        <bgColor rgb="FFCCFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF8D7DA"/>
+        <bgColor rgb="FFFFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -1068,7 +1116,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="41">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1101,10 +1149,6 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="165" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1117,6 +1161,10 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1125,7 +1173,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="167" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1133,11 +1181,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="167" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1153,7 +1201,7 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="167" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1161,11 +1209,19 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1177,7 +1233,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1185,11 +1241,19 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="169" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1209,7 +1273,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1733,7 +1797,7 @@
         <f aca="false">INDEX(Pipeline!$C$5:$C$14,MATCH($A5,Pipeline!$Y$5:$Y$14,0))</f>
         <v>46324</v>
       </c>
-      <c r="E5" s="11" t="n">
+      <c r="E5" s="8" t="n">
         <f aca="false">INDEX(Pipeline!$J$5:$J$14,MATCH($A5,Pipeline!$Y$5:$Y$14,0))</f>
         <v>9</v>
       </c>
@@ -1761,7 +1825,7 @@
         <f aca="false">INDEX(Pipeline!$X$5:$X$14,MATCH($A5,Pipeline!$Y$5:$Y$14,0))</f>
         <v>46315</v>
       </c>
-      <c r="L5" s="8" t="str">
+      <c r="L5" s="11" t="str">
         <f aca="false">INDEX(Pipeline!$AB$5:$AB$14,MATCH($A5,Pipeline!$Y$5:$Y$14,0))&amp;""</f>
         <v/>
       </c>
@@ -1782,7 +1846,7 @@
         <f aca="false">INDEX(Pipeline!$C$5:$C$14,MATCH($A6,Pipeline!$Y$5:$Y$14,0))</f>
         <v>46310</v>
       </c>
-      <c r="E6" s="11" t="n">
+      <c r="E6" s="8" t="n">
         <f aca="false">INDEX(Pipeline!$J$5:$J$14,MATCH($A6,Pipeline!$Y$5:$Y$14,0))</f>
         <v>-5</v>
       </c>
@@ -1810,7 +1874,7 @@
         <f aca="false">INDEX(Pipeline!$X$5:$X$14,MATCH($A6,Pipeline!$Y$5:$Y$14,0))</f>
         <v>46316</v>
       </c>
-      <c r="L6" s="8" t="str">
+      <c r="L6" s="11" t="str">
         <f aca="false">INDEX(Pipeline!$AB$5:$AB$14,MATCH($A6,Pipeline!$Y$5:$Y$14,0))&amp;""</f>
         <v>Yes: Manager, to agree the grace period before access is restricted</v>
       </c>
@@ -1831,7 +1895,7 @@
         <f aca="false">INDEX(Pipeline!$C$5:$C$14,MATCH($A7,Pipeline!$Y$5:$Y$14,0))</f>
         <v>46328</v>
       </c>
-      <c r="E7" s="11" t="n">
+      <c r="E7" s="8" t="n">
         <f aca="false">INDEX(Pipeline!$J$5:$J$14,MATCH($A7,Pipeline!$Y$5:$Y$14,0))</f>
         <v>13</v>
       </c>
@@ -1859,7 +1923,7 @@
         <f aca="false">INDEX(Pipeline!$X$5:$X$14,MATCH($A7,Pipeline!$Y$5:$Y$14,0))</f>
         <v>46317</v>
       </c>
-      <c r="L7" s="8" t="str">
+      <c r="L7" s="11" t="str">
         <f aca="false">INDEX(Pipeline!$AB$5:$AB$14,MATCH($A7,Pipeline!$Y$5:$Y$14,0))&amp;""</f>
         <v/>
       </c>
@@ -1880,7 +1944,7 @@
         <f aca="false">INDEX(Pipeline!$C$5:$C$14,MATCH($A8,Pipeline!$Y$5:$Y$14,0))</f>
         <v>46333</v>
       </c>
-      <c r="E8" s="11" t="n">
+      <c r="E8" s="8" t="n">
         <f aca="false">INDEX(Pipeline!$J$5:$J$14,MATCH($A8,Pipeline!$Y$5:$Y$14,0))</f>
         <v>18</v>
       </c>
@@ -1908,7 +1972,7 @@
         <f aca="false">INDEX(Pipeline!$X$5:$X$14,MATCH($A8,Pipeline!$Y$5:$Y$14,0))</f>
         <v>46318</v>
       </c>
-      <c r="L8" s="8" t="str">
+      <c r="L8" s="11" t="str">
         <f aca="false">INDEX(Pipeline!$AB$5:$AB$14,MATCH($A8,Pipeline!$Y$5:$Y$14,0))&amp;""</f>
         <v>Yes: Manager + VP CS, exec sponsor meeting with the new owner this week</v>
       </c>
@@ -1929,7 +1993,7 @@
         <f aca="false">INDEX(Pipeline!$C$5:$C$14,MATCH($A9,Pipeline!$Y$5:$Y$14,0))</f>
         <v>46344</v>
       </c>
-      <c r="E9" s="11" t="n">
+      <c r="E9" s="8" t="n">
         <f aca="false">INDEX(Pipeline!$J$5:$J$14,MATCH($A9,Pipeline!$Y$5:$Y$14,0))</f>
         <v>29</v>
       </c>
@@ -1957,7 +2021,7 @@
         <f aca="false">INDEX(Pipeline!$X$5:$X$14,MATCH($A9,Pipeline!$Y$5:$Y$14,0))</f>
         <v>46318</v>
       </c>
-      <c r="L9" s="8" t="str">
+      <c r="L9" s="11" t="str">
         <f aca="false">INDEX(Pipeline!$AB$5:$AB$14,MATCH($A9,Pipeline!$Y$5:$Y$14,0))&amp;""</f>
         <v>Yes: Legal lead, redline response by 30 Oct and renew on the current MSA</v>
       </c>
@@ -1978,7 +2042,7 @@
         <f aca="false">INDEX(Pipeline!$C$5:$C$14,MATCH($A10,Pipeline!$Y$5:$Y$14,0))</f>
         <v>46370</v>
       </c>
-      <c r="E10" s="11" t="n">
+      <c r="E10" s="8" t="n">
         <f aca="false">INDEX(Pipeline!$J$5:$J$14,MATCH($A10,Pipeline!$Y$5:$Y$14,0))</f>
         <v>55</v>
       </c>
@@ -2006,7 +2070,7 @@
         <f aca="false">INDEX(Pipeline!$X$5:$X$14,MATCH($A10,Pipeline!$Y$5:$Y$14,0))</f>
         <v>46315</v>
       </c>
-      <c r="L10" s="8" t="str">
+      <c r="L10" s="11" t="str">
         <f aca="false">INDEX(Pipeline!$AB$5:$AB$14,MATCH($A10,Pipeline!$Y$5:$Y$14,0))&amp;""</f>
         <v/>
       </c>
@@ -2027,7 +2091,7 @@
         <f aca="false">INDEX(Pipeline!$C$5:$C$14,MATCH($A11,Pipeline!$Y$5:$Y$14,0))</f>
         <v>46365</v>
       </c>
-      <c r="E11" s="11" t="n">
+      <c r="E11" s="8" t="n">
         <f aca="false">INDEX(Pipeline!$J$5:$J$14,MATCH($A11,Pipeline!$Y$5:$Y$14,0))</f>
         <v>50</v>
       </c>
@@ -2055,7 +2119,7 @@
         <f aca="false">INDEX(Pipeline!$X$5:$X$14,MATCH($A11,Pipeline!$Y$5:$Y$14,0))</f>
         <v>46322</v>
       </c>
-      <c r="L11" s="8" t="str">
+      <c r="L11" s="11" t="str">
         <f aca="false">INDEX(Pipeline!$AB$5:$AB$14,MATCH($A11,Pipeline!$Y$5:$Y$14,0))&amp;""</f>
         <v/>
       </c>
@@ -2076,7 +2140,7 @@
         <f aca="false">INDEX(Pipeline!$C$5:$C$14,MATCH($A12,Pipeline!$Y$5:$Y$14,0))</f>
         <v>46354</v>
       </c>
-      <c r="E12" s="11" t="n">
+      <c r="E12" s="8" t="n">
         <f aca="false">INDEX(Pipeline!$J$5:$J$14,MATCH($A12,Pipeline!$Y$5:$Y$14,0))</f>
         <v>39</v>
       </c>
@@ -2104,7 +2168,7 @@
         <f aca="false">INDEX(Pipeline!$X$5:$X$14,MATCH($A12,Pipeline!$Y$5:$Y$14,0))</f>
         <v>46323</v>
       </c>
-      <c r="L12" s="8" t="str">
+      <c r="L12" s="11" t="str">
         <f aca="false">INDEX(Pipeline!$AB$5:$AB$14,MATCH($A12,Pipeline!$Y$5:$Y$14,0))&amp;""</f>
         <v/>
       </c>
@@ -2125,7 +2189,7 @@
         <f aca="false">INDEX(Pipeline!$C$5:$C$14,MATCH($A13,Pipeline!$Y$5:$Y$14,0))</f>
         <v>46347</v>
       </c>
-      <c r="E13" s="11" t="n">
+      <c r="E13" s="8" t="n">
         <f aca="false">INDEX(Pipeline!$J$5:$J$14,MATCH($A13,Pipeline!$Y$5:$Y$14,0))</f>
         <v>32</v>
       </c>
@@ -2153,7 +2217,7 @@
         <f aca="false">INDEX(Pipeline!$X$5:$X$14,MATCH($A13,Pipeline!$Y$5:$Y$14,0))</f>
         <v>46317</v>
       </c>
-      <c r="L13" s="8" t="str">
+      <c r="L13" s="11" t="str">
         <f aca="false">INDEX(Pipeline!$AB$5:$AB$14,MATCH($A13,Pipeline!$Y$5:$Y$14,0))&amp;""</f>
         <v/>
       </c>
@@ -2174,7 +2238,7 @@
         <f aca="false">INDEX(Pipeline!$C$5:$C$14,MATCH($A14,Pipeline!$Y$5:$Y$14,0))</f>
         <v>46375</v>
       </c>
-      <c r="E14" s="11" t="n">
+      <c r="E14" s="8" t="n">
         <f aca="false">INDEX(Pipeline!$J$5:$J$14,MATCH($A14,Pipeline!$Y$5:$Y$14,0))</f>
         <v>60</v>
       </c>
@@ -2202,7 +2266,7 @@
         <f aca="false">INDEX(Pipeline!$X$5:$X$14,MATCH($A14,Pipeline!$Y$5:$Y$14,0))</f>
         <v>46325</v>
       </c>
-      <c r="L14" s="8" t="str">
+      <c r="L14" s="11" t="str">
         <f aca="false">INDEX(Pipeline!$AB$5:$AB$14,MATCH($A14,Pipeline!$Y$5:$Y$14,0))&amp;""</f>
         <v/>
       </c>
@@ -2267,7 +2331,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:AH34"/>
+  <dimension ref="A1:AJ37"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="20"/>
@@ -2297,6 +2361,8 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="32" min="32" style="0" width="26"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="33" min="33" style="0" width="10"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="34" min="34" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="35" min="35" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="36" min="36" style="0" width="14"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2424,10 +2490,16 @@
       <c r="AH4" s="6" t="s">
         <v>69</v>
       </c>
+      <c r="AI4" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="AJ4" s="6" t="s">
+        <v>71</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="15" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B5" s="16" t="n">
         <v>21000</v>
@@ -2436,19 +2508,19 @@
         <v>46310</v>
       </c>
       <c r="D5" s="18" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="E5" s="19" t="n">
         <v>0</v>
       </c>
       <c r="F5" s="18" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="G5" s="18" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="H5" s="20" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="I5" s="17" t="n">
         <v>46332</v>
@@ -2502,10 +2574,10 @@
         <v>Late</v>
       </c>
       <c r="V5" s="20" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="W5" s="18" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="X5" s="17" t="n">
         <v>46316</v>
@@ -2514,13 +2586,13 @@
         <v>2</v>
       </c>
       <c r="Z5" s="20" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="AA5" s="20" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="AB5" s="20" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="AC5" s="18"/>
       <c r="AD5" s="21" t="str">
@@ -2532,20 +2604,28 @@
         <v/>
       </c>
       <c r="AF5" s="20" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AG5" s="22" t="n">
         <f aca="false">IF(I5&lt;=O5,INDEX(Probability!$B$5:$F$19,MATCH(AF5,Probability!$A$5:$A$19,0),MATCH(IF(C5-$E$2&lt;0,"Overdue",IF(C5-$E$2&lt;=30,"0-30",IF(C5-$E$2&lt;=60,"31-60",IF(C5-$E$2&lt;=90,"61-90","&gt;90")))),Probability!$B$4:$F$4,0)),0)</f>
         <v>0.7</v>
       </c>
-      <c r="AH5" s="23" t="n">
+      <c r="AH5" s="24" t="n">
         <f aca="false">S5*AG5</f>
         <v>14700</v>
       </c>
+      <c r="AI5" s="22" t="n">
+        <f aca="false">IF(I5&lt;=O5,INDEX(Probability!$B$5:$F$19,MATCH(G5,Probability!$A$5:$A$19,0),MATCH(IF(C5-$E$2&lt;0,"Overdue",IF(C5-$E$2&lt;=30,"0-30",IF(C5-$E$2&lt;=60,"31-60",IF(C5-$E$2&lt;=90,"61-90","&gt;90")))),Probability!$B$4:$F$4,0)),0)</f>
+        <v>0.5</v>
+      </c>
+      <c r="AJ5" s="25" t="n">
+        <f aca="false">S5*AI5</f>
+        <v>10500</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="15" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B6" s="16" t="n">
         <v>48000</v>
@@ -2554,19 +2634,19 @@
         <v>46324</v>
       </c>
       <c r="D6" s="18" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="E6" s="19" t="n">
         <v>0.12</v>
       </c>
       <c r="F6" s="18" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="G6" s="18" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="H6" s="20" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="I6" s="17" t="n">
         <v>46324</v>
@@ -2620,10 +2700,10 @@
         <v>Late</v>
       </c>
       <c r="V6" s="20" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="W6" s="18" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="X6" s="17" t="n">
         <v>46315</v>
@@ -2632,10 +2712,10 @@
         <v>1</v>
       </c>
       <c r="Z6" s="20" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="AA6" s="20" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="AB6" s="20"/>
       <c r="AC6" s="18"/>
@@ -2648,20 +2728,28 @@
         <v/>
       </c>
       <c r="AF6" s="20" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="AG6" s="22" t="n">
         <f aca="false">IF(I6&lt;=O6,INDEX(Probability!$B$5:$F$19,MATCH(AF6,Probability!$A$5:$A$19,0),MATCH(IF(C6-$E$2&lt;0,"Overdue",IF(C6-$E$2&lt;=30,"0-30",IF(C6-$E$2&lt;=60,"31-60",IF(C6-$E$2&lt;=90,"61-90","&gt;90")))),Probability!$B$4:$F$4,0)),0)</f>
         <v>0.95</v>
       </c>
-      <c r="AH6" s="23" t="n">
+      <c r="AH6" s="24" t="n">
         <f aca="false">S6*AG6</f>
         <v>45600</v>
       </c>
+      <c r="AI6" s="22" t="n">
+        <f aca="false">IF(I6&lt;=O6,INDEX(Probability!$B$5:$F$19,MATCH(G6,Probability!$A$5:$A$19,0),MATCH(IF(C6-$E$2&lt;0,"Overdue",IF(C6-$E$2&lt;=30,"0-30",IF(C6-$E$2&lt;=60,"31-60",IF(C6-$E$2&lt;=90,"61-90","&gt;90")))),Probability!$B$4:$F$4,0)),0)</f>
+        <v>0.1</v>
+      </c>
+      <c r="AJ6" s="25" t="n">
+        <f aca="false">S6*AI6</f>
+        <v>4800</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="15" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B7" s="16" t="n">
         <v>26000</v>
@@ -2670,19 +2758,19 @@
         <v>46328</v>
       </c>
       <c r="D7" s="18" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="E7" s="19" t="n">
         <v>0</v>
       </c>
       <c r="F7" s="18" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="G7" s="18" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="H7" s="20" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="I7" s="17" t="n">
         <v>46328</v>
@@ -2736,10 +2824,10 @@
         <v>Late</v>
       </c>
       <c r="V7" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="W7" s="18" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="X7" s="17" t="n">
         <v>46317</v>
@@ -2748,10 +2836,10 @@
         <v>3</v>
       </c>
       <c r="Z7" s="20" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="AA7" s="20" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="AB7" s="20"/>
       <c r="AC7" s="18" t="n">
@@ -2766,20 +2854,28 @@
         <v/>
       </c>
       <c r="AF7" s="20" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="AG7" s="22" t="n">
         <f aca="false">IF(I7&lt;=O7,INDEX(Probability!$B$5:$F$19,MATCH(AF7,Probability!$A$5:$A$19,0),MATCH(IF(C7-$E$2&lt;0,"Overdue",IF(C7-$E$2&lt;=30,"0-30",IF(C7-$E$2&lt;=60,"31-60",IF(C7-$E$2&lt;=90,"61-90","&gt;90")))),Probability!$B$4:$F$4,0)),0)</f>
         <v>0.97</v>
       </c>
-      <c r="AH7" s="23" t="n">
+      <c r="AH7" s="24" t="n">
         <f aca="false">S7*AG7</f>
         <v>25220</v>
       </c>
+      <c r="AI7" s="22" t="n">
+        <f aca="false">IF(I7&lt;=O7,INDEX(Probability!$B$5:$F$19,MATCH(G7,Probability!$A$5:$A$19,0),MATCH(IF(C7-$E$2&lt;0,"Overdue",IF(C7-$E$2&lt;=30,"0-30",IF(C7-$E$2&lt;=60,"31-60",IF(C7-$E$2&lt;=90,"61-90","&gt;90")))),Probability!$B$4:$F$4,0)),0)</f>
+        <v>0.6</v>
+      </c>
+      <c r="AJ7" s="25" t="n">
+        <f aca="false">S7*AI7</f>
+        <v>15600</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="15" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B8" s="16" t="n">
         <v>45000</v>
@@ -2788,19 +2884,19 @@
         <v>46333</v>
       </c>
       <c r="D8" s="18" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="E8" s="19" t="n">
         <v>-0.35</v>
       </c>
       <c r="F8" s="18" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="G8" s="18" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="H8" s="20" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="I8" s="17" t="n">
         <v>46346</v>
@@ -2854,10 +2950,10 @@
         <v>Late</v>
       </c>
       <c r="V8" s="20" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="W8" s="18" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="X8" s="17" t="n">
         <v>46318</v>
@@ -2866,13 +2962,13 @@
         <v>4</v>
       </c>
       <c r="Z8" s="20" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="AA8" s="20" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="AB8" s="20" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="AC8" s="18" t="n">
         <v>30</v>
@@ -2886,20 +2982,28 @@
         <v>Under-usage: flag CSM</v>
       </c>
       <c r="AF8" s="20" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="AG8" s="22" t="n">
         <f aca="false">IF(I8&lt;=O8,INDEX(Probability!$B$5:$F$19,MATCH(AF8,Probability!$A$5:$A$19,0),MATCH(IF(C8-$E$2&lt;0,"Overdue",IF(C8-$E$2&lt;=30,"0-30",IF(C8-$E$2&lt;=60,"31-60",IF(C8-$E$2&lt;=90,"61-90","&gt;90")))),Probability!$B$4:$F$4,0)),0)</f>
         <v>0.25</v>
       </c>
-      <c r="AH8" s="23" t="n">
+      <c r="AH8" s="24" t="n">
         <f aca="false">S8*AG8</f>
         <v>7500</v>
       </c>
+      <c r="AI8" s="22" t="n">
+        <f aca="false">IF(I8&lt;=O8,INDEX(Probability!$B$5:$F$19,MATCH(G8,Probability!$A$5:$A$19,0),MATCH(IF(C8-$E$2&lt;0,"Overdue",IF(C8-$E$2&lt;=30,"0-30",IF(C8-$E$2&lt;=60,"31-60",IF(C8-$E$2&lt;=90,"61-90","&gt;90")))),Probability!$B$4:$F$4,0)),0)</f>
+        <v>0.1</v>
+      </c>
+      <c r="AJ8" s="25" t="n">
+        <f aca="false">S8*AI8</f>
+        <v>3000</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="15" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B9" s="16" t="n">
         <v>36000</v>
@@ -2908,19 +3012,19 @@
         <v>46370</v>
       </c>
       <c r="D9" s="18" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="E9" s="19" t="n">
         <v>-0.1</v>
       </c>
       <c r="F9" s="18" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="G9" s="18" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="H9" s="20" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="I9" s="17" t="n">
         <v>46356</v>
@@ -2974,10 +3078,10 @@
         <v>On time</v>
       </c>
       <c r="V9" s="20" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="W9" s="18" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="X9" s="17" t="n">
         <v>46315</v>
@@ -2986,10 +3090,10 @@
         <v>6</v>
       </c>
       <c r="Z9" s="20" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="AA9" s="20" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="AB9" s="20"/>
       <c r="AC9" s="18"/>
@@ -3002,20 +3106,28 @@
         <v/>
       </c>
       <c r="AF9" s="20" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="AG9" s="22" t="n">
         <f aca="false">IF(I9&lt;=O9,INDEX(Probability!$B$5:$F$19,MATCH(AF9,Probability!$A$5:$A$19,0),MATCH(IF(C9-$E$2&lt;0,"Overdue",IF(C9-$E$2&lt;=30,"0-30",IF(C9-$E$2&lt;=60,"31-60",IF(C9-$E$2&lt;=90,"61-90","&gt;90")))),Probability!$B$4:$F$4,0)),0)</f>
         <v>0.5</v>
       </c>
-      <c r="AH9" s="23" t="n">
+      <c r="AH9" s="24" t="n">
         <f aca="false">S9*AG9</f>
         <v>16200</v>
       </c>
+      <c r="AI9" s="22" t="n">
+        <f aca="false">IF(I9&lt;=O9,INDEX(Probability!$B$5:$F$19,MATCH(G9,Probability!$A$5:$A$19,0),MATCH(IF(C9-$E$2&lt;0,"Overdue",IF(C9-$E$2&lt;=30,"0-30",IF(C9-$E$2&lt;=60,"31-60",IF(C9-$E$2&lt;=90,"61-90","&gt;90")))),Probability!$B$4:$F$4,0)),0)</f>
+        <v>0.5</v>
+      </c>
+      <c r="AJ9" s="25" t="n">
+        <f aca="false">S9*AI9</f>
+        <v>16200</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="15" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B10" s="16" t="n">
         <v>50000</v>
@@ -3024,19 +3136,19 @@
         <v>46344</v>
       </c>
       <c r="D10" s="18" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="E10" s="19" t="n">
         <v>0.05</v>
       </c>
       <c r="F10" s="18" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="G10" s="18" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="H10" s="20" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="I10" s="17" t="n">
         <v>46360</v>
@@ -3090,10 +3202,10 @@
         <v>Late</v>
       </c>
       <c r="V10" s="20" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="W10" s="18" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="X10" s="17" t="n">
         <v>46318</v>
@@ -3102,13 +3214,13 @@
         <v>5</v>
       </c>
       <c r="Z10" s="20" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="AA10" s="20" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="AB10" s="20" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="AC10" s="18"/>
       <c r="AD10" s="21" t="str">
@@ -3120,20 +3232,28 @@
         <v/>
       </c>
       <c r="AF10" s="20" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="AG10" s="22" t="n">
         <f aca="false">IF(I10&lt;=O10,INDEX(Probability!$B$5:$F$19,MATCH(AF10,Probability!$A$5:$A$19,0),MATCH(IF(C10-$E$2&lt;0,"Overdue",IF(C10-$E$2&lt;=30,"0-30",IF(C10-$E$2&lt;=60,"31-60",IF(C10-$E$2&lt;=90,"61-90","&gt;90")))),Probability!$B$4:$F$4,0)),0)</f>
         <v>0.75</v>
       </c>
-      <c r="AH10" s="23" t="n">
+      <c r="AH10" s="24" t="n">
         <f aca="false">S10*AG10</f>
         <v>37500</v>
       </c>
+      <c r="AI10" s="22" t="n">
+        <f aca="false">IF(I10&lt;=O10,INDEX(Probability!$B$5:$F$19,MATCH(G10,Probability!$A$5:$A$19,0),MATCH(IF(C10-$E$2&lt;0,"Overdue",IF(C10-$E$2&lt;=30,"0-30",IF(C10-$E$2&lt;=60,"31-60",IF(C10-$E$2&lt;=90,"61-90","&gt;90")))),Probability!$B$4:$F$4,0)),0)</f>
+        <v>0.4</v>
+      </c>
+      <c r="AJ10" s="25" t="n">
+        <f aca="false">S10*AI10</f>
+        <v>20000</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="15" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B11" s="16" t="n">
         <v>28000</v>
@@ -3142,19 +3262,19 @@
         <v>46347</v>
       </c>
       <c r="D11" s="18" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="E11" s="19" t="n">
         <v>0.08</v>
       </c>
       <c r="F11" s="18" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="G11" s="18" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="H11" s="20" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="I11" s="17" t="n">
         <v>46347</v>
@@ -3208,10 +3328,10 @@
         <v>On time</v>
       </c>
       <c r="V11" s="20" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="W11" s="18" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="X11" s="17" t="n">
         <v>46317</v>
@@ -3220,10 +3340,10 @@
         <v>9</v>
       </c>
       <c r="Z11" s="20" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="AA11" s="20" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="AB11" s="20"/>
       <c r="AC11" s="18" t="n">
@@ -3238,20 +3358,28 @@
         <v/>
       </c>
       <c r="AF11" s="20" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="AG11" s="22" t="n">
         <f aca="false">IF(I11&lt;=O11,INDEX(Probability!$B$5:$F$19,MATCH(AF11,Probability!$A$5:$A$19,0),MATCH(IF(C11-$E$2&lt;0,"Overdue",IF(C11-$E$2&lt;=30,"0-30",IF(C11-$E$2&lt;=60,"31-60",IF(C11-$E$2&lt;=90,"61-90","&gt;90")))),Probability!$B$4:$F$4,0)),0)</f>
         <v>0.97</v>
       </c>
-      <c r="AH11" s="23" t="n">
+      <c r="AH11" s="24" t="n">
         <f aca="false">S11*AG11</f>
         <v>27160</v>
       </c>
+      <c r="AI11" s="22" t="n">
+        <f aca="false">IF(I11&lt;=O11,INDEX(Probability!$B$5:$F$19,MATCH(G11,Probability!$A$5:$A$19,0),MATCH(IF(C11-$E$2&lt;0,"Overdue",IF(C11-$E$2&lt;=30,"0-30",IF(C11-$E$2&lt;=60,"31-60",IF(C11-$E$2&lt;=90,"61-90","&gt;90")))),Probability!$B$4:$F$4,0)),0)</f>
+        <v>0.6</v>
+      </c>
+      <c r="AJ11" s="25" t="n">
+        <f aca="false">S11*AI11</f>
+        <v>16800</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="15" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B12" s="16" t="n">
         <v>35000</v>
@@ -3260,19 +3388,19 @@
         <v>46354</v>
       </c>
       <c r="D12" s="18" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="E12" s="19" t="n">
         <v>0.4</v>
       </c>
       <c r="F12" s="18" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="G12" s="18" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="H12" s="20" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="I12" s="17" t="n">
         <v>46354</v>
@@ -3326,10 +3454,10 @@
         <v>On time</v>
       </c>
       <c r="V12" s="20" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="W12" s="18" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="X12" s="17" t="n">
         <v>46323</v>
@@ -3338,10 +3466,10 @@
         <v>8</v>
       </c>
       <c r="Z12" s="20" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="AA12" s="20" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="AB12" s="20"/>
       <c r="AC12" s="18"/>
@@ -3354,20 +3482,28 @@
         <v>Over-usage: open Upsell opp + CSM/Renewals task</v>
       </c>
       <c r="AF12" s="20" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="AG12" s="22" t="n">
         <f aca="false">IF(I12&lt;=O12,INDEX(Probability!$B$5:$F$19,MATCH(AF12,Probability!$A$5:$A$19,0),MATCH(IF(C12-$E$2&lt;0,"Overdue",IF(C12-$E$2&lt;=30,"0-30",IF(C12-$E$2&lt;=60,"31-60",IF(C12-$E$2&lt;=90,"61-90","&gt;90")))),Probability!$B$4:$F$4,0)),0)</f>
         <v>0.75</v>
       </c>
-      <c r="AH12" s="23" t="n">
+      <c r="AH12" s="24" t="n">
         <f aca="false">S12*AG12</f>
         <v>26250</v>
       </c>
+      <c r="AI12" s="22" t="n">
+        <f aca="false">IF(I12&lt;=O12,INDEX(Probability!$B$5:$F$19,MATCH(G12,Probability!$A$5:$A$19,0),MATCH(IF(C12-$E$2&lt;0,"Overdue",IF(C12-$E$2&lt;=30,"0-30",IF(C12-$E$2&lt;=60,"31-60",IF(C12-$E$2&lt;=90,"61-90","&gt;90")))),Probability!$B$4:$F$4,0)),0)</f>
+        <v>0.1</v>
+      </c>
+      <c r="AJ12" s="25" t="n">
+        <f aca="false">S12*AI12</f>
+        <v>3500</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="15" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B13" s="16" t="n">
         <v>46000</v>
@@ -3376,19 +3512,19 @@
         <v>46365</v>
       </c>
       <c r="D13" s="18" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="E13" s="19" t="n">
         <v>0</v>
       </c>
       <c r="F13" s="18" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="G13" s="18" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="H13" s="20" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="I13" s="17" t="n">
         <v>46365</v>
@@ -3442,10 +3578,10 @@
         <v>On time</v>
       </c>
       <c r="V13" s="20" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="W13" s="18" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="X13" s="17" t="n">
         <v>46322</v>
@@ -3454,10 +3590,10 @@
         <v>7</v>
       </c>
       <c r="Z13" s="20" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="AA13" s="20" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="AB13" s="20"/>
       <c r="AC13" s="18"/>
@@ -3470,20 +3606,28 @@
         <v/>
       </c>
       <c r="AF13" s="20" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="AG13" s="22" t="n">
         <f aca="false">IF(I13&lt;=O13,INDEX(Probability!$B$5:$F$19,MATCH(AF13,Probability!$A$5:$A$19,0),MATCH(IF(C13-$E$2&lt;0,"Overdue",IF(C13-$E$2&lt;=30,"0-30",IF(C13-$E$2&lt;=60,"31-60",IF(C13-$E$2&lt;=90,"61-90","&gt;90")))),Probability!$B$4:$F$4,0)),0)</f>
         <v>0.7</v>
       </c>
-      <c r="AH13" s="23" t="n">
+      <c r="AH13" s="24" t="n">
         <f aca="false">S13*AG13</f>
         <v>32200</v>
       </c>
+      <c r="AI13" s="22" t="n">
+        <f aca="false">IF(I13&lt;=O13,INDEX(Probability!$B$5:$F$19,MATCH(G13,Probability!$A$5:$A$19,0),MATCH(IF(C13-$E$2&lt;0,"Overdue",IF(C13-$E$2&lt;=30,"0-30",IF(C13-$E$2&lt;=60,"31-60",IF(C13-$E$2&lt;=90,"61-90","&gt;90")))),Probability!$B$4:$F$4,0)),0)</f>
+        <v>0.35</v>
+      </c>
+      <c r="AJ13" s="25" t="n">
+        <f aca="false">S13*AI13</f>
+        <v>16100</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="15" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B14" s="16" t="n">
         <v>40000</v>
@@ -3492,19 +3636,19 @@
         <v>46375</v>
       </c>
       <c r="D14" s="18" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="E14" s="19" t="n">
         <v>-0.2</v>
       </c>
       <c r="F14" s="18" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="G14" s="18" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="H14" s="20" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="I14" s="17" t="n">
         <v>46375</v>
@@ -3558,10 +3702,10 @@
         <v>On time</v>
       </c>
       <c r="V14" s="20" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="W14" s="18" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="X14" s="17" t="n">
         <v>46325</v>
@@ -3570,10 +3714,10 @@
         <v>10</v>
       </c>
       <c r="Z14" s="20" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="AA14" s="20" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="AB14" s="20"/>
       <c r="AC14" s="18" t="n">
@@ -3588,60 +3732,72 @@
         <v>Under-usage: flag CSM; set At risk</v>
       </c>
       <c r="AF14" s="20" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="AG14" s="22" t="n">
         <f aca="false">IF(I14&lt;=O14,INDEX(Probability!$B$5:$F$19,MATCH(AF14,Probability!$A$5:$A$19,0),MATCH(IF(C14-$E$2&lt;0,"Overdue",IF(C14-$E$2&lt;=30,"0-30",IF(C14-$E$2&lt;=60,"31-60",IF(C14-$E$2&lt;=90,"61-90","&gt;90")))),Probability!$B$4:$F$4,0)),0)</f>
         <v>0.4</v>
       </c>
-      <c r="AH14" s="23" t="n">
+      <c r="AH14" s="24" t="n">
         <f aca="false">S14*AG14</f>
         <v>12800</v>
       </c>
+      <c r="AI14" s="22" t="n">
+        <f aca="false">IF(I14&lt;=O14,INDEX(Probability!$B$5:$F$19,MATCH(G14,Probability!$A$5:$A$19,0),MATCH(IF(C14-$E$2&lt;0,"Overdue",IF(C14-$E$2&lt;=30,"0-30",IF(C14-$E$2&lt;=60,"31-60",IF(C14-$E$2&lt;=90,"61-90","&gt;90")))),Probability!$B$4:$F$4,0)),0)</f>
+        <v>0.4</v>
+      </c>
+      <c r="AJ14" s="25" t="n">
+        <f aca="false">S14*AI14</f>
+        <v>12800</v>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>137</v>
-      </c>
-      <c r="B15" s="24" t="n">
+        <v>139</v>
+      </c>
+      <c r="B15" s="26" t="n">
         <f aca="false">SUM(B5:B14)</f>
         <v>375000</v>
       </c>
-      <c r="S15" s="24" t="n">
+      <c r="S15" s="26" t="n">
         <f aca="false">SUM(S5:S14)</f>
         <v>348400</v>
       </c>
-      <c r="T15" s="24" t="n">
+      <c r="T15" s="26" t="n">
         <f aca="false">SUM(T5:T14)</f>
         <v>132800</v>
       </c>
-      <c r="AH15" s="24" t="n">
+      <c r="AH15" s="26" t="n">
         <f aca="false">SUM(AH5:AH14)</f>
         <v>245130</v>
       </c>
+      <c r="AJ15" s="26" t="n">
+        <f aca="false">SUM(AJ5:AJ14)</f>
+        <v>119300</v>
+      </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="25" t="s">
-        <v>138</v>
+      <c r="A18" s="27" t="s">
+        <v>140</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="26" t="s">
-        <v>139</v>
-      </c>
-      <c r="B19" s="26" t="s">
+      <c r="A19" s="28" t="s">
+        <v>141</v>
+      </c>
+      <c r="B19" s="28" t="s">
         <v>62</v>
       </c>
-      <c r="C19" s="26" t="s">
-        <v>140</v>
-      </c>
-      <c r="D19" s="26" t="s">
-        <v>141</v>
+      <c r="C19" s="28" t="s">
+        <v>142</v>
+      </c>
+      <c r="D19" s="28" t="s">
+        <v>143</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="15" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="B20" s="23" t="n">
         <f aca="false">SUMIFS(T5:T14,U5:U14,"On time")</f>
@@ -3658,7 +3814,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="15" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="B21" s="23" t="n">
         <f aca="false">SUMIFS(T5:T14,U5:U14,"Late")</f>
@@ -3675,7 +3831,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="15" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="B22" s="23" t="n">
         <f aca="false">SUMIFS(T5:T14,U5:U14,"Slips quarter")</f>
@@ -3692,9 +3848,9 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="7" t="s">
-        <v>145</v>
-      </c>
-      <c r="B23" s="27" t="n">
+        <v>147</v>
+      </c>
+      <c r="B23" s="29" t="n">
         <f aca="false">SUM(B20:B22)</f>
         <v>132800</v>
       </c>
@@ -3702,88 +3858,115 @@
         <f aca="false">SUM(C20:C22)</f>
         <v>348400</v>
       </c>
-      <c r="D23" s="28"/>
+      <c r="D23" s="30"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="2" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="15" t="s">
-        <v>147</v>
-      </c>
-      <c r="B25" s="29" t="n">
+        <v>149</v>
+      </c>
+      <c r="B25" s="31" t="n">
         <f aca="false">'Opp summary'!E15</f>
         <v>-23000</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="15" t="s">
-        <v>148</v>
-      </c>
-      <c r="B26" s="29" t="n">
+        <v>150</v>
+      </c>
+      <c r="B26" s="31" t="n">
         <f aca="false">'Opp summary'!F15</f>
         <v>0</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="15" t="s">
-        <v>149</v>
-      </c>
-      <c r="B27" s="29" t="n">
+        <v>151</v>
+      </c>
+      <c r="B27" s="31" t="n">
         <f aca="false">'Opp summary'!H15</f>
         <v>-3600</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="15" t="s">
-        <v>150</v>
-      </c>
-      <c r="B28" s="30" t="n">
+        <v>152</v>
+      </c>
+      <c r="B28" s="32" t="n">
         <f aca="false">(B15+B25+B27)/B15</f>
         <v>0.929066666666667</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="15" t="s">
-        <v>151</v>
-      </c>
-      <c r="B29" s="30" t="n">
+        <v>153</v>
+      </c>
+      <c r="B29" s="32" t="n">
         <f aca="false">S15/B15</f>
         <v>0.929066666666667</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="25" t="s">
+      <c r="A31" s="27" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="15" t="s">
-        <v>152</v>
-      </c>
-      <c r="B32" s="27" t="n">
+        <v>154</v>
+      </c>
+      <c r="B32" s="29" t="n">
         <f aca="false">T15</f>
         <v>132800</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="15" t="s">
-        <v>153</v>
-      </c>
-      <c r="B33" s="27" t="n">
+        <v>155</v>
+      </c>
+      <c r="B33" s="33" t="n">
         <f aca="false">AH15</f>
         <v>245130</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="15" t="s">
-        <v>154</v>
-      </c>
-      <c r="B34" s="27" t="n">
+        <v>156</v>
+      </c>
+      <c r="B34" s="33" t="n">
         <f aca="false">B33-B32</f>
         <v>112330</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="15" t="s">
+        <v>157</v>
+      </c>
+      <c r="B35" s="34" t="n">
+        <f aca="false">AJ15</f>
+        <v>119300</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="15" t="s">
+        <v>158</v>
+      </c>
+      <c r="B36" s="34" t="n">
+        <f aca="false">B35-B32</f>
+        <v>-13500</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="15" t="s">
+        <v>159</v>
+      </c>
+      <c r="B37" s="33" t="n">
+        <f aca="false">B33-B35</f>
+        <v>125830</v>
       </c>
     </row>
   </sheetData>
@@ -3915,92 +4098,92 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="31" t="s">
-        <v>156</v>
-      </c>
-      <c r="B2" s="31"/>
-      <c r="C2" s="31"/>
-      <c r="D2" s="31"/>
-      <c r="E2" s="31"/>
-      <c r="F2" s="31"/>
-      <c r="G2" s="31"/>
-      <c r="H2" s="31"/>
-      <c r="I2" s="31"/>
-      <c r="J2" s="31"/>
-      <c r="K2" s="31"/>
-      <c r="L2" s="31"/>
-      <c r="M2" s="31"/>
-      <c r="N2" s="31"/>
+      <c r="A2" s="35" t="s">
+        <v>161</v>
+      </c>
+      <c r="B2" s="35"/>
+      <c r="C2" s="35"/>
+      <c r="D2" s="35"/>
+      <c r="E2" s="35"/>
+      <c r="F2" s="35"/>
+      <c r="G2" s="35"/>
+      <c r="H2" s="35"/>
+      <c r="I2" s="35"/>
+      <c r="J2" s="35"/>
+      <c r="K2" s="35"/>
+      <c r="L2" s="35"/>
+      <c r="M2" s="35"/>
+      <c r="N2" s="35"/>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>157</v>
+        <v>162</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>159</v>
+        <v>164</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>160</v>
+        <v>165</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>161</v>
+        <v>166</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>164</v>
+        <v>169</v>
       </c>
       <c r="I4" s="6" t="s">
-        <v>165</v>
+        <v>170</v>
       </c>
       <c r="J4" s="6" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="K4" s="6" t="s">
         <v>61</v>
       </c>
       <c r="L4" s="6" t="s">
-        <v>167</v>
+        <v>172</v>
       </c>
       <c r="M4" s="6" t="s">
-        <v>168</v>
+        <v>173</v>
       </c>
       <c r="N4" s="6" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
       <c r="O4" s="6" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="P4" s="6" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="15" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B5" s="15" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="C5" s="18" t="s">
-        <v>173</v>
+        <v>178</v>
       </c>
       <c r="D5" s="18" t="n">
         <v>1</v>
       </c>
       <c r="E5" s="18" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="F5" s="23" t="n">
         <v>21000</v>
@@ -4039,24 +4222,24 @@
         <v>n/a</v>
       </c>
       <c r="P5" s="15" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="15" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B6" s="15" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="C6" s="18" t="s">
-        <v>173</v>
+        <v>178</v>
       </c>
       <c r="D6" s="18" t="n">
         <v>1</v>
       </c>
       <c r="E6" s="18" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="F6" s="23" t="n">
         <v>48000</v>
@@ -4095,24 +4278,24 @@
         <v>n/a</v>
       </c>
       <c r="P6" s="15" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="15" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B7" s="15" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="C7" s="18" t="s">
-        <v>173</v>
+        <v>178</v>
       </c>
       <c r="D7" s="18" t="n">
         <v>1</v>
       </c>
       <c r="E7" s="18" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="F7" s="23" t="n">
         <v>26000</v>
@@ -4151,24 +4334,24 @@
         <v>n/a</v>
       </c>
       <c r="P7" s="15" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="15" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B8" s="15" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="C8" s="18" t="s">
-        <v>180</v>
+        <v>185</v>
       </c>
       <c r="D8" s="18" t="n">
         <v>1</v>
       </c>
       <c r="E8" s="18" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="F8" s="23" t="n">
         <v>45000</v>
@@ -4207,24 +4390,24 @@
         <v>n/a</v>
       </c>
       <c r="P8" s="15" t="s">
-        <v>181</v>
+        <v>186</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="15" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B9" s="15" t="s">
-        <v>182</v>
+        <v>187</v>
       </c>
       <c r="C9" s="18" t="s">
-        <v>173</v>
+        <v>178</v>
       </c>
       <c r="D9" s="18" t="n">
         <v>2</v>
       </c>
       <c r="E9" s="18" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="F9" s="23" t="n">
         <v>36000</v>
@@ -4263,24 +4446,24 @@
         <v>5% a year</v>
       </c>
       <c r="P9" s="15" t="s">
-        <v>183</v>
+        <v>188</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="15" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B10" s="15" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="C10" s="18" t="s">
-        <v>173</v>
+        <v>178</v>
       </c>
       <c r="D10" s="18" t="n">
         <v>1</v>
       </c>
       <c r="E10" s="18" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="F10" s="23" t="n">
         <v>50000</v>
@@ -4322,19 +4505,19 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="15" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B11" s="15" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="C11" s="18" t="s">
-        <v>173</v>
+        <v>178</v>
       </c>
       <c r="D11" s="18" t="n">
         <v>1</v>
       </c>
       <c r="E11" s="18" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="F11" s="23" t="n">
         <v>28000</v>
@@ -4373,24 +4556,24 @@
         <v>n/a</v>
       </c>
       <c r="P11" s="15" t="s">
-        <v>184</v>
+        <v>189</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="15" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B12" s="15" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="C12" s="18" t="s">
-        <v>173</v>
+        <v>178</v>
       </c>
       <c r="D12" s="18" t="n">
         <v>1</v>
       </c>
       <c r="E12" s="18" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="F12" s="23" t="n">
         <v>35000</v>
@@ -4429,24 +4612,24 @@
         <v>n/a</v>
       </c>
       <c r="P12" s="15" t="s">
-        <v>185</v>
+        <v>190</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="15" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B13" s="15" t="s">
-        <v>186</v>
+        <v>191</v>
       </c>
       <c r="C13" s="18" t="s">
-        <v>187</v>
+        <v>192</v>
       </c>
       <c r="D13" s="18" t="n">
         <v>1</v>
       </c>
       <c r="E13" s="18" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="F13" s="23" t="n">
         <v>0</v>
@@ -4485,24 +4668,24 @@
         <v>n/a</v>
       </c>
       <c r="P13" s="15" t="s">
-        <v>188</v>
+        <v>193</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="15" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B14" s="15" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="C14" s="18" t="s">
-        <v>173</v>
+        <v>178</v>
       </c>
       <c r="D14" s="18" t="n">
         <v>1</v>
       </c>
       <c r="E14" s="18" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="F14" s="23" t="n">
         <v>46000</v>
@@ -4544,19 +4727,19 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="15" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B15" s="15" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="C15" s="18" t="s">
-        <v>180</v>
+        <v>185</v>
       </c>
       <c r="D15" s="18" t="n">
         <v>1</v>
       </c>
       <c r="E15" s="18" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="F15" s="23" t="n">
         <v>40000</v>
@@ -4595,58 +4778,58 @@
         <v>n/a</v>
       </c>
       <c r="P15" s="15" t="s">
-        <v>189</v>
+        <v>194</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>137</v>
-      </c>
-      <c r="F17" s="24" t="n">
+        <v>139</v>
+      </c>
+      <c r="F17" s="26" t="n">
         <f aca="false">SUM(F5:F15)</f>
         <v>375000</v>
       </c>
-      <c r="G17" s="24" t="n">
+      <c r="G17" s="26" t="n">
         <f aca="false">SUM(G5:G15)</f>
         <v>-23000</v>
       </c>
-      <c r="J17" s="24" t="n">
+      <c r="J17" s="26" t="n">
         <f aca="false">SUM(J5:J15)</f>
         <v>352000</v>
       </c>
-      <c r="K17" s="24" t="n">
+      <c r="K17" s="26" t="n">
         <f aca="false">SUM(K5:K15)</f>
         <v>348400</v>
       </c>
-      <c r="L17" s="24" t="n">
+      <c r="L17" s="26" t="n">
         <f aca="false">SUM(L5:L15)</f>
         <v>-26600</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>190</v>
+        <v>195</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="31" t="s">
-        <v>191</v>
-      </c>
-      <c r="B20" s="31"/>
-      <c r="C20" s="31"/>
-      <c r="D20" s="31"/>
-      <c r="E20" s="31"/>
-      <c r="F20" s="31"/>
-      <c r="G20" s="31"/>
-      <c r="H20" s="31"/>
-      <c r="I20" s="31"/>
-      <c r="J20" s="31"/>
-      <c r="K20" s="31"/>
-      <c r="L20" s="31"/>
-      <c r="M20" s="31"/>
-      <c r="N20" s="31"/>
-      <c r="O20" s="31"/>
-      <c r="P20" s="31"/>
+      <c r="A20" s="35" t="s">
+        <v>196</v>
+      </c>
+      <c r="B20" s="35"/>
+      <c r="C20" s="35"/>
+      <c r="D20" s="35"/>
+      <c r="E20" s="35"/>
+      <c r="F20" s="35"/>
+      <c r="G20" s="35"/>
+      <c r="H20" s="35"/>
+      <c r="I20" s="35"/>
+      <c r="J20" s="35"/>
+      <c r="K20" s="35"/>
+      <c r="L20" s="35"/>
+      <c r="M20" s="35"/>
+      <c r="N20" s="35"/>
+      <c r="O20" s="35"/>
+      <c r="P20" s="35"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -4708,46 +4891,46 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>192</v>
+        <v>197</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="s">
-        <v>157</v>
+        <v>162</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>193</v>
+        <v>198</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>194</v>
+        <v>199</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>195</v>
+        <v>200</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>196</v>
+        <v>201</v>
       </c>
       <c r="G3" s="6" t="s">
-        <v>197</v>
+        <v>202</v>
       </c>
       <c r="H3" s="6" t="s">
-        <v>198</v>
+        <v>203</v>
       </c>
       <c r="I3" s="6" t="s">
         <v>61</v>
       </c>
       <c r="J3" s="6" t="s">
-        <v>199</v>
+        <v>204</v>
       </c>
       <c r="K3" s="6" t="s">
-        <v>200</v>
+        <v>205</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="32" t="str">
+      <c r="A4" s="36" t="str">
         <f aca="false">Pipeline!A5</f>
         <v>Vantage Freight</v>
       </c>
@@ -4787,7 +4970,7 @@
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="32" t="str">
+      <c r="A5" s="36" t="str">
         <f aca="false">Pipeline!A6</f>
         <v>Northwind Logistics</v>
       </c>
@@ -4827,7 +5010,7 @@
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="32" t="str">
+      <c r="A6" s="36" t="str">
         <f aca="false">Pipeline!A7</f>
         <v>Pixelforge</v>
       </c>
@@ -4867,7 +5050,7 @@
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="32" t="str">
+      <c r="A7" s="36" t="str">
         <f aca="false">Pipeline!A8</f>
         <v>Halden Health</v>
       </c>
@@ -4888,10 +5071,10 @@
         <v>-15000</v>
       </c>
       <c r="F7" s="18" t="s">
-        <v>201</v>
+        <v>206</v>
       </c>
       <c r="G7" s="18" t="s">
-        <v>202</v>
+        <v>207</v>
       </c>
       <c r="H7" s="23" t="n">
         <f aca="false">MIN(0,C7-(SUMIFS(Products!$J:$J,Products!$A:$A,$A7)-SUMIFS(Products!$K:$K,Products!$A:$A,$A7)))</f>
@@ -4911,7 +5094,7 @@
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="32" t="str">
+      <c r="A8" s="36" t="str">
         <f aca="false">Pipeline!A9</f>
         <v>Brightloop</v>
       </c>
@@ -4951,7 +5134,7 @@
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="32" t="str">
+      <c r="A9" s="36" t="str">
         <f aca="false">Pipeline!A10</f>
         <v>Tessera Finance</v>
       </c>
@@ -4991,7 +5174,7 @@
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="32" t="str">
+      <c r="A10" s="36" t="str">
         <f aca="false">Pipeline!A11</f>
         <v>Lumen Retail</v>
       </c>
@@ -5031,7 +5214,7 @@
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="32" t="str">
+      <c r="A11" s="36" t="str">
         <f aca="false">Pipeline!A12</f>
         <v>Kestrel Analytics</v>
       </c>
@@ -5071,7 +5254,7 @@
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="32" t="str">
+      <c r="A12" s="36" t="str">
         <f aca="false">Pipeline!A13</f>
         <v>Marlowe Insurance</v>
       </c>
@@ -5111,7 +5294,7 @@
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="32" t="str">
+      <c r="A13" s="36" t="str">
         <f aca="false">Pipeline!A14</f>
         <v>Quanta Labs</v>
       </c>
@@ -5132,10 +5315,10 @@
         <v>-8000</v>
       </c>
       <c r="F13" s="18" t="s">
-        <v>201</v>
+        <v>206</v>
       </c>
       <c r="G13" s="18" t="s">
-        <v>203</v>
+        <v>208</v>
       </c>
       <c r="H13" s="23" t="n">
         <f aca="false">MIN(0,C13-(SUMIFS(Products!$J:$J,Products!$A:$A,$A13)-SUMIFS(Products!$K:$K,Products!$A:$A,$A13)))</f>
@@ -5156,78 +5339,78 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>137</v>
-      </c>
-      <c r="B14" s="24" t="n">
+        <v>139</v>
+      </c>
+      <c r="B14" s="26" t="n">
         <f aca="false">SUM(B4:B13)</f>
         <v>375000</v>
       </c>
-      <c r="C14" s="24" t="n">
+      <c r="C14" s="26" t="n">
         <f aca="false">SUM(C4:C13)</f>
         <v>0</v>
       </c>
-      <c r="D14" s="24" t="n">
+      <c r="D14" s="26" t="n">
         <f aca="false">SUM(D4:D13)</f>
         <v>0</v>
       </c>
-      <c r="E14" s="24" t="n">
+      <c r="E14" s="26" t="n">
         <f aca="false">SUM(E4:E13)</f>
         <v>-23000</v>
       </c>
-      <c r="H14" s="24" t="n">
+      <c r="H14" s="26" t="n">
         <f aca="false">SUM(H4:H13)</f>
         <v>-3600</v>
       </c>
-      <c r="I14" s="24" t="n">
+      <c r="I14" s="26" t="n">
         <f aca="false">SUM(I4:I13)</f>
         <v>348400</v>
       </c>
-      <c r="J14" s="24" t="n">
+      <c r="J14" s="26" t="n">
         <f aca="false">SUM(J4:J13)</f>
         <v>-26600</v>
       </c>
-      <c r="K14" s="33" t="n">
+      <c r="K14" s="37" t="n">
         <f aca="false">IF(B14=0,0,J14/B14)</f>
         <v>-0.0709333333333333</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="34" t="s">
-        <v>204</v>
-      </c>
-      <c r="E15" s="35" t="n">
+      <c r="A15" s="38" t="s">
+        <v>209</v>
+      </c>
+      <c r="E15" s="39" t="n">
         <f aca="false">SUMIFS(E4:E13,F4:F13,"Regrettable")</f>
         <v>-23000</v>
       </c>
-      <c r="F15" s="35" t="n">
+      <c r="F15" s="39" t="n">
         <f aca="false">SUMIFS(E4:E13,F4:F13,"Non-regrettable")</f>
         <v>0</v>
       </c>
-      <c r="H15" s="35" t="n">
+      <c r="H15" s="39" t="n">
         <f aca="false">H14</f>
         <v>-3600</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>205</v>
-      </c>
-      <c r="B16" s="31" t="s">
-        <v>206</v>
-      </c>
-      <c r="C16" s="31"/>
-      <c r="D16" s="31"/>
-      <c r="E16" s="31"/>
-      <c r="F16" s="31"/>
-      <c r="G16" s="31"/>
-      <c r="H16" s="31"/>
-      <c r="I16" s="31"/>
-      <c r="J16" s="31"/>
-      <c r="K16" s="31"/>
+        <v>210</v>
+      </c>
+      <c r="B16" s="35" t="s">
+        <v>211</v>
+      </c>
+      <c r="C16" s="35"/>
+      <c r="D16" s="35"/>
+      <c r="E16" s="35"/>
+      <c r="F16" s="35"/>
+      <c r="G16" s="35"/>
+      <c r="H16" s="35"/>
+      <c r="I16" s="35"/>
+      <c r="J16" s="35"/>
+      <c r="K16" s="35"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>207</v>
+        <v>212</v>
       </c>
       <c r="B17" s="12" t="str">
         <f aca="false">COUNTIFS(E4:E13,"&lt;0",F4:F13,"")&amp;" opportunities with churn but no category"</f>
@@ -5236,7 +5419,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="12" t="s">
-        <v>208</v>
+        <v>213</v>
       </c>
       <c r="B18" s="12" t="str">
         <f aca="false">IF(ABS(I14-Pipeline!S15)&lt;1,"OK","MISMATCH")</f>
@@ -5300,7 +5483,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>209</v>
+        <v>214</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5311,7 +5494,7 @@
         <v>56</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>210</v>
+        <v>215</v>
       </c>
       <c r="D3" s="6" t="s">
         <v>47</v>
@@ -5320,27 +5503,27 @@
         <v>61</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>211</v>
+        <v>216</v>
       </c>
       <c r="G3" s="6" t="s">
-        <v>212</v>
+        <v>217</v>
       </c>
       <c r="H3" s="6" t="s">
-        <v>213</v>
+        <v>218</v>
       </c>
       <c r="I3" s="6" t="s">
-        <v>214</v>
+        <v>219</v>
       </c>
       <c r="J3" s="6" t="s">
-        <v>215</v>
+        <v>220</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="15" t="s">
-        <v>216</v>
+        <v>221</v>
       </c>
       <c r="B4" s="15" t="s">
-        <v>217</v>
+        <v>222</v>
       </c>
       <c r="C4" s="15" t="n">
         <f aca="false">COUNTIFS(Pipeline!$M$5:$M$14,B4)</f>
@@ -5377,10 +5560,10 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="15" t="s">
-        <v>216</v>
+        <v>221</v>
       </c>
       <c r="B5" s="15" t="s">
-        <v>218</v>
+        <v>223</v>
       </c>
       <c r="C5" s="15" t="n">
         <f aca="false">COUNTIFS(Pipeline!$M$5:$M$14,B5)</f>
@@ -5417,10 +5600,10 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="15" t="s">
-        <v>216</v>
+        <v>221</v>
       </c>
       <c r="B6" s="15" t="s">
-        <v>219</v>
+        <v>224</v>
       </c>
       <c r="C6" s="15" t="n">
         <f aca="false">COUNTIFS(Pipeline!$M$5:$M$14,B6)</f>
@@ -5457,37 +5640,37 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>220</v>
+        <v>225</v>
       </c>
       <c r="C7" s="2" t="n">
         <f aca="false">SUM(C4:C6)</f>
         <v>10</v>
       </c>
-      <c r="D7" s="24" t="n">
+      <c r="D7" s="26" t="n">
         <f aca="false">SUM(D4:D6)</f>
         <v>375000</v>
       </c>
-      <c r="E7" s="24" t="n">
+      <c r="E7" s="26" t="n">
         <f aca="false">SUM(E4:E6)</f>
         <v>348400</v>
       </c>
-      <c r="F7" s="24" t="n">
+      <c r="F7" s="26" t="n">
         <f aca="false">SUM(F4:F6)</f>
         <v>132800</v>
       </c>
-      <c r="G7" s="24" t="n">
+      <c r="G7" s="26" t="n">
         <f aca="false">SUM(G4:G6)</f>
         <v>71700</v>
       </c>
-      <c r="H7" s="24" t="n">
+      <c r="H7" s="26" t="n">
         <f aca="false">SUM(H4:H6)</f>
         <v>61100</v>
       </c>
-      <c r="I7" s="24" t="n">
+      <c r="I7" s="26" t="n">
         <f aca="false">SUM(I4:I6)</f>
         <v>21000</v>
       </c>
-      <c r="J7" s="24" t="n">
+      <c r="J7" s="26" t="n">
         <f aca="false">SUM(J4:J6)</f>
         <v>-23000</v>
       </c>
@@ -5529,12 +5712,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>222</v>
+        <v>227</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5542,474 +5725,474 @@
         <v>34</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>223</v>
+        <v>228</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>224</v>
+        <v>229</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>225</v>
+        <v>230</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>226</v>
+        <v>231</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>227</v>
+        <v>232</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>228</v>
+        <v>233</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>229</v>
+        <v>234</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>230</v>
-      </c>
-      <c r="B5" s="36" t="n">
-        <v>0</v>
-      </c>
-      <c r="C5" s="36" t="n">
-        <v>0</v>
-      </c>
-      <c r="D5" s="36" t="n">
-        <v>0</v>
-      </c>
-      <c r="E5" s="36" t="n">
-        <v>0</v>
-      </c>
-      <c r="F5" s="36" t="n">
+        <v>235</v>
+      </c>
+      <c r="B5" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" s="40" t="n">
         <v>0</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>231</v>
+        <v>236</v>
       </c>
       <c r="H5" s="15" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>99</v>
-      </c>
-      <c r="B6" s="36" t="n">
+        <v>101</v>
+      </c>
+      <c r="B6" s="40" t="n">
         <v>0.05</v>
       </c>
-      <c r="C6" s="36" t="n">
+      <c r="C6" s="40" t="n">
         <v>0.1</v>
       </c>
-      <c r="D6" s="36" t="n">
+      <c r="D6" s="40" t="n">
         <v>0.2</v>
       </c>
-      <c r="E6" s="36" t="n">
+      <c r="E6" s="40" t="n">
         <v>0.3</v>
       </c>
-      <c r="F6" s="36" t="n">
+      <c r="F6" s="40" t="n">
         <v>0.35</v>
       </c>
       <c r="G6" s="8" t="s">
-        <v>232</v>
+        <v>237</v>
       </c>
       <c r="H6" s="15" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>83</v>
-      </c>
-      <c r="B7" s="36" t="n">
+        <v>85</v>
+      </c>
+      <c r="B7" s="40" t="n">
         <v>0.1</v>
       </c>
-      <c r="C7" s="36" t="n">
+      <c r="C7" s="40" t="n">
         <v>0.25</v>
       </c>
-      <c r="D7" s="36" t="n">
+      <c r="D7" s="40" t="n">
         <v>0.35</v>
       </c>
-      <c r="E7" s="36" t="n">
+      <c r="E7" s="40" t="n">
         <v>0.45</v>
       </c>
-      <c r="F7" s="36" t="n">
+      <c r="F7" s="40" t="n">
         <v>0.5</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>233</v>
+        <v>238</v>
       </c>
       <c r="H7" s="15" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
-        <v>106</v>
-      </c>
-      <c r="B8" s="36" t="n">
+        <v>108</v>
+      </c>
+      <c r="B8" s="40" t="n">
         <v>0.2</v>
       </c>
-      <c r="C8" s="36" t="n">
+      <c r="C8" s="40" t="n">
         <v>0.4</v>
       </c>
-      <c r="D8" s="36" t="n">
+      <c r="D8" s="40" t="n">
         <v>0.5</v>
       </c>
-      <c r="E8" s="36" t="n">
+      <c r="E8" s="40" t="n">
         <v>0.55</v>
       </c>
-      <c r="F8" s="36" t="n">
+      <c r="F8" s="40" t="n">
         <v>0.55</v>
       </c>
       <c r="G8" s="8" t="s">
-        <v>234</v>
+        <v>239</v>
       </c>
       <c r="H8" s="15" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="B9" s="40" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C9" s="40" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="D9" s="40" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="E9" s="40" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="F9" s="40" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="G9" s="8" t="s">
+        <v>240</v>
+      </c>
+      <c r="H9" s="15" t="s">
         <v>73</v>
-      </c>
-      <c r="B9" s="36" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="C9" s="36" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="D9" s="36" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="E9" s="36" t="n">
-        <v>0.65</v>
-      </c>
-      <c r="F9" s="36" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="G9" s="8" t="s">
-        <v>235</v>
-      </c>
-      <c r="H9" s="15" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
-        <v>80</v>
-      </c>
-      <c r="B10" s="36" t="n">
+        <v>82</v>
+      </c>
+      <c r="B10" s="40" t="n">
         <v>0.7</v>
       </c>
-      <c r="C10" s="36" t="n">
+      <c r="C10" s="40" t="n">
         <v>0.9</v>
       </c>
-      <c r="D10" s="36" t="n">
+      <c r="D10" s="40" t="n">
         <v>0.85</v>
       </c>
-      <c r="E10" s="36" t="n">
+      <c r="E10" s="40" t="n">
         <v>0.8</v>
       </c>
-      <c r="F10" s="36" t="n">
+      <c r="F10" s="40" t="n">
         <v>0.75</v>
       </c>
       <c r="G10" s="8" t="s">
-        <v>236</v>
+        <v>241</v>
       </c>
       <c r="H10" s="15" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>88</v>
-      </c>
-      <c r="B11" s="36" t="n">
+        <v>90</v>
+      </c>
+      <c r="B11" s="40" t="n">
         <v>0.95</v>
       </c>
-      <c r="C11" s="36" t="n">
+      <c r="C11" s="40" t="n">
         <v>0.99</v>
       </c>
-      <c r="D11" s="36" t="n">
+      <c r="D11" s="40" t="n">
         <v>0.97</v>
       </c>
-      <c r="E11" s="36" t="n">
+      <c r="E11" s="40" t="n">
         <v>0.95</v>
       </c>
-      <c r="F11" s="36" t="n">
+      <c r="F11" s="40" t="n">
         <v>0.9</v>
       </c>
       <c r="G11" s="8" t="s">
-        <v>237</v>
+        <v>242</v>
       </c>
       <c r="H11" s="15" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>238</v>
-      </c>
-      <c r="B12" s="36" t="n">
+        <v>243</v>
+      </c>
+      <c r="B12" s="40" t="n">
         <v>1</v>
       </c>
-      <c r="C12" s="36" t="n">
+      <c r="C12" s="40" t="n">
         <v>1</v>
       </c>
-      <c r="D12" s="36" t="n">
+      <c r="D12" s="40" t="n">
         <v>1</v>
       </c>
-      <c r="E12" s="36" t="n">
+      <c r="E12" s="40" t="n">
         <v>1</v>
       </c>
-      <c r="F12" s="36" t="n">
+      <c r="F12" s="40" t="n">
         <v>1</v>
       </c>
       <c r="G12" s="8" t="s">
-        <v>239</v>
+        <v>244</v>
       </c>
       <c r="H12" s="15" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
-        <v>240</v>
-      </c>
-      <c r="B13" s="36" t="n">
-        <v>0</v>
-      </c>
-      <c r="C13" s="36" t="n">
-        <v>0</v>
-      </c>
-      <c r="D13" s="36" t="n">
-        <v>0</v>
-      </c>
-      <c r="E13" s="36" t="n">
-        <v>0</v>
-      </c>
-      <c r="F13" s="36" t="n">
+        <v>245</v>
+      </c>
+      <c r="B13" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" s="40" t="n">
         <v>0</v>
       </c>
       <c r="G13" s="8" t="s">
-        <v>241</v>
+        <v>246</v>
       </c>
       <c r="H13" s="15" t="s">
-        <v>242</v>
+        <v>247</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="s">
-        <v>96</v>
-      </c>
-      <c r="B14" s="36" t="n">
+        <v>98</v>
+      </c>
+      <c r="B14" s="40" t="n">
         <v>0.4</v>
       </c>
-      <c r="C14" s="36" t="n">
+      <c r="C14" s="40" t="n">
         <v>0.97</v>
       </c>
-      <c r="D14" s="36" t="n">
+      <c r="D14" s="40" t="n">
         <v>0.95</v>
       </c>
-      <c r="E14" s="36" t="n">
+      <c r="E14" s="40" t="n">
         <v>0.92</v>
       </c>
-      <c r="F14" s="36" t="n">
+      <c r="F14" s="40" t="n">
         <v>0.9</v>
       </c>
       <c r="G14" s="8" t="s">
-        <v>243</v>
+        <v>248</v>
       </c>
       <c r="H14" s="15" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="7" t="s">
-        <v>91</v>
-      </c>
-      <c r="B15" s="36" t="n">
+        <v>93</v>
+      </c>
+      <c r="B15" s="40" t="n">
         <v>0.4</v>
       </c>
-      <c r="C15" s="36" t="n">
+      <c r="C15" s="40" t="n">
         <v>0.6</v>
       </c>
-      <c r="D15" s="36" t="n">
+      <c r="D15" s="40" t="n">
         <v>0.7</v>
       </c>
-      <c r="E15" s="36" t="n">
+      <c r="E15" s="40" t="n">
         <v>0.75</v>
       </c>
-      <c r="F15" s="36" t="n">
+      <c r="F15" s="40" t="n">
         <v>0.8</v>
       </c>
       <c r="G15" s="8" t="s">
-        <v>244</v>
+        <v>249</v>
       </c>
       <c r="H15" s="15" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="s">
-        <v>133</v>
-      </c>
-      <c r="B16" s="36" t="n">
+        <v>135</v>
+      </c>
+      <c r="B16" s="40" t="n">
         <v>0.2</v>
       </c>
-      <c r="C16" s="36" t="n">
+      <c r="C16" s="40" t="n">
         <v>0.35</v>
       </c>
-      <c r="D16" s="36" t="n">
+      <c r="D16" s="40" t="n">
         <v>0.4</v>
       </c>
-      <c r="E16" s="36" t="n">
+      <c r="E16" s="40" t="n">
         <v>0.45</v>
       </c>
-      <c r="F16" s="36" t="n">
+      <c r="F16" s="40" t="n">
         <v>0.5</v>
       </c>
       <c r="G16" s="8" t="s">
-        <v>245</v>
+        <v>250</v>
       </c>
       <c r="H16" s="15" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="s">
-        <v>246</v>
-      </c>
-      <c r="B17" s="36" t="n">
+        <v>251</v>
+      </c>
+      <c r="B17" s="40" t="n">
         <v>0.5</v>
       </c>
-      <c r="C17" s="36" t="n">
+      <c r="C17" s="40" t="n">
         <v>0.8</v>
       </c>
-      <c r="D17" s="36" t="n">
+      <c r="D17" s="40" t="n">
         <v>0.8</v>
       </c>
-      <c r="E17" s="36" t="n">
+      <c r="E17" s="40" t="n">
         <v>0.8</v>
       </c>
-      <c r="F17" s="36" t="n">
+      <c r="F17" s="40" t="n">
         <v>0.8</v>
       </c>
       <c r="G17" s="8" t="s">
-        <v>247</v>
+        <v>252</v>
       </c>
       <c r="H17" s="15" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="7" t="s">
-        <v>248</v>
-      </c>
-      <c r="B18" s="36" t="n">
-        <v>0</v>
-      </c>
-      <c r="C18" s="36" t="n">
+        <v>253</v>
+      </c>
+      <c r="B18" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="40" t="n">
         <v>0.1</v>
       </c>
-      <c r="D18" s="36" t="n">
+      <c r="D18" s="40" t="n">
         <v>0.1</v>
       </c>
-      <c r="E18" s="36" t="n">
+      <c r="E18" s="40" t="n">
         <v>0.1</v>
       </c>
-      <c r="F18" s="36" t="n">
+      <c r="F18" s="40" t="n">
         <v>0.1</v>
       </c>
       <c r="G18" s="8" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="H18" s="15" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="s">
-        <v>250</v>
-      </c>
-      <c r="B19" s="36" t="n">
+        <v>255</v>
+      </c>
+      <c r="B19" s="40" t="n">
         <v>1</v>
       </c>
-      <c r="C19" s="36" t="n">
+      <c r="C19" s="40" t="n">
         <v>1</v>
       </c>
-      <c r="D19" s="36" t="n">
+      <c r="D19" s="40" t="n">
         <v>1</v>
       </c>
-      <c r="E19" s="36" t="n">
+      <c r="E19" s="40" t="n">
         <v>1</v>
       </c>
-      <c r="F19" s="36" t="n">
+      <c r="F19" s="40" t="n">
         <v>1</v>
       </c>
       <c r="G19" s="8" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="H19" s="15" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B21" s="31" t="s">
-        <v>252</v>
-      </c>
-      <c r="C21" s="31"/>
-      <c r="D21" s="31"/>
-      <c r="E21" s="31"/>
-      <c r="F21" s="31"/>
-      <c r="G21" s="31"/>
+      <c r="B21" s="35" t="s">
+        <v>257</v>
+      </c>
+      <c r="C21" s="35"/>
+      <c r="D21" s="35"/>
+      <c r="E21" s="35"/>
+      <c r="F21" s="35"/>
+      <c r="G21" s="35"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B22" s="31"/>
-      <c r="C22" s="31"/>
-      <c r="D22" s="31"/>
-      <c r="E22" s="31"/>
-      <c r="F22" s="31"/>
-      <c r="G22" s="31"/>
+      <c r="B22" s="35"/>
+      <c r="C22" s="35"/>
+      <c r="D22" s="35"/>
+      <c r="E22" s="35"/>
+      <c r="F22" s="35"/>
+      <c r="G22" s="35"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B23" s="31"/>
-      <c r="C23" s="31"/>
-      <c r="D23" s="31"/>
-      <c r="E23" s="31"/>
-      <c r="F23" s="31"/>
-      <c r="G23" s="31"/>
+      <c r="B23" s="35"/>
+      <c r="C23" s="35"/>
+      <c r="D23" s="35"/>
+      <c r="E23" s="35"/>
+      <c r="F23" s="35"/>
+      <c r="G23" s="35"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B25" s="31" t="s">
-        <v>253</v>
-      </c>
-      <c r="C25" s="31"/>
-      <c r="D25" s="31"/>
-      <c r="E25" s="31"/>
-      <c r="F25" s="31"/>
-      <c r="G25" s="31"/>
+      <c r="B25" s="35" t="s">
+        <v>258</v>
+      </c>
+      <c r="C25" s="35"/>
+      <c r="D25" s="35"/>
+      <c r="E25" s="35"/>
+      <c r="F25" s="35"/>
+      <c r="G25" s="35"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B26" s="31"/>
-      <c r="C26" s="31"/>
-      <c r="D26" s="31"/>
-      <c r="E26" s="31"/>
-      <c r="F26" s="31"/>
-      <c r="G26" s="31"/>
+      <c r="B26" s="35"/>
+      <c r="C26" s="35"/>
+      <c r="D26" s="35"/>
+      <c r="E26" s="35"/>
+      <c r="F26" s="35"/>
+      <c r="G26" s="35"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B27" s="31"/>
-      <c r="C27" s="31"/>
-      <c r="D27" s="31"/>
-      <c r="E27" s="31"/>
-      <c r="F27" s="31"/>
-      <c r="G27" s="31"/>
+      <c r="B27" s="35"/>
+      <c r="C27" s="35"/>
+      <c r="D27" s="35"/>
+      <c r="E27" s="35"/>
+      <c r="F27" s="35"/>
+      <c r="G27" s="35"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -6053,95 +6236,95 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>254</v>
+        <v>259</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="s">
-        <v>255</v>
+        <v>260</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>256</v>
+        <v>261</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>257</v>
+        <v>262</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>258</v>
+        <v>263</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>259</v>
+        <v>264</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>260</v>
+        <v>265</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>261</v>
+        <v>266</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>262</v>
+        <v>267</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>263</v>
+        <v>268</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>264</v>
+        <v>269</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>265</v>
+        <v>270</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>267</v>
+        <v>272</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>268</v>
+        <v>273</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>269</v>
+        <v>274</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>180</v>
+        <v>185</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>270</v>
+        <v>275</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>271</v>
+        <v>276</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="8" t="s">
-        <v>272</v>
+        <v>277</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>273</v>
+        <v>278</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>274</v>
+        <v>279</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="8" t="s">
-        <v>275</v>
+        <v>280</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>276</v>
+        <v>281</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>277</v>
+        <v>282</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Clarify how the CSM finds named contacts at Vantage
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CVAHSCDuy4tEBaMUUSRsNB
</commit_message>
<xml_diff>
--- a/n8n-renewals-challenge/renewal_tracker.xlsx
+++ b/n8n-renewals-challenge/renewal_tracker.xlsx
@@ -303,7 +303,7 @@
     <t xml:space="preserve">No named contact (shared inbox)</t>
   </si>
   <si>
-    <t xml:space="preserve">CSM pulls instance owner/admin emails from product data; I call and email the named person and agree a signing date. Manager confirms the grace period before access is restricted.</t>
+    <t xml:space="preserve">CSM looks up the instance owner and admin users (names, emails) in product data, to replace the shared inbox; I call and email the named person and agree a signing date. Manager confirms the grace period before access is restricted.</t>
   </si>
   <si>
     <t xml:space="preserve">Me</t>
@@ -1860,7 +1860,7 @@
       </c>
       <c r="H6" s="8" t="str">
         <f aca="false">INDEX(Pipeline!$V$5:$V$14,MATCH($A6,Pipeline!$Y$5:$Y$14,0))&amp;""</f>
-        <v>CSM pulls instance owner/admin emails from product data; I call and email the named person and agree a signing date. Manager confirms the grace period before access is restricted.</v>
+        <v>CSM looks up the instance owner and admin users (names, emails) in product data, to replace the shared inbox; I call and email the named person and agree a signing date. Manager confirms the grace period before access is restricted.</v>
       </c>
       <c r="I6" s="8" t="str">
         <f aca="false">INDEX(Pipeline!$W$5:$W$14,MATCH($A6,Pipeline!$Y$5:$Y$14,0))</f>

</xml_diff>

<commit_message>
Tessera: drop the current-MSA shortcut; triage redlines, joint call, extension fallback
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CVAHSCDuy4tEBaMUUSRsNB
</commit_message>
<xml_diff>
--- a/n8n-renewals-challenge/renewal_tracker.xlsx
+++ b/n8n-renewals-challenge/renewal_tracker.xlsx
@@ -417,7 +417,7 @@
     <t xml:space="preserve">MSA redlines open since Sep; security review</t>
   </si>
   <si>
-    <t xml:space="preserve">ESCALATE TODAY to Legal: redline response by 30 Oct. Security pack today. Renew on the current MSA and negotiate the MSA in parallel.</t>
+    <t xml:space="preserve">ESCALATE TODAY to Legal: redline response by 30 Oct. List PO-blocking redlines, agree positions; joint redline call. Quote + security pack today. Fallback: 1-2 month extension if MSA not signed by 18 Nov.</t>
   </si>
   <si>
     <t xml:space="preserve">Legal</t>
@@ -429,7 +429,7 @@
     <t xml:space="preserve">Me, Security</t>
   </si>
   <si>
-    <t xml:space="preserve">Yes: Legal lead, redline response by 30 Oct and renew on the current MSA</t>
+    <t xml:space="preserve">Yes: Legal lead, redline response by 30 Oct; extension fallback approved</t>
   </si>
   <si>
     <t xml:space="preserve">Lumen Retail</t>
@@ -2007,7 +2007,7 @@
       </c>
       <c r="H9" s="8" t="str">
         <f aca="false">INDEX(Pipeline!$V$5:$V$14,MATCH($A9,Pipeline!$Y$5:$Y$14,0))&amp;""</f>
-        <v>ESCALATE TODAY to Legal: redline response by 30 Oct. Security pack today. Renew on the current MSA and negotiate the MSA in parallel.</v>
+        <v>ESCALATE TODAY to Legal: redline response by 30 Oct. List PO-blocking redlines, agree positions; joint redline call. Quote + security pack today. Fallback: 1-2 month extension if MSA not signed by 18 Nov.</v>
       </c>
       <c r="I9" s="8" t="str">
         <f aca="false">INDEX(Pipeline!$W$5:$W$14,MATCH($A9,Pipeline!$Y$5:$Y$14,0))</f>
@@ -2023,7 +2023,7 @@
       </c>
       <c r="L9" s="11" t="str">
         <f aca="false">INDEX(Pipeline!$AB$5:$AB$14,MATCH($A9,Pipeline!$Y$5:$Y$14,0))&amp;""</f>
-        <v>Yes: Legal lead, redline response by 30 Oct and renew on the current MSA</v>
+        <v>Yes: Legal lead, redline response by 30 Oct; extension fallback approved</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Kestrel: one quote separating renewal and upsell, after CSM approval
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CVAHSCDuy4tEBaMUUSRsNB
</commit_message>
<xml_diff>
--- a/n8n-renewals-challenge/renewal_tracker.xlsx
+++ b/n8n-renewals-challenge/renewal_tracker.xlsx
@@ -453,7 +453,7 @@
     <t xml:space="preserve">Close to execution cap</t>
   </si>
   <si>
-    <t xml:space="preserve">CSM usage review; quote like-for-like (€35k) and open a linked Upsell opportunity for the next execution tier.</t>
+    <t xml:space="preserve">CSM usage review and approves the tier; one quote with renewal (€35k like-for-like) and upsell (next tier) as separate lines; upsell on its own linked Upsell opportunity.</t>
   </si>
   <si>
     <t xml:space="preserve">Usage +40%, near the execution cap: expansion, and a throttling risk.</t>
@@ -2154,7 +2154,7 @@
       </c>
       <c r="H12" s="8" t="str">
         <f aca="false">INDEX(Pipeline!$V$5:$V$14,MATCH($A12,Pipeline!$Y$5:$Y$14,0))&amp;""</f>
-        <v>CSM usage review; quote like-for-like (€35k) and open a linked Upsell opportunity for the next execution tier.</v>
+        <v>CSM usage review and approves the tier; one quote with renewal (€35k like-for-like) and upsell (next tier) as separate lines; upsell on its own linked Upsell opportunity.</v>
       </c>
       <c r="I12" s="8" t="str">
         <f aca="false">INDEX(Pipeline!$W$5:$W$14,MATCH($A12,Pipeline!$Y$5:$Y$14,0))</f>

</xml_diff>

<commit_message>
Pixelforge: explain the dunning pause in plain words
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CVAHSCDuy4tEBaMUUSRsNB
</commit_message>
<xml_diff>
--- a/n8n-renewals-challenge/renewal_tracker.xlsx
+++ b/n8n-renewals-challenge/renewal_tracker.xlsx
@@ -357,7 +357,7 @@
     <t xml:space="preserve">Card expired; billing contact unknown</t>
   </si>
   <si>
-    <t xml:space="preserve">CSM gets the billing contact today; I send a secure card-update link or switch to invoice; Finance holds dunning. Renews at €26k (renewal value).</t>
+    <t xml:space="preserve">CSM gets the billing contact today; I send a secure card-update link or switch to invoice; Finance pauses the automatic failed-payment process (reminders, retries, suspension) until the card is fixed. Renews at €26k (renewal value).</t>
   </si>
   <si>
     <t xml:space="preserve">Auto-renewal fails in 13 days on an expired card: involuntary churn on a green account.</t>
@@ -1909,7 +1909,7 @@
       </c>
       <c r="H7" s="8" t="str">
         <f aca="false">INDEX(Pipeline!$V$5:$V$14,MATCH($A7,Pipeline!$Y$5:$Y$14,0))&amp;""</f>
-        <v>CSM gets the billing contact today; I send a secure card-update link or switch to invoice; Finance holds dunning. Renews at €26k (renewal value).</v>
+        <v>CSM gets the billing contact today; I send a secure card-update link or switch to invoice; Finance pauses the automatic failed-payment process (reminders, retries, suspension) until the card is fixed. Renews at €26k (renewal value).</v>
       </c>
       <c r="I7" s="8" t="str">
         <f aca="false">INDEX(Pipeline!$W$5:$W$14,MATCH($A7,Pipeline!$Y$5:$Y$14,0))</f>

</xml_diff>

<commit_message>
Triage: show who does what in each action
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CVAHSCDuy4tEBaMUUSRsNB
</commit_message>
<xml_diff>
--- a/n8n-renewals-challenge/renewal_tracker.xlsx
+++ b/n8n-renewals-challenge/renewal_tracker.xlsx
@@ -70,7 +70,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="408" uniqueCount="283">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="408" uniqueCount="286">
   <si>
     <t xml:space="preserve">Renewal tracker: a mock-up of the CRM renewal model</t>
   </si>
@@ -90,7 +90,7 @@
     <t xml:space="preserve">Triage</t>
   </si>
   <si>
-    <t xml:space="preserve">Rank, why first, next action, one owner (Me / CSM / Finance / Legal) plus who else is involved, due date, and today's escalations. Sorted by rank; edit the rank on the Pipeline tab.</t>
+    <t xml:space="preserve">Rank, why first, next action, one lead owner (Me / CSM / Finance / Legal) plus who does what, due date, and today's escalations. Sorted by rank; edit the rank on the Pipeline tab.</t>
   </si>
   <si>
     <t xml:space="preserve">Probability</t>
@@ -186,7 +186,7 @@
     <t xml:space="preserve">Owner</t>
   </si>
   <si>
-    <t xml:space="preserve">Also involved</t>
+    <t xml:space="preserve">Who does what</t>
   </si>
   <si>
     <t xml:space="preserve">Due</t>
@@ -312,7 +312,9 @@
     <t xml:space="preserve">Already overdue. The blocker is a shared inbox, not price: find a named person.</t>
   </si>
   <si>
-    <t xml:space="preserve">CSM, Manager</t>
+    <t xml:space="preserve">CSM: finds the instance owner and admins
+Me: calls them and agrees a signing date
+Manager: confirms the grace period</t>
   </si>
   <si>
     <t xml:space="preserve">Yes: Manager, to agree the grace period before access is restricted</t>
@@ -339,31 +341,36 @@
     <t xml:space="preserve">Biggest near-term ARR, 9 days out, no quote, signed 3 days late last year. One hour of work removes most of the risk.</t>
   </si>
   <si>
+    <t xml:space="preserve">Me: quote, order form, signatory, signature on 27 Oct</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PO received</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pixelforge</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Auto</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Billing blocker</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Card expired; billing contact unknown</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CSM gets the billing contact today; I send a secure card-update link or switch to invoice; Finance pauses the automatic failed-payment process (reminders, retries, suspension) until the card is fixed. Renews at €26k (renewal value).</t>
+  </si>
+  <si>
     <t xml:space="preserve">CSM</t>
   </si>
   <si>
-    <t xml:space="preserve">PO received</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pixelforge</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Auto</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Billing blocker</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Card expired; billing contact unknown</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CSM gets the billing contact today; I send a secure card-update link or switch to invoice; Finance pauses the automatic failed-payment process (reminders, retries, suspension) until the card is fixed. Renews at €26k (renewal value).</t>
-  </si>
-  <si>
     <t xml:space="preserve">Auto-renewal fails in 13 days on an expired card: involuntary churn on a green account.</t>
   </si>
   <si>
-    <t xml:space="preserve">Me, Finance</t>
+    <t xml:space="preserve">CSM: finds the billing contact
+Me: card-update link or switch to invoice
+Finance: pauses the failed-payment process</t>
   </si>
   <si>
     <t xml:space="preserve">Renewing: no blockers</t>
@@ -387,7 +394,10 @@
     <t xml:space="preserve">Red, usage -35%, champion gone, new owner unknown, 18 days left.</t>
   </si>
   <si>
-    <t xml:space="preserve">Me, Manager, VP CS (exec sponsor)</t>
+    <t xml:space="preserve">CSM (lead): meets the new owner, value review
+Exec sponsor: joins that meeting
+Legal: checks the 8 Oct notice date
+Me: escalates, prepares the right-sized option</t>
   </si>
   <si>
     <t xml:space="preserve">Yes: Manager + VP CS, exec sponsor meeting with the new owner this week</t>
@@ -408,7 +418,9 @@
     <t xml:space="preserve">Live negotiation; procurement sets the pace. Reply and pre-approvals today.</t>
   </si>
   <si>
-    <t xml:space="preserve">Finance, Legal, CSM</t>
+    <t xml:space="preserve">Me: reply to Sam, the call, the order form
+Finance: pre-approves up to 12% and net 60
+VP CS: pre-approves the buffer</t>
   </si>
   <si>
     <t xml:space="preserve">Tessera Finance</t>
@@ -426,7 +438,9 @@
     <t xml:space="preserve">MSA redlines open since September and a security review can block the PO; 29 days left.</t>
   </si>
   <si>
-    <t xml:space="preserve">Me, Security</t>
+    <t xml:space="preserve">Legal (lead): positions on PO-blocking redlines, joint call, response by 30 Oct
+Me: redline list, quote and security pack, runs the timeline
+Finance + Legal: approve the extension fallback</t>
   </si>
   <si>
     <t xml:space="preserve">Yes: Legal lead, redline response by 30 Oct; extension fallback approved</t>
@@ -444,7 +458,9 @@
     <t xml:space="preserve">Auto-renewal would invoice the wrong legal entity; cancellation deadline 22 Oct (assumed 30-day notice).</t>
   </si>
   <si>
-    <t xml:space="preserve">Finance, Legal</t>
+    <t xml:space="preserve">Me: gets the new entity's details
+Legal: billing change or assignment
+Finance: updates billing before the invoice run</t>
   </si>
   <si>
     <t xml:space="preserve">Kestrel Analytics</t>
@@ -459,6 +475,10 @@
     <t xml:space="preserve">Usage +40%, near the execution cap: expansion, and a throttling risk.</t>
   </si>
   <si>
+    <t xml:space="preserve">CSM: usage review, approves the tier
+Me: one quote, renewal and upsell on separate lines; upsell opportunity</t>
+  </si>
+  <si>
     <t xml:space="preserve">Marlowe Insurance</t>
   </si>
   <si>
@@ -471,7 +491,9 @@
     <t xml:space="preserve">Insurance procurement is slow; no DPA and questionnaire means no PO.</t>
   </si>
   <si>
-    <t xml:space="preserve">Legal, Security</t>
+    <t xml:space="preserve">Me: quote, questionnaire, PO lead time
+Security: reviews the questionnaire answers
+Legal: the DPA</t>
   </si>
   <si>
     <t xml:space="preserve">Quanta Labs</t>
@@ -487,6 +509,10 @@
   </si>
   <si>
     <t xml:space="preserve">Auto-renewal, usage -20%, Q1 budget cuts, unresponsive. 60 days, but the notice deadline is ~19 Nov (assumed 30-day notice).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CSM + exec sponsor: reach a new contact
+Me: confirms the notice date, offers the lock or right-size</t>
   </si>
   <si>
     <t xml:space="preserve">Total</t>
@@ -1728,7 +1754,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="42"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="60"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="48"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="40"/>
   </cols>
@@ -1819,7 +1845,7 @@
       </c>
       <c r="J5" s="8" t="str">
         <f aca="false">INDEX(Pipeline!$AA$5:$AA$14,MATCH($A5,Pipeline!$Y$5:$Y$14,0))&amp;""</f>
-        <v>CSM</v>
+        <v>Me: quote, order form, signatory, signature on 27 Oct</v>
       </c>
       <c r="K5" s="10" t="n">
         <f aca="false">INDEX(Pipeline!$X$5:$X$14,MATCH($A5,Pipeline!$Y$5:$Y$14,0))</f>
@@ -1868,7 +1894,9 @@
       </c>
       <c r="J6" s="8" t="str">
         <f aca="false">INDEX(Pipeline!$AA$5:$AA$14,MATCH($A6,Pipeline!$Y$5:$Y$14,0))&amp;""</f>
-        <v>CSM, Manager</v>
+        <v>CSM: finds the instance owner and admins
+Me: calls them and agrees a signing date
+Manager: confirms the grace period</v>
       </c>
       <c r="K6" s="10" t="n">
         <f aca="false">INDEX(Pipeline!$X$5:$X$14,MATCH($A6,Pipeline!$Y$5:$Y$14,0))</f>
@@ -1917,7 +1945,9 @@
       </c>
       <c r="J7" s="8" t="str">
         <f aca="false">INDEX(Pipeline!$AA$5:$AA$14,MATCH($A7,Pipeline!$Y$5:$Y$14,0))&amp;""</f>
-        <v>Me, Finance</v>
+        <v>CSM: finds the billing contact
+Me: card-update link or switch to invoice
+Finance: pauses the failed-payment process</v>
       </c>
       <c r="K7" s="10" t="n">
         <f aca="false">INDEX(Pipeline!$X$5:$X$14,MATCH($A7,Pipeline!$Y$5:$Y$14,0))</f>
@@ -1966,7 +1996,10 @@
       </c>
       <c r="J8" s="8" t="str">
         <f aca="false">INDEX(Pipeline!$AA$5:$AA$14,MATCH($A8,Pipeline!$Y$5:$Y$14,0))&amp;""</f>
-        <v>Me, Manager, VP CS (exec sponsor)</v>
+        <v>CSM (lead): meets the new owner, value review
+Exec sponsor: joins that meeting
+Legal: checks the 8 Oct notice date
+Me: escalates, prepares the right-sized option</v>
       </c>
       <c r="K8" s="10" t="n">
         <f aca="false">INDEX(Pipeline!$X$5:$X$14,MATCH($A8,Pipeline!$Y$5:$Y$14,0))</f>
@@ -2015,7 +2048,9 @@
       </c>
       <c r="J9" s="8" t="str">
         <f aca="false">INDEX(Pipeline!$AA$5:$AA$14,MATCH($A9,Pipeline!$Y$5:$Y$14,0))&amp;""</f>
-        <v>Me, Security</v>
+        <v>Legal (lead): positions on PO-blocking redlines, joint call, response by 30 Oct
+Me: redline list, quote and security pack, runs the timeline
+Finance + Legal: approve the extension fallback</v>
       </c>
       <c r="K9" s="10" t="n">
         <f aca="false">INDEX(Pipeline!$X$5:$X$14,MATCH($A9,Pipeline!$Y$5:$Y$14,0))</f>
@@ -2064,7 +2099,9 @@
       </c>
       <c r="J10" s="8" t="str">
         <f aca="false">INDEX(Pipeline!$AA$5:$AA$14,MATCH($A10,Pipeline!$Y$5:$Y$14,0))&amp;""</f>
-        <v>Finance, Legal, CSM</v>
+        <v>Me: reply to Sam, the call, the order form
+Finance: pre-approves up to 12% and net 60
+VP CS: pre-approves the buffer</v>
       </c>
       <c r="K10" s="10" t="n">
         <f aca="false">INDEX(Pipeline!$X$5:$X$14,MATCH($A10,Pipeline!$Y$5:$Y$14,0))</f>
@@ -2113,7 +2150,9 @@
       </c>
       <c r="J11" s="8" t="str">
         <f aca="false">INDEX(Pipeline!$AA$5:$AA$14,MATCH($A11,Pipeline!$Y$5:$Y$14,0))&amp;""</f>
-        <v>Legal, Security</v>
+        <v>Me: quote, questionnaire, PO lead time
+Security: reviews the questionnaire answers
+Legal: the DPA</v>
       </c>
       <c r="K11" s="10" t="n">
         <f aca="false">INDEX(Pipeline!$X$5:$X$14,MATCH($A11,Pipeline!$Y$5:$Y$14,0))</f>
@@ -2162,7 +2201,8 @@
       </c>
       <c r="J12" s="8" t="str">
         <f aca="false">INDEX(Pipeline!$AA$5:$AA$14,MATCH($A12,Pipeline!$Y$5:$Y$14,0))&amp;""</f>
-        <v>Me</v>
+        <v>CSM: usage review, approves the tier
+Me: one quote, renewal and upsell on separate lines; upsell opportunity</v>
       </c>
       <c r="K12" s="10" t="n">
         <f aca="false">INDEX(Pipeline!$X$5:$X$14,MATCH($A12,Pipeline!$Y$5:$Y$14,0))</f>
@@ -2211,7 +2251,9 @@
       </c>
       <c r="J13" s="8" t="str">
         <f aca="false">INDEX(Pipeline!$AA$5:$AA$14,MATCH($A13,Pipeline!$Y$5:$Y$14,0))&amp;""</f>
-        <v>Finance, Legal</v>
+        <v>Me: gets the new entity's details
+Legal: billing change or assignment
+Finance: updates billing before the invoice run</v>
       </c>
       <c r="K13" s="10" t="n">
         <f aca="false">INDEX(Pipeline!$X$5:$X$14,MATCH($A13,Pipeline!$Y$5:$Y$14,0))</f>
@@ -2260,7 +2302,8 @@
       </c>
       <c r="J14" s="8" t="str">
         <f aca="false">INDEX(Pipeline!$AA$5:$AA$14,MATCH($A14,Pipeline!$Y$5:$Y$14,0))&amp;""</f>
-        <v>Me</v>
+        <v>CSM + exec sponsor: reach a new contact
+Me: confirms the notice date, offers the lock or right-size</v>
       </c>
       <c r="K14" s="10" t="n">
         <f aca="false">INDEX(Pipeline!$X$5:$X$14,MATCH($A14,Pipeline!$Y$5:$Y$14,0))</f>
@@ -2353,7 +2396,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="24" min="24" style="0" width="12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="25" min="25" style="0" width="7"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="26" style="0" width="50"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="27" min="27" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="27" min="27" style="0" width="48"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="28" min="28" style="0" width="40"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="29" min="29" style="0" width="10"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="30" min="30" style="0" width="13"/>
@@ -2827,7 +2870,7 @@
         <v>95</v>
       </c>
       <c r="W7" s="18" t="s">
-        <v>89</v>
+        <v>96</v>
       </c>
       <c r="X7" s="17" t="n">
         <v>46317</v>
@@ -2836,10 +2879,10 @@
         <v>3</v>
       </c>
       <c r="Z7" s="20" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="AA7" s="20" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AB7" s="20"/>
       <c r="AC7" s="18" t="n">
@@ -2854,7 +2897,7 @@
         <v/>
       </c>
       <c r="AF7" s="20" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="AG7" s="22" t="n">
         <f aca="false">IF(I7&lt;=O7,INDEX(Probability!$B$5:$F$19,MATCH(AF7,Probability!$A$5:$A$19,0),MATCH(IF(C7-$E$2&lt;0,"Overdue",IF(C7-$E$2&lt;=30,"0-30",IF(C7-$E$2&lt;=60,"31-60",IF(C7-$E$2&lt;=90,"61-90","&gt;90")))),Probability!$B$4:$F$4,0)),0)</f>
@@ -2875,7 +2918,7 @@
     </row>
     <row r="8" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="15" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B8" s="16" t="n">
         <v>45000</v>
@@ -2890,13 +2933,13 @@
         <v>-0.35</v>
       </c>
       <c r="F8" s="18" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="G8" s="18" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="H8" s="20" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="I8" s="17" t="n">
         <v>46346</v>
@@ -2950,10 +2993,10 @@
         <v>Late</v>
       </c>
       <c r="V8" s="20" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="W8" s="18" t="s">
-        <v>89</v>
+        <v>96</v>
       </c>
       <c r="X8" s="17" t="n">
         <v>46318</v>
@@ -2962,13 +3005,13 @@
         <v>4</v>
       </c>
       <c r="Z8" s="20" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="AA8" s="20" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="AB8" s="20" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="AC8" s="18" t="n">
         <v>30</v>
@@ -3003,7 +3046,7 @@
     </row>
     <row r="9" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="15" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B9" s="16" t="n">
         <v>36000</v>
@@ -3021,10 +3064,10 @@
         <v>74</v>
       </c>
       <c r="G9" s="18" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="H9" s="20" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="I9" s="17" t="n">
         <v>46356</v>
@@ -3078,7 +3121,7 @@
         <v>On time</v>
       </c>
       <c r="V9" s="20" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="W9" s="18" t="s">
         <v>78</v>
@@ -3090,10 +3133,10 @@
         <v>6</v>
       </c>
       <c r="Z9" s="20" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="AA9" s="20" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="AB9" s="20"/>
       <c r="AC9" s="18"/>
@@ -3106,7 +3149,7 @@
         <v/>
       </c>
       <c r="AF9" s="20" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="AG9" s="22" t="n">
         <f aca="false">IF(I9&lt;=O9,INDEX(Probability!$B$5:$F$19,MATCH(AF9,Probability!$A$5:$A$19,0),MATCH(IF(C9-$E$2&lt;0,"Overdue",IF(C9-$E$2&lt;=30,"0-30",IF(C9-$E$2&lt;=60,"31-60",IF(C9-$E$2&lt;=90,"61-90","&gt;90")))),Probability!$B$4:$F$4,0)),0)</f>
@@ -3127,7 +3170,7 @@
     </row>
     <row r="10" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="15" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B10" s="16" t="n">
         <v>50000</v>
@@ -3145,10 +3188,10 @@
         <v>74</v>
       </c>
       <c r="G10" s="18" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="H10" s="20" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="I10" s="17" t="n">
         <v>46360</v>
@@ -3202,10 +3245,10 @@
         <v>Late</v>
       </c>
       <c r="V10" s="20" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="W10" s="18" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="X10" s="17" t="n">
         <v>46318</v>
@@ -3214,13 +3257,13 @@
         <v>5</v>
       </c>
       <c r="Z10" s="20" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AA10" s="20" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AB10" s="20" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="AC10" s="18"/>
       <c r="AD10" s="21" t="str">
@@ -3253,7 +3296,7 @@
     </row>
     <row r="11" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="15" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B11" s="16" t="n">
         <v>28000</v>
@@ -3274,7 +3317,7 @@
         <v>93</v>
       </c>
       <c r="H11" s="20" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="I11" s="17" t="n">
         <v>46347</v>
@@ -3328,7 +3371,7 @@
         <v>On time</v>
       </c>
       <c r="V11" s="20" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="W11" s="18" t="s">
         <v>78</v>
@@ -3340,10 +3383,10 @@
         <v>9</v>
       </c>
       <c r="Z11" s="20" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="AA11" s="20" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="AB11" s="20"/>
       <c r="AC11" s="18" t="n">
@@ -3358,7 +3401,7 @@
         <v/>
       </c>
       <c r="AF11" s="20" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="AG11" s="22" t="n">
         <f aca="false">IF(I11&lt;=O11,INDEX(Probability!$B$5:$F$19,MATCH(AF11,Probability!$A$5:$A$19,0),MATCH(IF(C11-$E$2&lt;0,"Overdue",IF(C11-$E$2&lt;=30,"0-30",IF(C11-$E$2&lt;=60,"31-60",IF(C11-$E$2&lt;=90,"61-90","&gt;90")))),Probability!$B$4:$F$4,0)),0)</f>
@@ -3379,7 +3422,7 @@
     </row>
     <row r="12" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="15" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B12" s="16" t="n">
         <v>35000</v>
@@ -3397,10 +3440,10 @@
         <v>84</v>
       </c>
       <c r="G12" s="18" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="H12" s="20" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="I12" s="17" t="n">
         <v>46354</v>
@@ -3454,10 +3497,10 @@
         <v>On time</v>
       </c>
       <c r="V12" s="20" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="W12" s="18" t="s">
-        <v>89</v>
+        <v>96</v>
       </c>
       <c r="X12" s="17" t="n">
         <v>46323</v>
@@ -3466,10 +3509,10 @@
         <v>8</v>
       </c>
       <c r="Z12" s="20" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="AA12" s="20" t="s">
-        <v>78</v>
+        <v>130</v>
       </c>
       <c r="AB12" s="20"/>
       <c r="AC12" s="18"/>
@@ -3503,7 +3546,7 @@
     </row>
     <row r="13" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="15" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B13" s="16" t="n">
         <v>46000</v>
@@ -3524,7 +3567,7 @@
         <v>85</v>
       </c>
       <c r="H13" s="20" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="I13" s="17" t="n">
         <v>46365</v>
@@ -3578,7 +3621,7 @@
         <v>On time</v>
       </c>
       <c r="V13" s="20" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="W13" s="18" t="s">
         <v>78</v>
@@ -3590,10 +3633,10 @@
         <v>7</v>
       </c>
       <c r="Z13" s="20" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="AA13" s="20" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="AB13" s="20"/>
       <c r="AC13" s="18"/>
@@ -3627,7 +3670,7 @@
     </row>
     <row r="14" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="15" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="B14" s="16" t="n">
         <v>40000</v>
@@ -3645,10 +3688,10 @@
         <v>74</v>
       </c>
       <c r="G14" s="18" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="H14" s="20" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="I14" s="17" t="n">
         <v>46375</v>
@@ -3702,10 +3745,10 @@
         <v>On time</v>
       </c>
       <c r="V14" s="20" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="W14" s="18" t="s">
-        <v>89</v>
+        <v>96</v>
       </c>
       <c r="X14" s="17" t="n">
         <v>46325</v>
@@ -3714,10 +3757,10 @@
         <v>10</v>
       </c>
       <c r="Z14" s="20" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="AA14" s="20" t="s">
-        <v>78</v>
+        <v>141</v>
       </c>
       <c r="AB14" s="20"/>
       <c r="AC14" s="18" t="n">
@@ -3732,7 +3775,7 @@
         <v>Under-usage: flag CSM; set At risk</v>
       </c>
       <c r="AF14" s="20" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="AG14" s="22" t="n">
         <f aca="false">IF(I14&lt;=O14,INDEX(Probability!$B$5:$F$19,MATCH(AF14,Probability!$A$5:$A$19,0),MATCH(IF(C14-$E$2&lt;0,"Overdue",IF(C14-$E$2&lt;=30,"0-30",IF(C14-$E$2&lt;=60,"31-60",IF(C14-$E$2&lt;=90,"61-90","&gt;90")))),Probability!$B$4:$F$4,0)),0)</f>
@@ -3753,7 +3796,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="B15" s="26" t="n">
         <f aca="false">SUM(B5:B14)</f>
@@ -3778,26 +3821,26 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="27" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="28" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="B19" s="28" t="s">
         <v>62</v>
       </c>
       <c r="C19" s="28" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="D19" s="28" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="15" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="B20" s="23" t="n">
         <f aca="false">SUMIFS(T5:T14,U5:U14,"On time")</f>
@@ -3814,7 +3857,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="15" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="B21" s="23" t="n">
         <f aca="false">SUMIFS(T5:T14,U5:U14,"Late")</f>
@@ -3831,7 +3874,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="15" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="B22" s="23" t="n">
         <f aca="false">SUMIFS(T5:T14,U5:U14,"Slips quarter")</f>
@@ -3848,7 +3891,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="7" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="B23" s="29" t="n">
         <f aca="false">SUM(B20:B22)</f>
@@ -3862,12 +3905,12 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="2" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="15" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="B25" s="31" t="n">
         <f aca="false">'Opp summary'!E15</f>
@@ -3876,7 +3919,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="15" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="B26" s="31" t="n">
         <f aca="false">'Opp summary'!F15</f>
@@ -3885,7 +3928,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="15" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="B27" s="31" t="n">
         <f aca="false">'Opp summary'!H15</f>
@@ -3894,7 +3937,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="15" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="B28" s="32" t="n">
         <f aca="false">(B15+B25+B27)/B15</f>
@@ -3903,7 +3946,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="15" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="B29" s="32" t="n">
         <f aca="false">S15/B15</f>
@@ -3917,7 +3960,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="15" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="B32" s="29" t="n">
         <f aca="false">T15</f>
@@ -3926,7 +3969,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="15" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="B33" s="33" t="n">
         <f aca="false">AH15</f>
@@ -3935,7 +3978,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="15" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="B34" s="33" t="n">
         <f aca="false">B33-B32</f>
@@ -3944,7 +3987,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="15" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="B35" s="34" t="n">
         <f aca="false">AJ15</f>
@@ -3953,7 +3996,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="15" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="B36" s="34" t="n">
         <f aca="false">B35-B32</f>
@@ -3962,7 +4005,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="15" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="B37" s="33" t="n">
         <f aca="false">B33-B35</f>
@@ -4098,12 +4141,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="35" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="B2" s="35"/>
       <c r="C2" s="35"/>
@@ -4121,52 +4164,52 @@
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="I4" s="6" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="J4" s="6" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="K4" s="6" t="s">
         <v>61</v>
       </c>
       <c r="L4" s="6" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="M4" s="6" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="N4" s="6" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="O4" s="6" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="P4" s="6" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4174,16 +4217,16 @@
         <v>72</v>
       </c>
       <c r="B5" s="15" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="C5" s="18" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="D5" s="18" t="n">
         <v>1</v>
       </c>
       <c r="E5" s="18" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="F5" s="23" t="n">
         <v>21000</v>
@@ -4222,7 +4265,7 @@
         <v>n/a</v>
       </c>
       <c r="P5" s="15" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4230,16 +4273,16 @@
         <v>83</v>
       </c>
       <c r="B6" s="15" t="s">
+        <v>184</v>
+      </c>
+      <c r="C6" s="18" t="s">
         <v>181</v>
-      </c>
-      <c r="C6" s="18" t="s">
-        <v>178</v>
       </c>
       <c r="D6" s="18" t="n">
         <v>1</v>
       </c>
       <c r="E6" s="18" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="F6" s="23" t="n">
         <v>48000</v>
@@ -4278,7 +4321,7 @@
         <v>n/a</v>
       </c>
       <c r="P6" s="15" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4286,16 +4329,16 @@
         <v>91</v>
       </c>
       <c r="B7" s="15" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="C7" s="18" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="D7" s="18" t="n">
         <v>1</v>
       </c>
       <c r="E7" s="18" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="F7" s="23" t="n">
         <v>26000</v>
@@ -4334,24 +4377,24 @@
         <v>n/a</v>
       </c>
       <c r="P7" s="15" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="15" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B8" s="15" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="C8" s="18" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="D8" s="18" t="n">
         <v>1</v>
       </c>
       <c r="E8" s="18" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="F8" s="23" t="n">
         <v>45000</v>
@@ -4390,24 +4433,24 @@
         <v>n/a</v>
       </c>
       <c r="P8" s="15" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="15" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B9" s="15" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="C9" s="18" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="D9" s="18" t="n">
         <v>2</v>
       </c>
       <c r="E9" s="18" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="F9" s="23" t="n">
         <v>36000</v>
@@ -4446,24 +4489,24 @@
         <v>5% a year</v>
       </c>
       <c r="P9" s="15" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="15" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B10" s="15" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="C10" s="18" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="D10" s="18" t="n">
         <v>1</v>
       </c>
       <c r="E10" s="18" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="F10" s="23" t="n">
         <v>50000</v>
@@ -4505,19 +4548,19 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="15" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B11" s="15" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="C11" s="18" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="D11" s="18" t="n">
         <v>1</v>
       </c>
       <c r="E11" s="18" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="F11" s="23" t="n">
         <v>28000</v>
@@ -4556,24 +4599,24 @@
         <v>n/a</v>
       </c>
       <c r="P11" s="15" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="15" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B12" s="15" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="C12" s="18" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="D12" s="18" t="n">
         <v>1</v>
       </c>
       <c r="E12" s="18" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="F12" s="23" t="n">
         <v>35000</v>
@@ -4612,24 +4655,24 @@
         <v>n/a</v>
       </c>
       <c r="P12" s="15" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="15" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B13" s="15" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="C13" s="18" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="D13" s="18" t="n">
         <v>1</v>
       </c>
       <c r="E13" s="18" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="F13" s="23" t="n">
         <v>0</v>
@@ -4668,24 +4711,24 @@
         <v>n/a</v>
       </c>
       <c r="P13" s="15" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="15" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B14" s="15" t="s">
+        <v>184</v>
+      </c>
+      <c r="C14" s="18" t="s">
         <v>181</v>
-      </c>
-      <c r="C14" s="18" t="s">
-        <v>178</v>
       </c>
       <c r="D14" s="18" t="n">
         <v>1</v>
       </c>
       <c r="E14" s="18" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="F14" s="23" t="n">
         <v>46000</v>
@@ -4727,19 +4770,19 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="15" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="B15" s="15" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="C15" s="18" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="D15" s="18" t="n">
         <v>1</v>
       </c>
       <c r="E15" s="18" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="F15" s="23" t="n">
         <v>40000</v>
@@ -4778,12 +4821,12 @@
         <v>n/a</v>
       </c>
       <c r="P15" s="15" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="F17" s="26" t="n">
         <f aca="false">SUM(F5:F15)</f>
@@ -4808,12 +4851,12 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="35" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="B20" s="35"/>
       <c r="C20" s="35"/>
@@ -4891,42 +4934,42 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="G3" s="6" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="H3" s="6" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="I3" s="6" t="s">
         <v>61</v>
       </c>
       <c r="J3" s="6" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="K3" s="6" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5071,10 +5114,10 @@
         <v>-15000</v>
       </c>
       <c r="F7" s="18" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="G7" s="18" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="H7" s="23" t="n">
         <f aca="false">MIN(0,C7-(SUMIFS(Products!$J:$J,Products!$A:$A,$A7)-SUMIFS(Products!$K:$K,Products!$A:$A,$A7)))</f>
@@ -5315,10 +5358,10 @@
         <v>-8000</v>
       </c>
       <c r="F13" s="18" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="G13" s="18" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="H13" s="23" t="n">
         <f aca="false">MIN(0,C13-(SUMIFS(Products!$J:$J,Products!$A:$A,$A13)-SUMIFS(Products!$K:$K,Products!$A:$A,$A13)))</f>
@@ -5339,7 +5382,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="B14" s="26" t="n">
         <f aca="false">SUM(B4:B13)</f>
@@ -5376,7 +5419,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="38" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="E15" s="39" t="n">
         <f aca="false">SUMIFS(E4:E13,F4:F13,"Regrettable")</f>
@@ -5393,10 +5436,10 @@
     </row>
     <row r="16" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="B16" s="35" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="C16" s="35"/>
       <c r="D16" s="35"/>
@@ -5410,7 +5453,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="B17" s="12" t="str">
         <f aca="false">COUNTIFS(E4:E13,"&lt;0",F4:F13,"")&amp;" opportunities with churn but no category"</f>
@@ -5419,7 +5462,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="12" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="B18" s="12" t="str">
         <f aca="false">IF(ABS(I14-Pipeline!S15)&lt;1,"OK","MISMATCH")</f>
@@ -5483,7 +5526,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5494,7 +5537,7 @@
         <v>56</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="D3" s="6" t="s">
         <v>47</v>
@@ -5503,27 +5546,27 @@
         <v>61</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="G3" s="6" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="H3" s="6" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
       <c r="I3" s="6" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="J3" s="6" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="15" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="B4" s="15" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="C4" s="15" t="n">
         <f aca="false">COUNTIFS(Pipeline!$M$5:$M$14,B4)</f>
@@ -5560,10 +5603,10 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="15" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="B5" s="15" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="C5" s="15" t="n">
         <f aca="false">COUNTIFS(Pipeline!$M$5:$M$14,B5)</f>
@@ -5600,10 +5643,10 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="15" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="B6" s="15" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="C6" s="15" t="n">
         <f aca="false">COUNTIFS(Pipeline!$M$5:$M$14,B6)</f>
@@ -5640,7 +5683,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="C7" s="2" t="n">
         <f aca="false">SUM(C4:C6)</f>
@@ -5712,12 +5755,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5725,30 +5768,30 @@
         <v>34</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
       <c r="B5" s="40" t="n">
         <v>0</v>
@@ -5766,7 +5809,7 @@
         <v>0</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="H5" s="15" t="s">
         <v>73</v>
@@ -5774,7 +5817,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B6" s="40" t="n">
         <v>0.05</v>
@@ -5792,7 +5835,7 @@
         <v>0.35</v>
       </c>
       <c r="G6" s="8" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="H6" s="15" t="s">
         <v>73</v>
@@ -5818,7 +5861,7 @@
         <v>0.5</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="H7" s="15" t="s">
         <v>73</v>
@@ -5826,7 +5869,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B8" s="40" t="n">
         <v>0.2</v>
@@ -5844,7 +5887,7 @@
         <v>0.55</v>
       </c>
       <c r="G8" s="8" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
       <c r="H8" s="15" t="s">
         <v>73</v>
@@ -5870,7 +5913,7 @@
         <v>0.6</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="H9" s="15" t="s">
         <v>73</v>
@@ -5896,7 +5939,7 @@
         <v>0.75</v>
       </c>
       <c r="G10" s="8" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="H10" s="15" t="s">
         <v>73</v>
@@ -5922,7 +5965,7 @@
         <v>0.9</v>
       </c>
       <c r="G11" s="8" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="H11" s="15" t="s">
         <v>73</v>
@@ -5930,7 +5973,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
       <c r="B12" s="40" t="n">
         <v>1</v>
@@ -5948,7 +5991,7 @@
         <v>1</v>
       </c>
       <c r="G12" s="8" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
       <c r="H12" s="15" t="s">
         <v>73</v>
@@ -5956,7 +5999,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="B13" s="40" t="n">
         <v>0</v>
@@ -5974,15 +6017,15 @@
         <v>0</v>
       </c>
       <c r="G13" s="8" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="H13" s="15" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B14" s="40" t="n">
         <v>0.4</v>
@@ -6000,7 +6043,7 @@
         <v>0.9</v>
       </c>
       <c r="G14" s="8" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="H14" s="15" t="s">
         <v>92</v>
@@ -6026,7 +6069,7 @@
         <v>0.8</v>
       </c>
       <c r="G15" s="8" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="H15" s="15" t="s">
         <v>92</v>
@@ -6034,7 +6077,7 @@
     </row>
     <row r="16" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B16" s="40" t="n">
         <v>0.2</v>
@@ -6052,7 +6095,7 @@
         <v>0.5</v>
       </c>
       <c r="G16" s="8" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="H16" s="15" t="s">
         <v>92</v>
@@ -6060,7 +6103,7 @@
     </row>
     <row r="17" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
       <c r="B17" s="40" t="n">
         <v>0.5</v>
@@ -6078,7 +6121,7 @@
         <v>0.8</v>
       </c>
       <c r="G17" s="8" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="H17" s="15" t="s">
         <v>92</v>
@@ -6086,7 +6129,7 @@
     </row>
     <row r="18" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="7" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
       <c r="B18" s="40" t="n">
         <v>0</v>
@@ -6104,7 +6147,7 @@
         <v>0.1</v>
       </c>
       <c r="G18" s="8" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
       <c r="H18" s="15" t="s">
         <v>92</v>
@@ -6112,7 +6155,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="B19" s="40" t="n">
         <v>1</v>
@@ -6130,7 +6173,7 @@
         <v>1</v>
       </c>
       <c r="G19" s="8" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
       <c r="H19" s="15" t="s">
         <v>92</v>
@@ -6141,7 +6184,7 @@
         <v>15</v>
       </c>
       <c r="B21" s="35" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="C21" s="35"/>
       <c r="D21" s="35"/>
@@ -6170,7 +6213,7 @@
         <v>11</v>
       </c>
       <c r="B25" s="35" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
       <c r="C25" s="35"/>
       <c r="D25" s="35"/>
@@ -6236,95 +6279,95 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>263</v>
+        <v>266</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>264</v>
+        <v>267</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>265</v>
+        <v>268</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>266</v>
+        <v>269</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>269</v>
+        <v>272</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>272</v>
+        <v>275</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>273</v>
+        <v>276</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>275</v>
+        <v>278</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="8" t="s">
-        <v>277</v>
+        <v>280</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="8" t="s">
-        <v>280</v>
+        <v>283</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>281</v>
+        <v>284</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
     </row>
   </sheetData>

</xml_diff>